<commit_message>
updated spreadsheet. solved 2 more sliding window problems.
</commit_message>
<xml_diff>
--- a/leetcode_roadmap.xlsx
+++ b/leetcode_roadmap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="917" uniqueCount="225">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="227">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -79,7 +79,13 @@
     <t xml:space="preserve">https://leetcode.com/problems/minimum-size-subarray-sum/</t>
   </si>
   <si>
+    <t xml:space="preserve">Read the question in its entirety before coming up with a solution ;)</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/longest-repeating-character-replacement/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Don’t think too much about what character to substitute with, but rather create a window that satisfies all k substitutions</t>
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/permutation-in-string/</t>
@@ -1362,7 +1368,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="69.98"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="95.83"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1462,8 +1468,8 @@
       <c r="D4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E4" s="8" t="s">
-        <v>11</v>
+      <c r="E4" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F4" s="8" t="s">
         <v>11</v>
@@ -1471,7 +1477,9 @@
       <c r="G4" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H4" s="10"/>
+      <c r="H4" s="10" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="s">
@@ -1488,16 +1496,18 @@
       <c r="D5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E5" s="15" t="s">
-        <v>11</v>
+      <c r="E5" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F5" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G5" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="17"/>
+        <v>19</v>
+      </c>
+      <c r="H5" s="17" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
@@ -1521,7 +1531,7 @@
         <v>11</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H6" s="10"/>
     </row>
@@ -1547,13 +1557,13 @@
         <v>11</v>
       </c>
       <c r="G7" s="16" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="H7" s="17"/>
     </row>
     <row r="8" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B8" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/container-with-most-water/", "11")</f>
@@ -1573,13 +1583,13 @@
         <v>11</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="H8" s="10"/>
     </row>
     <row r="9" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B9" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/3sum/", "15")</f>
@@ -1599,13 +1609,13 @@
         <v>11</v>
       </c>
       <c r="G9" s="16" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="H9" s="17"/>
     </row>
     <row r="10" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B10" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/3sum-closest/", "16")</f>
@@ -1625,13 +1635,13 @@
         <v>11</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H10" s="10"/>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B11" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/4sum/", "18")</f>
@@ -1651,13 +1661,13 @@
         <v>11</v>
       </c>
       <c r="G11" s="16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H11" s="17"/>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B12" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/trapping-rain-water/", "42")</f>
@@ -1677,13 +1687,13 @@
         <v>11</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="H12" s="10"/>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B13" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/two-sum-ii-input-array-is-sorted/", "167")</f>
@@ -1703,13 +1713,13 @@
         <v>11</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="H13" s="17"/>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B14" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/linked-list-cycle/", "141")</f>
@@ -1720,7 +1730,7 @@
         <v>Linked List Cycle</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>11</v>
@@ -1729,13 +1739,13 @@
         <v>11</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="H14" s="10"/>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B15" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/linked-list-cycle-ii/", "142")</f>
@@ -1755,13 +1765,13 @@
         <v>11</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="H15" s="17"/>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B16" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/remove-nth-node-from-end-of-list/", "19")</f>
@@ -1781,13 +1791,13 @@
         <v>11</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="H16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B17" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/middle-of-the-linked-list/", "876")</f>
@@ -1798,7 +1808,7 @@
         <v>Middle of the Linked List</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E17" s="15" t="s">
         <v>11</v>
@@ -1807,13 +1817,13 @@
         <v>11</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="H17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B18" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/intersection-of-two-linked-lists/", "160")</f>
@@ -1824,7 +1834,7 @@
         <v>Intersection of Two Linked Lists</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>11</v>
@@ -1833,13 +1843,13 @@
         <v>11</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="B19" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/palindrome-linked-list/", "234")</f>
@@ -1850,7 +1860,7 @@
         <v>Palindrome Linked List</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E19" s="15" t="s">
         <v>11</v>
@@ -1859,13 +1869,13 @@
         <v>11</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H19" s="17"/>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B20" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-rotated-sorted-array/", "33")</f>
@@ -1885,13 +1895,13 @@
         <v>11</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="H20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B21" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/", "34")</f>
@@ -1911,13 +1921,13 @@
         <v>11</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="H21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B22" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-insert-position/", "35")</f>
@@ -1928,7 +1938,7 @@
         <v>Search Insert Position</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>11</v>
@@ -1937,13 +1947,13 @@
         <v>11</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B23" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/", "153")</f>
@@ -1963,13 +1973,13 @@
         <v>11</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="H23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B24" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-peak-element/", "162")</f>
@@ -1989,13 +1999,13 @@
         <v>11</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="H24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B25" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-search/", "704")</f>
@@ -2006,7 +2016,7 @@
         <v>Binary Search</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E25" s="15" t="s">
         <v>11</v>
@@ -2015,13 +2025,13 @@
         <v>11</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B26" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/koko-eating-bananas/", "875")</f>
@@ -2041,13 +2051,13 @@
         <v>11</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B27" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/capacity-to-ship-packages-within-d-days/", "1011")</f>
@@ -2067,13 +2077,13 @@
         <v>11</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="H27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B28" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/split-array-largest-sum/", "410")</f>
@@ -2093,13 +2103,13 @@
         <v>11</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="H28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B29" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimize-max-distance-to-gas-station/", "774")</f>
@@ -2119,15 +2129,15 @@
         <v>11</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B30" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-smallest-divisor-given-a-threshold/", "1283")</f>
@@ -2147,13 +2157,13 @@
         <v>11</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="B31" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-days-to-make-m-bouquets/", "1482")</f>
@@ -2173,13 +2183,13 @@
         <v>11</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H31" s="17"/>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B32" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/two-sum/", "1")</f>
@@ -2190,7 +2200,7 @@
         <v>Two Sum</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>11</v>
@@ -2199,13 +2209,13 @@
         <v>11</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="H32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B33" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/group-anagrams/", "49")</f>
@@ -2225,13 +2235,13 @@
         <v>11</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B34" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-consecutive-sequence/", "128")</f>
@@ -2251,13 +2261,13 @@
         <v>11</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="H34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B35" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/contains-duplicate/", "217")</f>
@@ -2268,7 +2278,7 @@
         <v>Contains Duplicate</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E35" s="15" t="s">
         <v>11</v>
@@ -2277,13 +2287,13 @@
         <v>11</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B36" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/valid-anagram/", "242")</f>
@@ -2294,7 +2304,7 @@
         <v>Valid Anagram</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E36" s="8" t="s">
         <v>11</v>
@@ -2303,13 +2313,13 @@
         <v>11</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="H36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B37" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -2329,13 +2339,13 @@
         <v>11</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B38" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-sum-query-immutable/", "303")</f>
@@ -2346,7 +2356,7 @@
         <v>Range Sum Query - Immutable</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E38" s="8" t="s">
         <v>11</v>
@@ -2355,13 +2365,13 @@
         <v>11</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="H38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B39" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sum-equals-k/", "560")</f>
@@ -2381,13 +2391,13 @@
         <v>11</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="H39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B40" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-pivot-index/", "724")</f>
@@ -2398,7 +2408,7 @@
         <v>Find Pivot Index</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E40" s="8" t="s">
         <v>11</v>
@@ -2407,13 +2417,13 @@
         <v>11</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="H40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B41" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-subarrays-with-sum/", "930")</f>
@@ -2433,13 +2443,13 @@
         <v>11</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="H41" s="17"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B42" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sums-divisible-by-k/", "974")</f>
@@ -2459,13 +2469,13 @@
         <v>11</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="H42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="B43" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/continuous-subarray-sum/", "523")</f>
@@ -2485,13 +2495,13 @@
         <v>11</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="H43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B44" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-addition/", "370")</f>
@@ -2511,15 +2521,15 @@
         <v>11</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H44" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B45" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/car-pooling/", "1094")</f>
@@ -2539,13 +2549,13 @@
         <v>11</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="H45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B46" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/corporate-flight-bookings/", "1109")</f>
@@ -2565,13 +2575,13 @@
         <v>11</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B47" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/check-if-all-the-integers-in-a-range-are-covered/", "1893")</f>
@@ -2582,7 +2592,7 @@
         <v>Check if All the Integers in a Range Are Covered</v>
       </c>
       <c r="D47" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E47" s="15" t="s">
         <v>11</v>
@@ -2591,13 +2601,13 @@
         <v>11</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B48" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/describe-the-painting/", "1943")</f>
@@ -2617,13 +2627,13 @@
         <v>11</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B49" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shifting-letters-ii/", "2381")</f>
@@ -2643,13 +2653,13 @@
         <v>11</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H49" s="17"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B50" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/daily-temperatures/", "739")</f>
@@ -2669,13 +2679,13 @@
         <v>11</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="H50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B51" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-i/", "496")</f>
@@ -2686,7 +2696,7 @@
         <v>Next Greater Element I</v>
       </c>
       <c r="D51" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E51" s="15" t="s">
         <v>11</v>
@@ -2695,13 +2705,13 @@
         <v>11</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="H51" s="17"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B52" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-ii/", "503")</f>
@@ -2721,13 +2731,13 @@
         <v>11</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B53" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/largest-rectangle-in-histogram/", "84")</f>
@@ -2747,13 +2757,13 @@
         <v>11</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="H53" s="17"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B54" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-rectangle/", "85")</f>
@@ -2773,13 +2783,13 @@
         <v>11</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="H54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="B55" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/online-stock-span/", "901")</f>
@@ -2799,13 +2809,13 @@
         <v>11</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="H55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B56" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sliding-window-maximum/", "239")</f>
@@ -2825,13 +2835,13 @@
         <v>11</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="H56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B57" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-subarray-with-sum-at-least-k/", "862")</f>
@@ -2851,13 +2861,13 @@
         <v>11</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="H57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B58" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/constrained-subsequence-sum/", "1425")</f>
@@ -2877,13 +2887,13 @@
         <v>11</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B59" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-continuous-subarray-with-absolute-diff-less-than-or-equal-to-limit/", "1438")</f>
@@ -2903,13 +2913,13 @@
         <v>11</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="H59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B60" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-value-of-equation/", "1499")</f>
@@ -2929,13 +2939,13 @@
         <v>11</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="H60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B61" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-vi/", "1696")</f>
@@ -2955,13 +2965,13 @@
         <v>11</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="H61" s="17"/>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B62" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-an-array/", "215")</f>
@@ -2981,13 +2991,13 @@
         <v>11</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B63" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -3007,13 +3017,13 @@
         <v>11</v>
       </c>
       <c r="G63" s="16" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="H63" s="17"/>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B64" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-words/", "692")</f>
@@ -3033,13 +3043,13 @@
         <v>11</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="H64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B65" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-a-stream/", "703")</f>
@@ -3050,7 +3060,7 @@
         <v>Kth Largest Element in a Stream</v>
       </c>
       <c r="D65" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E65" s="15" t="s">
         <v>11</v>
@@ -3059,13 +3069,13 @@
         <v>11</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="H65" s="17"/>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B66" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/k-closest-points-to-origin/", "973")</f>
@@ -3085,13 +3095,13 @@
         <v>11</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="H66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="B67" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight/", "1046")</f>
@@ -3102,7 +3112,7 @@
         <v>Last Stone Weight</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E67" s="15" t="s">
         <v>11</v>
@@ -3111,13 +3121,13 @@
         <v>11</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H67" s="17"/>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B68" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-intervals/", "56")</f>
@@ -3137,13 +3147,13 @@
         <v>11</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="H68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B69" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/insert-interval/", "57")</f>
@@ -3163,13 +3173,13 @@
         <v>11</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="H69" s="17"/>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B70" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms/", "252")</f>
@@ -3180,7 +3190,7 @@
         <v>Meeting Rooms</v>
       </c>
       <c r="D70" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E70" s="8" t="s">
         <v>11</v>
@@ -3189,15 +3199,15 @@
         <v>11</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="H70" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B71" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms-ii/", "253")</f>
@@ -3217,15 +3227,15 @@
         <v>11</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="H71" s="19" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B72" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/non-overlapping-intervals/", "435")</f>
@@ -3245,13 +3255,13 @@
         <v>11</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="H72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B73" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-arrows-to-burst-balloons/", "452")</f>
@@ -3271,13 +3281,13 @@
         <v>11</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H73" s="17"/>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B74" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-ii/", "45")</f>
@@ -3297,13 +3307,13 @@
         <v>11</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="H74" s="10"/>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B75" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game/", "55")</f>
@@ -3323,13 +3333,13 @@
         <v>11</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="H75" s="17"/>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B76" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/queue-reconstruction-by-height/", "406")</f>
@@ -3349,13 +3359,13 @@
         <v>11</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="H76" s="10"/>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B77" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/task-scheduler/", "621")</f>
@@ -3375,13 +3385,13 @@
         <v>11</v>
       </c>
       <c r="G77" s="16" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="H77" s="17"/>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B78" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-labels/", "763")</f>
@@ -3401,13 +3411,13 @@
         <v>11</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="H78" s="10"/>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B79" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/gas-station/", "134")</f>
@@ -3427,13 +3437,13 @@
         <v>11</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="H79" s="17"/>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B80" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/", "21")</f>
@@ -3444,7 +3454,7 @@
         <v>Merge Two Sorted Lists</v>
       </c>
       <c r="D80" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E80" s="8" t="s">
         <v>11</v>
@@ -3453,13 +3463,13 @@
         <v>11</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H80" s="10"/>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B81" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-k-sorted-lists/", "23")</f>
@@ -3479,13 +3489,13 @@
         <v>11</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="H81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B82" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swap-nodes-in-pairs/", "24")</f>
@@ -3505,13 +3515,13 @@
         <v>11</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="H82" s="10"/>
     </row>
     <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B83" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-nodes-in-k-group/", "25")</f>
@@ -3531,13 +3541,13 @@
         <v>11</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H83" s="17"/>
     </row>
     <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B84" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-linked-list-ii/", "92")</f>
@@ -3557,13 +3567,13 @@
         <v>11</v>
       </c>
       <c r="G84" s="9" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="H84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B85" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/copy-list-with-random-pointer/", "138")</f>
@@ -3583,13 +3593,13 @@
         <v>11</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="H85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B86" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximum-depth-of-binary-tree/", "104")</f>
@@ -3600,7 +3610,7 @@
         <v>Maximum Depth of Binary Tree</v>
       </c>
       <c r="D86" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E86" s="8" t="s">
         <v>11</v>
@@ -3609,13 +3619,13 @@
         <v>11</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="H86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B87" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum/", "112")</f>
@@ -3626,7 +3636,7 @@
         <v>Path Sum</v>
       </c>
       <c r="D87" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E87" s="15" t="s">
         <v>11</v>
@@ -3635,13 +3645,13 @@
         <v>11</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="H87" s="17"/>
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B88" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum-ii/", "113")</f>
@@ -3661,13 +3671,13 @@
         <v>11</v>
       </c>
       <c r="G88" s="9" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="H88" s="10"/>
     </row>
     <row r="89" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B89" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/diameter-of-binary-tree/", "543")</f>
@@ -3678,7 +3688,7 @@
         <v>Diameter of Binary Tree</v>
       </c>
       <c r="D89" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E89" s="15" t="s">
         <v>11</v>
@@ -3687,13 +3697,13 @@
         <v>11</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="H89" s="17"/>
     </row>
     <row r="90" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B90" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-maximum-path-sum/", "124")</f>
@@ -3713,13 +3723,13 @@
         <v>11</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="H90" s="10"/>
     </row>
     <row r="91" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B91" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/invert-binary-tree/", "226")</f>
@@ -3730,7 +3740,7 @@
         <v>Invert Binary Tree</v>
       </c>
       <c r="D91" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E91" s="15" t="s">
         <v>11</v>
@@ -3739,13 +3749,13 @@
         <v>11</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="H91" s="17"/>
     </row>
     <row r="92" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B92" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-level-order-traversal/", "102")</f>
@@ -3765,13 +3775,13 @@
         <v>11</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H92" s="10"/>
     </row>
     <row r="93" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B93" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/", "103")</f>
@@ -3791,13 +3801,13 @@
         <v>11</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="H93" s="17"/>
     </row>
     <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B94" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-right-side-view/", "199")</f>
@@ -3817,13 +3827,13 @@
         <v>11</v>
       </c>
       <c r="G94" s="9" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="H94" s="10"/>
     </row>
     <row r="95" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B95" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-largest-value-in-each-tree-row/", "515")</f>
@@ -3843,13 +3853,13 @@
         <v>11</v>
       </c>
       <c r="G95" s="16" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="H95" s="17"/>
     </row>
     <row r="96" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B96" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/average-of-levels-in-binary-tree/", "637")</f>
@@ -3860,7 +3870,7 @@
         <v>Average of Levels in Binary Tree</v>
       </c>
       <c r="D96" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E96" s="8" t="s">
         <v>11</v>
@@ -3869,13 +3879,13 @@
         <v>11</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H96" s="10"/>
     </row>
     <row r="97" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B97" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/populating-next-right-pointers-in-each-node/", "116")</f>
@@ -3895,13 +3905,13 @@
         <v>11</v>
       </c>
       <c r="G97" s="16" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="H97" s="17"/>
     </row>
     <row r="98" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B98" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/validate-binary-search-tree/", "98")</f>
@@ -3921,13 +3931,13 @@
         <v>11</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="H98" s="10"/>
     </row>
     <row r="99" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B99" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/recover-binary-search-tree/", "99")</f>
@@ -3947,13 +3957,13 @@
         <v>11</v>
       </c>
       <c r="G99" s="16" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H99" s="17"/>
     </row>
     <row r="100" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B100" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-smallest-element-in-a-bst/", "230")</f>
@@ -3973,13 +3983,13 @@
         <v>11</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="H100" s="10"/>
     </row>
     <row r="101" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B101" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/", "235")</f>
@@ -3999,13 +4009,13 @@
         <v>11</v>
       </c>
       <c r="G101" s="16" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H101" s="17"/>
     </row>
     <row r="102" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B102" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-node-in-a-bst/", "450")</f>
@@ -4025,13 +4035,13 @@
         <v>11</v>
       </c>
       <c r="G102" s="9" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="H102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B103" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-a-binary-search-tree/", "700")</f>
@@ -4042,7 +4052,7 @@
         <v>Search in a Binary Search Tree</v>
       </c>
       <c r="D103" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E103" s="15" t="s">
         <v>11</v>
@@ -4051,13 +4061,13 @@
         <v>11</v>
       </c>
       <c r="G103" s="16" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H103" s="17"/>
     </row>
     <row r="104" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B104" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations/", "46")</f>
@@ -4077,13 +4087,13 @@
         <v>11</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="H104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B105" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations-ii/", "47")</f>
@@ -4103,13 +4113,13 @@
         <v>11</v>
       </c>
       <c r="G105" s="16" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H105" s="17"/>
     </row>
     <row r="106" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B106" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combinations/", "77")</f>
@@ -4129,13 +4139,13 @@
         <v>11</v>
       </c>
       <c r="G106" s="9" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="H106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B107" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets/", "78")</f>
@@ -4155,13 +4165,13 @@
         <v>11</v>
       </c>
       <c r="G107" s="16" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="H107" s="17"/>
     </row>
     <row r="108" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B108" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets-ii/", "90")</f>
@@ -4181,13 +4191,13 @@
         <v>11</v>
       </c>
       <c r="G108" s="9" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="H108" s="10"/>
     </row>
     <row r="109" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="B109" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum/", "39")</f>
@@ -4207,13 +4217,13 @@
         <v>11</v>
       </c>
       <c r="G109" s="16" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="H109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B110" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum-ii/", "40")</f>
@@ -4233,13 +4243,13 @@
         <v>11</v>
       </c>
       <c r="G110" s="9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="H110" s="10"/>
     </row>
     <row r="111" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B111" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/letter-combinations-of-a-phone-number/", "17")</f>
@@ -4259,13 +4269,13 @@
         <v>11</v>
       </c>
       <c r="G111" s="16" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="H111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B112" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search/", "79")</f>
@@ -4285,13 +4295,13 @@
         <v>11</v>
       </c>
       <c r="G112" s="9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="H112" s="10"/>
     </row>
     <row r="113" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B113" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/palindrome-partitioning/", "131")</f>
@@ -4311,13 +4321,13 @@
         <v>11</v>
       </c>
       <c r="G113" s="16" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="H113" s="17"/>
     </row>
     <row r="114" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B114" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens/", "51")</f>
@@ -4337,13 +4347,13 @@
         <v>11</v>
       </c>
       <c r="G114" s="9" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="H114" s="10"/>
     </row>
     <row r="115" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="B115" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens-ii/", "52")</f>
@@ -4363,13 +4373,13 @@
         <v>11</v>
       </c>
       <c r="G115" s="16" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="H115" s="17"/>
     </row>
     <row r="116" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B116" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-islands/", "200")</f>
@@ -4389,13 +4399,13 @@
         <v>11</v>
       </c>
       <c r="G116" s="9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="H116" s="10"/>
     </row>
     <row r="117" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B117" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-area-of-island/", "695")</f>
@@ -4415,13 +4425,13 @@
         <v>11</v>
       </c>
       <c r="G117" s="16" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="H117" s="17"/>
     </row>
     <row r="118" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B118" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/flood-fill/", "733")</f>
@@ -4432,7 +4442,7 @@
         <v>Flood Fill</v>
       </c>
       <c r="D118" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E118" s="8" t="s">
         <v>11</v>
@@ -4441,13 +4451,13 @@
         <v>11</v>
       </c>
       <c r="G118" s="9" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="H118" s="10"/>
     </row>
     <row r="119" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B119" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/rotting-oranges/", "994")</f>
@@ -4467,13 +4477,13 @@
         <v>11</v>
       </c>
       <c r="G119" s="16" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="H119" s="17"/>
     </row>
     <row r="120" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B120" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-path-in-binary-matrix/", "1091")</f>
@@ -4493,13 +4503,13 @@
         <v>11</v>
       </c>
       <c r="G120" s="9" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="H120" s="10"/>
     </row>
     <row r="121" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="B121" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-closed-islands/", "1254")</f>
@@ -4519,13 +4529,13 @@
         <v>11</v>
       </c>
       <c r="G121" s="16" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="H121" s="17"/>
     </row>
     <row r="122" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B122" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule/", "207")</f>
@@ -4545,13 +4555,13 @@
         <v>11</v>
       </c>
       <c r="G122" s="9" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="H122" s="10"/>
     </row>
     <row r="123" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B123" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-ii/", "210")</f>
@@ -4571,13 +4581,13 @@
         <v>11</v>
       </c>
       <c r="G123" s="16" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="H123" s="17"/>
     </row>
     <row r="124" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B124" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-eventual-safe-states/", "802")</f>
@@ -4597,13 +4607,13 @@
         <v>11</v>
       </c>
       <c r="G124" s="9" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="H124" s="10"/>
     </row>
     <row r="125" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B125" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-iv/", "1462")</f>
@@ -4623,13 +4633,13 @@
         <v>11</v>
       </c>
       <c r="G125" s="16" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="H125" s="17"/>
     </row>
     <row r="126" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B126" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sort-items-by-groups-respecting-dependencies/", "1203")</f>
@@ -4649,13 +4659,13 @@
         <v>11</v>
       </c>
       <c r="G126" s="9" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="H126" s="10"/>
     </row>
     <row r="127" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="11" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="B127" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-all-possible-recipes-from-given-supplies/", "2115")</f>
@@ -4675,13 +4685,13 @@
         <v>11</v>
       </c>
       <c r="G127" s="16" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="H127" s="17"/>
     </row>
     <row r="128" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B128" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-provinces/", "547")</f>
@@ -4701,13 +4711,13 @@
         <v>11</v>
       </c>
       <c r="G128" s="9" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="H128" s="10"/>
     </row>
     <row r="129" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B129" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/redundant-connection/", "684")</f>
@@ -4727,13 +4737,13 @@
         <v>11</v>
       </c>
       <c r="G129" s="16" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="H129" s="17"/>
     </row>
     <row r="130" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B130" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-operations-to-make-network-connected/", "1319")</f>
@@ -4753,13 +4763,13 @@
         <v>11</v>
       </c>
       <c r="G130" s="9" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="H130" s="10"/>
     </row>
     <row r="131" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B131" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/remove-max-number-of-edges-to-keep-graph-fully-traversable/", "1579")</f>
@@ -4779,13 +4789,13 @@
         <v>11</v>
       </c>
       <c r="G131" s="16" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="H131" s="17"/>
     </row>
     <row r="132" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B132" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/satisfiability-of-equality-equations/", "990")</f>
@@ -4805,13 +4815,13 @@
         <v>11</v>
       </c>
       <c r="G132" s="9" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="H132" s="10"/>
     </row>
     <row r="133" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="11" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="B133" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/smallest-string-with-swaps/", "1202")</f>
@@ -4831,13 +4841,13 @@
         <v>11</v>
       </c>
       <c r="G133" s="16" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="H133" s="17"/>
     </row>
     <row r="134" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B134" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/network-delay-time/", "743")</f>
@@ -4857,13 +4867,13 @@
         <v>11</v>
       </c>
       <c r="G134" s="9" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="H134" s="10"/>
     </row>
     <row r="135" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B135" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/cheapest-flights-within-k-stops/", "787")</f>
@@ -4883,13 +4893,13 @@
         <v>11</v>
       </c>
       <c r="G135" s="16" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="H135" s="17"/>
     </row>
     <row r="136" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B136" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-probability/", "1514")</f>
@@ -4909,13 +4919,13 @@
         <v>11</v>
       </c>
       <c r="G136" s="9" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
       <c r="H136" s="10"/>
     </row>
     <row r="137" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B137" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-minimum-effort/", "1631")</f>
@@ -4935,13 +4945,13 @@
         <v>11</v>
       </c>
       <c r="G137" s="16" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="H137" s="17"/>
     </row>
     <row r="138" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B138" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/", "1334")</f>
@@ -4961,13 +4971,13 @@
         <v>11</v>
       </c>
       <c r="G138" s="9" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="H138" s="10"/>
     </row>
     <row r="139" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="11" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="B139" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-ways-to-arrive-at-destination/", "1976")</f>
@@ -4987,13 +4997,13 @@
         <v>11</v>
       </c>
       <c r="G139" s="16" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="H139" s="17"/>
     </row>
     <row r="140" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B140" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/min-cost-to-connect-all-points/", "1584")</f>
@@ -5013,13 +5023,13 @@
         <v>11</v>
       </c>
       <c r="G140" s="9" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="H140" s="10"/>
     </row>
     <row r="141" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B141" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/connecting-cities-with-minimum-cost/", "1135")</f>
@@ -5039,15 +5049,15 @@
         <v>11</v>
       </c>
       <c r="G141" s="16" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="H141" s="19" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B142" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/optimize-water-distribution-in-a-village/", "1168")</f>
@@ -5067,15 +5077,15 @@
         <v>11</v>
       </c>
       <c r="G142" s="9" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="H142" s="20" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B143" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-critical-and-pseudo-critical-edges-in-minimum-spanning-tree/", "1489")</f>
@@ -5095,13 +5105,13 @@
         <v>11</v>
       </c>
       <c r="G143" s="16" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="H143" s="17"/>
     </row>
     <row r="144" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B144" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swim-in-rising-water/", "778")</f>
@@ -5121,13 +5131,13 @@
         <v>11</v>
       </c>
       <c r="G144" s="9" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="H144" s="10"/>
     </row>
     <row r="145" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="11" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B145" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-minimum-value/", "1102")</f>
@@ -5147,15 +5157,15 @@
         <v>11</v>
       </c>
       <c r="G145" s="16" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="H145" s="19" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B146" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/implement-trie-prefix-tree/", "208")</f>
@@ -5175,13 +5185,13 @@
         <v>11</v>
       </c>
       <c r="G146" s="9" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="H146" s="10"/>
     </row>
     <row r="147" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B147" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/design-add-and-search-words-data-structure/", "211")</f>
@@ -5201,13 +5211,13 @@
         <v>11</v>
       </c>
       <c r="G147" s="16" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="H147" s="17"/>
     </row>
     <row r="148" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B148" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search-ii/", "212")</f>
@@ -5227,13 +5237,13 @@
         <v>11</v>
       </c>
       <c r="G148" s="9" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H148" s="10"/>
     </row>
     <row r="149" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B149" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/replace-words/", "648")</f>
@@ -5253,13 +5263,13 @@
         <v>11</v>
       </c>
       <c r="G149" s="16" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="H149" s="17"/>
     </row>
     <row r="150" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B150" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/map-sum-pairs/", "677")</f>
@@ -5279,13 +5289,13 @@
         <v>11</v>
       </c>
       <c r="G150" s="9" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="H150" s="10"/>
     </row>
     <row r="151" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="11" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="B151" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-suggestions-system/", "1268")</f>
@@ -5305,13 +5315,13 @@
         <v>11</v>
       </c>
       <c r="G151" s="16" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="H151" s="17"/>
     </row>
     <row r="152" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B152" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number/", "136")</f>
@@ -5322,7 +5332,7 @@
         <v>Single Number</v>
       </c>
       <c r="D152" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E152" s="8" t="s">
         <v>11</v>
@@ -5331,13 +5341,13 @@
         <v>11</v>
       </c>
       <c r="G152" s="9" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="H152" s="10"/>
     </row>
     <row r="153" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B153" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number-ii/", "137")</f>
@@ -5357,13 +5367,13 @@
         <v>11</v>
       </c>
       <c r="G153" s="16" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="H153" s="17"/>
     </row>
     <row r="154" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B154" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-1-bits/", "191")</f>
@@ -5374,7 +5384,7 @@
         <v>Number of 1 Bits</v>
       </c>
       <c r="D154" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E154" s="8" t="s">
         <v>11</v>
@@ -5383,13 +5393,13 @@
         <v>11</v>
       </c>
       <c r="G154" s="9" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="H154" s="10"/>
     </row>
     <row r="155" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B155" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/counting-bits/", "338")</f>
@@ -5400,7 +5410,7 @@
         <v>Counting Bits</v>
       </c>
       <c r="D155" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E155" s="15" t="s">
         <v>11</v>
@@ -5409,13 +5419,13 @@
         <v>11</v>
       </c>
       <c r="G155" s="16" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="H155" s="17"/>
     </row>
     <row r="156" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B156" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/missing-number/", "268")</f>
@@ -5426,7 +5436,7 @@
         <v>Missing Number</v>
       </c>
       <c r="D156" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E156" s="8" t="s">
         <v>11</v>
@@ -5435,13 +5445,13 @@
         <v>11</v>
       </c>
       <c r="G156" s="9" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="H156" s="10"/>
     </row>
     <row r="157" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="11" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B157" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-bits/", "190")</f>
@@ -5452,7 +5462,7 @@
         <v>Reverse Bits</v>
       </c>
       <c r="D157" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E157" s="15" t="s">
         <v>11</v>
@@ -5461,13 +5471,13 @@
         <v>11</v>
       </c>
       <c r="G157" s="16" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="H157" s="17"/>
     </row>
     <row r="158" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B158" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/climbing-stairs/", "70")</f>
@@ -5478,7 +5488,7 @@
         <v>Climbing Stairs</v>
       </c>
       <c r="D158" s="18" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="E158" s="8" t="s">
         <v>11</v>
@@ -5487,13 +5497,13 @@
         <v>11</v>
       </c>
       <c r="G158" s="9" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="H158" s="10"/>
     </row>
     <row r="159" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B159" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber/", "198")</f>
@@ -5513,13 +5523,13 @@
         <v>11</v>
       </c>
       <c r="G159" s="16" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="H159" s="17"/>
     </row>
     <row r="160" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B160" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber-ii/", "213")</f>
@@ -5539,13 +5549,13 @@
         <v>11</v>
       </c>
       <c r="G160" s="9" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="H160" s="10"/>
     </row>
     <row r="161" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B161" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change/", "322")</f>
@@ -5565,13 +5575,13 @@
         <v>11</v>
       </c>
       <c r="G161" s="16" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="H161" s="17"/>
     </row>
     <row r="162" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B162" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/perfect-squares/", "279")</f>
@@ -5591,13 +5601,13 @@
         <v>11</v>
       </c>
       <c r="G162" s="9" t="s">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="H162" s="10"/>
     </row>
     <row r="163" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="11" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B163" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-increasing-subsequence/", "300")</f>
@@ -5617,13 +5627,13 @@
         <v>11</v>
       </c>
       <c r="G163" s="16" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="H163" s="17"/>
     </row>
     <row r="164" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B164" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-equal-subset-sum/", "416")</f>
@@ -5643,13 +5653,13 @@
         <v>11</v>
       </c>
       <c r="G164" s="9" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="H164" s="10"/>
     </row>
     <row r="165" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="11" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B165" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/target-sum/", "494")</f>
@@ -5669,13 +5679,13 @@
         <v>11</v>
       </c>
       <c r="G165" s="16" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="H165" s="17"/>
     </row>
     <row r="166" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B166" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change-ii/", "518")</f>
@@ -5695,13 +5705,13 @@
         <v>11</v>
       </c>
       <c r="G166" s="9" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="H166" s="10"/>
     </row>
     <row r="167" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="11" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B167" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/ones-and-zeroes/", "474")</f>
@@ -5721,13 +5731,13 @@
         <v>11</v>
       </c>
       <c r="G167" s="16" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="H167" s="17"/>
     </row>
     <row r="168" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="3" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B168" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight-ii/", "1049")</f>
@@ -5747,13 +5757,13 @@
         <v>11</v>
       </c>
       <c r="G168" s="9" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="H168" s="10"/>
     </row>
     <row r="169" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="11" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="B169" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/profitable-schemes/", "879")</f>
@@ -5773,13 +5783,13 @@
         <v>11</v>
       </c>
       <c r="G169" s="16" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="H169" s="17"/>
     </row>
     <row r="170" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B170" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths/", "62")</f>
@@ -5799,13 +5809,13 @@
         <v>11</v>
       </c>
       <c r="G170" s="9" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="H170" s="10"/>
     </row>
     <row r="171" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B171" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths-ii/", "63")</f>
@@ -5825,13 +5835,13 @@
         <v>11</v>
       </c>
       <c r="G171" s="16" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="H171" s="17"/>
     </row>
     <row r="172" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B172" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-path-sum/", "64")</f>
@@ -5851,13 +5861,13 @@
         <v>11</v>
       </c>
       <c r="G172" s="9" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="H172" s="10"/>
     </row>
     <row r="173" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="11" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B173" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-square/", "221")</f>
@@ -5877,13 +5887,13 @@
         <v>11</v>
       </c>
       <c r="G173" s="16" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="H173" s="17"/>
     </row>
     <row r="174" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B174" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-falling-path-sum/", "931")</f>
@@ -5903,13 +5913,13 @@
         <v>11</v>
       </c>
       <c r="G174" s="9" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="H174" s="10"/>
     </row>
     <row r="175" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="11" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="B175" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/triangle/", "120")</f>
@@ -5929,13 +5939,13 @@
         <v>11</v>
       </c>
       <c r="G175" s="16" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="H175" s="17"/>
     </row>
     <row r="176" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B176" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-common-subsequence/", "1143")</f>
@@ -5955,13 +5965,13 @@
         <v>11</v>
       </c>
       <c r="G176" s="9" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="H176" s="10"/>
     </row>
     <row r="177" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="11" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B177" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/edit-distance/", "72")</f>
@@ -5981,13 +5991,13 @@
         <v>11</v>
       </c>
       <c r="G177" s="16" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="H177" s="17"/>
     </row>
     <row r="178" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B178" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/distinct-subsequences/", "115")</f>
@@ -6007,13 +6017,13 @@
         <v>11</v>
       </c>
       <c r="G178" s="9" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="H178" s="10"/>
     </row>
     <row r="179" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="11" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B179" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-operation-for-two-strings/", "583")</f>
@@ -6033,13 +6043,13 @@
         <v>11</v>
       </c>
       <c r="G179" s="16" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="H179" s="17"/>
     </row>
     <row r="180" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="3" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B180" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/interleaving-string/", "97")</f>
@@ -6059,13 +6069,13 @@
         <v>11</v>
       </c>
       <c r="G180" s="9" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="H180" s="10"/>
     </row>
     <row r="181" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="11" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B181" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-insertion-steps-to-make-a-string-palindrome/", "1312")</f>
@@ -6085,7 +6095,7 @@
         <v>11</v>
       </c>
       <c r="G181" s="16" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="H181" s="17"/>
     </row>

</xml_diff>

<commit_message>
finished linked list problems and 4sum. updated spreadsheet.
</commit_message>
<xml_diff>
--- a/leetcode_roadmap.xlsx
+++ b/leetcode_roadmap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="922" uniqueCount="230">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="233">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -118,6 +118,9 @@
     <t xml:space="preserve">https://leetcode.com/problems/4sum/</t>
   </si>
   <si>
+    <t xml:space="preserve">Using 3sum and 2sum together. No overthinking.</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/trapping-rain-water/</t>
   </si>
   <si>
@@ -133,7 +136,13 @@
     <t xml:space="preserve">https://leetcode.com/problems/linked-list-cycle/</t>
   </si>
   <si>
+    <t xml:space="preserve">very simple. Fast and slow pointers. Don’t overcomplicate.</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/linked-list-cycle-ii/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">easy if using extra memory. Tricky if not. Remember tortoise-hare pattern for most linked list problems.</t>
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
@@ -1669,8 +1678,8 @@
       <c r="D11" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E11" s="15" t="s">
-        <v>11</v>
+      <c r="E11" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F11" s="15" t="s">
         <v>11</v>
@@ -1678,7 +1687,9 @@
       <c r="G11" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="H11" s="17"/>
+      <c r="H11" s="17" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
@@ -1702,7 +1713,7 @@
         <v>11</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="H12" s="10"/>
     </row>
@@ -1728,13 +1739,13 @@
         <v>11</v>
       </c>
       <c r="G13" s="16" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="H13" s="17"/>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B14" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/linked-list-cycle/", "141")</f>
@@ -1745,22 +1756,24 @@
         <v>Linked List Cycle</v>
       </c>
       <c r="D14" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="E14" s="8" t="s">
-        <v>11</v>
+        <v>35</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F14" s="8" t="s">
         <v>11</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="H14" s="10"/>
+        <v>36</v>
+      </c>
+      <c r="H14" s="10" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B15" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/linked-list-cycle-ii/", "142")</f>
@@ -1773,20 +1786,22 @@
       <c r="D15" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="15" t="s">
-        <v>11</v>
+      <c r="E15" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F15" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>36</v>
-      </c>
-      <c r="H15" s="17"/>
+        <v>38</v>
+      </c>
+      <c r="H15" s="17" t="s">
+        <v>39</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B16" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/remove-nth-node-from-end-of-list/", "19")</f>
@@ -1799,20 +1814,20 @@
       <c r="D16" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E16" s="8" t="s">
-        <v>11</v>
+      <c r="E16" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F16" s="8" t="s">
         <v>11</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="H16" s="10"/>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B17" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/middle-of-the-linked-list/", "876")</f>
@@ -1823,22 +1838,22 @@
         <v>Middle of the Linked List</v>
       </c>
       <c r="D17" s="18" t="s">
-        <v>34</v>
-      </c>
-      <c r="E17" s="15" t="s">
-        <v>11</v>
+        <v>35</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F17" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="H17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B18" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/intersection-of-two-linked-lists/", "160")</f>
@@ -1849,7 +1864,7 @@
         <v>Intersection of Two Linked Lists</v>
       </c>
       <c r="D18" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>11</v>
@@ -1858,13 +1873,13 @@
         <v>11</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="H18" s="10"/>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B19" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/palindrome-linked-list/", "234")</f>
@@ -1875,7 +1890,7 @@
         <v>Palindrome Linked List</v>
       </c>
       <c r="D19" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E19" s="15" t="s">
         <v>11</v>
@@ -1884,13 +1899,13 @@
         <v>11</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="H19" s="17"/>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B20" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-rotated-sorted-array/", "33")</f>
@@ -1910,13 +1925,13 @@
         <v>11</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="H20" s="10"/>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B21" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/", "34")</f>
@@ -1936,13 +1951,13 @@
         <v>11</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="H21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B22" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-insert-position/", "35")</f>
@@ -1953,7 +1968,7 @@
         <v>Search Insert Position</v>
       </c>
       <c r="D22" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>11</v>
@@ -1962,13 +1977,13 @@
         <v>11</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H22" s="10"/>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B23" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/", "153")</f>
@@ -1988,13 +2003,13 @@
         <v>11</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="H23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B24" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-peak-element/", "162")</f>
@@ -2014,13 +2029,13 @@
         <v>11</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="H24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B25" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-search/", "704")</f>
@@ -2031,7 +2046,7 @@
         <v>Binary Search</v>
       </c>
       <c r="D25" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E25" s="15" t="s">
         <v>11</v>
@@ -2040,13 +2055,13 @@
         <v>11</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B26" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/koko-eating-bananas/", "875")</f>
@@ -2066,13 +2081,13 @@
         <v>11</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="H26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B27" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/capacity-to-ship-packages-within-d-days/", "1011")</f>
@@ -2092,13 +2107,13 @@
         <v>11</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B28" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/split-array-largest-sum/", "410")</f>
@@ -2118,13 +2133,13 @@
         <v>11</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="H28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B29" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimize-max-distance-to-gas-station/", "774")</f>
@@ -2144,15 +2159,15 @@
         <v>11</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B30" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-smallest-divisor-given-a-threshold/", "1283")</f>
@@ -2172,13 +2187,13 @@
         <v>11</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="H30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B31" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-days-to-make-m-bouquets/", "1482")</f>
@@ -2198,13 +2213,13 @@
         <v>11</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="H31" s="17"/>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B32" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/two-sum/", "1")</f>
@@ -2215,7 +2230,7 @@
         <v>Two Sum</v>
       </c>
       <c r="D32" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>11</v>
@@ -2224,13 +2239,13 @@
         <v>11</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="H32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B33" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/group-anagrams/", "49")</f>
@@ -2250,13 +2265,13 @@
         <v>11</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B34" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-consecutive-sequence/", "128")</f>
@@ -2276,13 +2291,13 @@
         <v>11</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="H34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B35" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/contains-duplicate/", "217")</f>
@@ -2293,7 +2308,7 @@
         <v>Contains Duplicate</v>
       </c>
       <c r="D35" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E35" s="15" t="s">
         <v>11</v>
@@ -2302,13 +2317,13 @@
         <v>11</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="H35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B36" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/valid-anagram/", "242")</f>
@@ -2319,7 +2334,7 @@
         <v>Valid Anagram</v>
       </c>
       <c r="D36" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E36" s="8" t="s">
         <v>11</v>
@@ -2328,13 +2343,13 @@
         <v>11</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="H36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="B37" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -2354,13 +2369,13 @@
         <v>11</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B38" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-sum-query-immutable/", "303")</f>
@@ -2371,7 +2386,7 @@
         <v>Range Sum Query - Immutable</v>
       </c>
       <c r="D38" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E38" s="8" t="s">
         <v>11</v>
@@ -2380,13 +2395,13 @@
         <v>11</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B39" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sum-equals-k/", "560")</f>
@@ -2406,13 +2421,13 @@
         <v>11</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="H39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B40" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-pivot-index/", "724")</f>
@@ -2423,7 +2438,7 @@
         <v>Find Pivot Index</v>
       </c>
       <c r="D40" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E40" s="8" t="s">
         <v>11</v>
@@ -2432,13 +2447,13 @@
         <v>11</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="H40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B41" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-subarrays-with-sum/", "930")</f>
@@ -2458,13 +2473,13 @@
         <v>11</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H41" s="17"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B42" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sums-divisible-by-k/", "974")</f>
@@ -2484,13 +2499,13 @@
         <v>11</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="B43" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/continuous-subarray-sum/", "523")</f>
@@ -2510,13 +2525,13 @@
         <v>11</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B44" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-addition/", "370")</f>
@@ -2536,15 +2551,15 @@
         <v>11</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H44" s="20" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B45" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/car-pooling/", "1094")</f>
@@ -2564,13 +2579,13 @@
         <v>11</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="H45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B46" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/corporate-flight-bookings/", "1109")</f>
@@ -2590,13 +2605,13 @@
         <v>11</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="H46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B47" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/check-if-all-the-integers-in-a-range-are-covered/", "1893")</f>
@@ -2607,7 +2622,7 @@
         <v>Check if All the Integers in a Range Are Covered</v>
       </c>
       <c r="D47" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E47" s="15" t="s">
         <v>11</v>
@@ -2616,13 +2631,13 @@
         <v>11</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B48" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/describe-the-painting/", "1943")</f>
@@ -2642,13 +2657,13 @@
         <v>11</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B49" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shifting-letters-ii/", "2381")</f>
@@ -2668,13 +2683,13 @@
         <v>11</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H49" s="17"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B50" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/daily-temperatures/", "739")</f>
@@ -2694,13 +2709,13 @@
         <v>11</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B51" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-i/", "496")</f>
@@ -2711,7 +2726,7 @@
         <v>Next Greater Element I</v>
       </c>
       <c r="D51" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E51" s="15" t="s">
         <v>11</v>
@@ -2720,13 +2735,13 @@
         <v>11</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="H51" s="17"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B52" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-ii/", "503")</f>
@@ -2746,13 +2761,13 @@
         <v>11</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="H52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B53" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/largest-rectangle-in-histogram/", "84")</f>
@@ -2772,13 +2787,13 @@
         <v>11</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="H53" s="17"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B54" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-rectangle/", "85")</f>
@@ -2798,13 +2813,13 @@
         <v>11</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="B55" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/online-stock-span/", "901")</f>
@@ -2824,13 +2839,13 @@
         <v>11</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="H55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B56" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sliding-window-maximum/", "239")</f>
@@ -2850,13 +2865,13 @@
         <v>11</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="H56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B57" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-subarray-with-sum-at-least-k/", "862")</f>
@@ -2876,13 +2891,13 @@
         <v>11</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="H57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B58" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/constrained-subsequence-sum/", "1425")</f>
@@ -2902,13 +2917,13 @@
         <v>11</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="H58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B59" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-continuous-subarray-with-absolute-diff-less-than-or-equal-to-limit/", "1438")</f>
@@ -2928,13 +2943,13 @@
         <v>11</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="H59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B60" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-value-of-equation/", "1499")</f>
@@ -2954,13 +2969,13 @@
         <v>11</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="H60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="B61" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-vi/", "1696")</f>
@@ -2980,13 +2995,13 @@
         <v>11</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="H61" s="17"/>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B62" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-an-array/", "215")</f>
@@ -3006,13 +3021,13 @@
         <v>11</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="H62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B63" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -3032,13 +3047,13 @@
         <v>11</v>
       </c>
       <c r="G63" s="16" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="H63" s="17"/>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B64" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-words/", "692")</f>
@@ -3058,13 +3073,13 @@
         <v>11</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="H64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B65" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-a-stream/", "703")</f>
@@ -3075,7 +3090,7 @@
         <v>Kth Largest Element in a Stream</v>
       </c>
       <c r="D65" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E65" s="15" t="s">
         <v>11</v>
@@ -3084,13 +3099,13 @@
         <v>11</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="H65" s="17"/>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B66" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/k-closest-points-to-origin/", "973")</f>
@@ -3110,13 +3125,13 @@
         <v>11</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="H66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B67" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight/", "1046")</f>
@@ -3127,7 +3142,7 @@
         <v>Last Stone Weight</v>
       </c>
       <c r="D67" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E67" s="15" t="s">
         <v>11</v>
@@ -3136,13 +3151,13 @@
         <v>11</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="H67" s="17"/>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B68" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-intervals/", "56")</f>
@@ -3162,13 +3177,13 @@
         <v>11</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="H68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B69" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/insert-interval/", "57")</f>
@@ -3188,13 +3203,13 @@
         <v>11</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="H69" s="17"/>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B70" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms/", "252")</f>
@@ -3205,7 +3220,7 @@
         <v>Meeting Rooms</v>
       </c>
       <c r="D70" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E70" s="8" t="s">
         <v>11</v>
@@ -3214,15 +3229,15 @@
         <v>11</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="H70" s="20" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B71" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms-ii/", "253")</f>
@@ -3242,15 +3257,15 @@
         <v>11</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="H71" s="19" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B72" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/non-overlapping-intervals/", "435")</f>
@@ -3270,13 +3285,13 @@
         <v>11</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="H72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="B73" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-arrows-to-burst-balloons/", "452")</f>
@@ -3296,13 +3311,13 @@
         <v>11</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="H73" s="17"/>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B74" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-ii/", "45")</f>
@@ -3322,13 +3337,13 @@
         <v>11</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="H74" s="10"/>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B75" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game/", "55")</f>
@@ -3348,13 +3363,13 @@
         <v>11</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="H75" s="17"/>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B76" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/queue-reconstruction-by-height/", "406")</f>
@@ -3374,13 +3389,13 @@
         <v>11</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="H76" s="10"/>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B77" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/task-scheduler/", "621")</f>
@@ -3400,13 +3415,13 @@
         <v>11</v>
       </c>
       <c r="G77" s="16" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="H77" s="17"/>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B78" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-labels/", "763")</f>
@@ -3426,13 +3441,13 @@
         <v>11</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="H78" s="10"/>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B79" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/gas-station/", "134")</f>
@@ -3452,13 +3467,13 @@
         <v>11</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="H79" s="17"/>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B80" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/", "21")</f>
@@ -3469,7 +3484,7 @@
         <v>Merge Two Sorted Lists</v>
       </c>
       <c r="D80" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E80" s="8" t="s">
         <v>11</v>
@@ -3478,13 +3493,13 @@
         <v>11</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="H80" s="10"/>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B81" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-k-sorted-lists/", "23")</f>
@@ -3504,13 +3519,13 @@
         <v>11</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="H81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B82" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swap-nodes-in-pairs/", "24")</f>
@@ -3530,13 +3545,13 @@
         <v>11</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="H82" s="10"/>
     </row>
     <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B83" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-nodes-in-k-group/", "25")</f>
@@ -3556,13 +3571,13 @@
         <v>11</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="H83" s="17"/>
     </row>
     <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B84" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-linked-list-ii/", "92")</f>
@@ -3582,13 +3597,13 @@
         <v>11</v>
       </c>
       <c r="G84" s="9" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="H84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B85" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/copy-list-with-random-pointer/", "138")</f>
@@ -3608,13 +3623,13 @@
         <v>11</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="H85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B86" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximum-depth-of-binary-tree/", "104")</f>
@@ -3625,7 +3640,7 @@
         <v>Maximum Depth of Binary Tree</v>
       </c>
       <c r="D86" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E86" s="8" t="s">
         <v>11</v>
@@ -3634,13 +3649,13 @@
         <v>11</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="H86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B87" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum/", "112")</f>
@@ -3651,7 +3666,7 @@
         <v>Path Sum</v>
       </c>
       <c r="D87" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E87" s="15" t="s">
         <v>11</v>
@@ -3660,13 +3675,13 @@
         <v>11</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="H87" s="17"/>
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B88" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum-ii/", "113")</f>
@@ -3686,13 +3701,13 @@
         <v>11</v>
       </c>
       <c r="G88" s="9" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="H88" s="10"/>
     </row>
     <row r="89" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B89" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/diameter-of-binary-tree/", "543")</f>
@@ -3703,7 +3718,7 @@
         <v>Diameter of Binary Tree</v>
       </c>
       <c r="D89" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E89" s="15" t="s">
         <v>11</v>
@@ -3712,13 +3727,13 @@
         <v>11</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="H89" s="17"/>
     </row>
     <row r="90" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B90" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-maximum-path-sum/", "124")</f>
@@ -3738,13 +3753,13 @@
         <v>11</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="H90" s="10"/>
     </row>
     <row r="91" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B91" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/invert-binary-tree/", "226")</f>
@@ -3755,7 +3770,7 @@
         <v>Invert Binary Tree</v>
       </c>
       <c r="D91" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E91" s="15" t="s">
         <v>11</v>
@@ -3764,13 +3779,13 @@
         <v>11</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="H91" s="17"/>
     </row>
     <row r="92" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B92" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-level-order-traversal/", "102")</f>
@@ -3790,13 +3805,13 @@
         <v>11</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="H92" s="10"/>
     </row>
     <row r="93" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B93" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/", "103")</f>
@@ -3816,13 +3831,13 @@
         <v>11</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="H93" s="17"/>
     </row>
     <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B94" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-right-side-view/", "199")</f>
@@ -3842,13 +3857,13 @@
         <v>11</v>
       </c>
       <c r="G94" s="9" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="H94" s="10"/>
     </row>
     <row r="95" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B95" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-largest-value-in-each-tree-row/", "515")</f>
@@ -3868,13 +3883,13 @@
         <v>11</v>
       </c>
       <c r="G95" s="16" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="H95" s="17"/>
     </row>
     <row r="96" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B96" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/average-of-levels-in-binary-tree/", "637")</f>
@@ -3885,7 +3900,7 @@
         <v>Average of Levels in Binary Tree</v>
       </c>
       <c r="D96" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E96" s="8" t="s">
         <v>11</v>
@@ -3894,13 +3909,13 @@
         <v>11</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="H96" s="10"/>
     </row>
     <row r="97" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B97" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/populating-next-right-pointers-in-each-node/", "116")</f>
@@ -3920,13 +3935,13 @@
         <v>11</v>
       </c>
       <c r="G97" s="16" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H97" s="17"/>
     </row>
     <row r="98" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B98" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/validate-binary-search-tree/", "98")</f>
@@ -3946,13 +3961,13 @@
         <v>11</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="H98" s="10"/>
     </row>
     <row r="99" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B99" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/recover-binary-search-tree/", "99")</f>
@@ -3972,13 +3987,13 @@
         <v>11</v>
       </c>
       <c r="G99" s="16" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="H99" s="17"/>
     </row>
     <row r="100" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B100" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-smallest-element-in-a-bst/", "230")</f>
@@ -3998,13 +4013,13 @@
         <v>11</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="H100" s="10"/>
     </row>
     <row r="101" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B101" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/", "235")</f>
@@ -4024,13 +4039,13 @@
         <v>11</v>
       </c>
       <c r="G101" s="16" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="H101" s="17"/>
     </row>
     <row r="102" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B102" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-node-in-a-bst/", "450")</f>
@@ -4050,13 +4065,13 @@
         <v>11</v>
       </c>
       <c r="G102" s="9" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="H102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B103" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-a-binary-search-tree/", "700")</f>
@@ -4067,7 +4082,7 @@
         <v>Search in a Binary Search Tree</v>
       </c>
       <c r="D103" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E103" s="15" t="s">
         <v>11</v>
@@ -4076,13 +4091,13 @@
         <v>11</v>
       </c>
       <c r="G103" s="16" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="H103" s="17"/>
     </row>
     <row r="104" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B104" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations/", "46")</f>
@@ -4102,13 +4117,13 @@
         <v>11</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="H104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B105" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations-ii/", "47")</f>
@@ -4128,13 +4143,13 @@
         <v>11</v>
       </c>
       <c r="G105" s="16" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="H105" s="17"/>
     </row>
     <row r="106" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B106" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combinations/", "77")</f>
@@ -4154,13 +4169,13 @@
         <v>11</v>
       </c>
       <c r="G106" s="9" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="H106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B107" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets/", "78")</f>
@@ -4180,13 +4195,13 @@
         <v>11</v>
       </c>
       <c r="G107" s="16" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="H107" s="17"/>
     </row>
     <row r="108" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B108" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets-ii/", "90")</f>
@@ -4206,13 +4221,13 @@
         <v>11</v>
       </c>
       <c r="G108" s="9" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="H108" s="10"/>
     </row>
     <row r="109" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="11" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B109" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum/", "39")</f>
@@ -4232,13 +4247,13 @@
         <v>11</v>
       </c>
       <c r="G109" s="16" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="H109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B110" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum-ii/", "40")</f>
@@ -4258,13 +4273,13 @@
         <v>11</v>
       </c>
       <c r="G110" s="9" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="H110" s="10"/>
     </row>
     <row r="111" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B111" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/letter-combinations-of-a-phone-number/", "17")</f>
@@ -4284,13 +4299,13 @@
         <v>11</v>
       </c>
       <c r="G111" s="16" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="H111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B112" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search/", "79")</f>
@@ -4310,13 +4325,13 @@
         <v>11</v>
       </c>
       <c r="G112" s="9" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="H112" s="10"/>
     </row>
     <row r="113" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B113" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/palindrome-partitioning/", "131")</f>
@@ -4336,13 +4351,13 @@
         <v>11</v>
       </c>
       <c r="G113" s="16" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="H113" s="17"/>
     </row>
     <row r="114" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B114" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens/", "51")</f>
@@ -4362,13 +4377,13 @@
         <v>11</v>
       </c>
       <c r="G114" s="9" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="H114" s="10"/>
     </row>
     <row r="115" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B115" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens-ii/", "52")</f>
@@ -4388,13 +4403,13 @@
         <v>11</v>
       </c>
       <c r="G115" s="16" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="H115" s="17"/>
     </row>
     <row r="116" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B116" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-islands/", "200")</f>
@@ -4414,13 +4429,13 @@
         <v>11</v>
       </c>
       <c r="G116" s="9" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="H116" s="10"/>
     </row>
     <row r="117" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="11" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B117" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-area-of-island/", "695")</f>
@@ -4440,13 +4455,13 @@
         <v>11</v>
       </c>
       <c r="G117" s="16" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="H117" s="17"/>
     </row>
     <row r="118" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B118" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/flood-fill/", "733")</f>
@@ -4457,7 +4472,7 @@
         <v>Flood Fill</v>
       </c>
       <c r="D118" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E118" s="8" t="s">
         <v>11</v>
@@ -4466,13 +4481,13 @@
         <v>11</v>
       </c>
       <c r="G118" s="9" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="H118" s="10"/>
     </row>
     <row r="119" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B119" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/rotting-oranges/", "994")</f>
@@ -4492,13 +4507,13 @@
         <v>11</v>
       </c>
       <c r="G119" s="16" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="H119" s="17"/>
     </row>
     <row r="120" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B120" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-path-in-binary-matrix/", "1091")</f>
@@ -4518,13 +4533,13 @@
         <v>11</v>
       </c>
       <c r="G120" s="9" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="H120" s="10"/>
     </row>
     <row r="121" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="11" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B121" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-closed-islands/", "1254")</f>
@@ -4544,13 +4559,13 @@
         <v>11</v>
       </c>
       <c r="G121" s="16" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="H121" s="17"/>
     </row>
     <row r="122" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B122" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule/", "207")</f>
@@ -4570,13 +4585,13 @@
         <v>11</v>
       </c>
       <c r="G122" s="9" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="H122" s="10"/>
     </row>
     <row r="123" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B123" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-ii/", "210")</f>
@@ -4596,13 +4611,13 @@
         <v>11</v>
       </c>
       <c r="G123" s="16" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="H123" s="17"/>
     </row>
     <row r="124" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B124" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-eventual-safe-states/", "802")</f>
@@ -4622,13 +4637,13 @@
         <v>11</v>
       </c>
       <c r="G124" s="9" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="H124" s="10"/>
     </row>
     <row r="125" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B125" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-iv/", "1462")</f>
@@ -4648,13 +4663,13 @@
         <v>11</v>
       </c>
       <c r="G125" s="16" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="H125" s="17"/>
     </row>
     <row r="126" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B126" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sort-items-by-groups-respecting-dependencies/", "1203")</f>
@@ -4674,13 +4689,13 @@
         <v>11</v>
       </c>
       <c r="G126" s="9" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="H126" s="10"/>
     </row>
     <row r="127" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="11" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B127" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-all-possible-recipes-from-given-supplies/", "2115")</f>
@@ -4700,13 +4715,13 @@
         <v>11</v>
       </c>
       <c r="G127" s="16" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="H127" s="17"/>
     </row>
     <row r="128" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B128" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-provinces/", "547")</f>
@@ -4726,13 +4741,13 @@
         <v>11</v>
       </c>
       <c r="G128" s="9" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="H128" s="10"/>
     </row>
     <row r="129" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="11" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B129" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/redundant-connection/", "684")</f>
@@ -4752,13 +4767,13 @@
         <v>11</v>
       </c>
       <c r="G129" s="16" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="H129" s="17"/>
     </row>
     <row r="130" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B130" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-operations-to-make-network-connected/", "1319")</f>
@@ -4778,13 +4793,13 @@
         <v>11</v>
       </c>
       <c r="G130" s="9" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="H130" s="10"/>
     </row>
     <row r="131" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="11" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B131" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/remove-max-number-of-edges-to-keep-graph-fully-traversable/", "1579")</f>
@@ -4804,13 +4819,13 @@
         <v>11</v>
       </c>
       <c r="G131" s="16" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="H131" s="17"/>
     </row>
     <row r="132" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B132" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/satisfiability-of-equality-equations/", "990")</f>
@@ -4830,13 +4845,13 @@
         <v>11</v>
       </c>
       <c r="G132" s="9" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="H132" s="10"/>
     </row>
     <row r="133" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="11" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B133" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/smallest-string-with-swaps/", "1202")</f>
@@ -4856,13 +4871,13 @@
         <v>11</v>
       </c>
       <c r="G133" s="16" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="H133" s="17"/>
     </row>
     <row r="134" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B134" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/network-delay-time/", "743")</f>
@@ -4882,13 +4897,13 @@
         <v>11</v>
       </c>
       <c r="G134" s="9" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="H134" s="10"/>
     </row>
     <row r="135" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="11" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B135" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/cheapest-flights-within-k-stops/", "787")</f>
@@ -4908,13 +4923,13 @@
         <v>11</v>
       </c>
       <c r="G135" s="16" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="H135" s="17"/>
     </row>
     <row r="136" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B136" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-probability/", "1514")</f>
@@ -4934,13 +4949,13 @@
         <v>11</v>
       </c>
       <c r="G136" s="9" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="H136" s="10"/>
     </row>
     <row r="137" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="11" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B137" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-minimum-effort/", "1631")</f>
@@ -4960,13 +4975,13 @@
         <v>11</v>
       </c>
       <c r="G137" s="16" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="H137" s="17"/>
     </row>
     <row r="138" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B138" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/", "1334")</f>
@@ -4986,13 +5001,13 @@
         <v>11</v>
       </c>
       <c r="G138" s="9" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="H138" s="10"/>
     </row>
     <row r="139" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="11" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B139" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-ways-to-arrive-at-destination/", "1976")</f>
@@ -5012,13 +5027,13 @@
         <v>11</v>
       </c>
       <c r="G139" s="16" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="H139" s="17"/>
     </row>
     <row r="140" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B140" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/min-cost-to-connect-all-points/", "1584")</f>
@@ -5038,13 +5053,13 @@
         <v>11</v>
       </c>
       <c r="G140" s="9" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="H140" s="10"/>
     </row>
     <row r="141" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="11" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B141" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/connecting-cities-with-minimum-cost/", "1135")</f>
@@ -5064,15 +5079,15 @@
         <v>11</v>
       </c>
       <c r="G141" s="16" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="H141" s="19" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B142" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/optimize-water-distribution-in-a-village/", "1168")</f>
@@ -5092,15 +5107,15 @@
         <v>11</v>
       </c>
       <c r="G142" s="9" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="H142" s="20" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="11" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B143" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-critical-and-pseudo-critical-edges-in-minimum-spanning-tree/", "1489")</f>
@@ -5120,13 +5135,13 @@
         <v>11</v>
       </c>
       <c r="G143" s="16" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="H143" s="17"/>
     </row>
     <row r="144" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B144" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swim-in-rising-water/", "778")</f>
@@ -5146,13 +5161,13 @@
         <v>11</v>
       </c>
       <c r="G144" s="9" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="H144" s="10"/>
     </row>
     <row r="145" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="11" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="B145" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-minimum-value/", "1102")</f>
@@ -5172,15 +5187,15 @@
         <v>11</v>
       </c>
       <c r="G145" s="16" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="H145" s="19" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B146" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/implement-trie-prefix-tree/", "208")</f>
@@ -5200,13 +5215,13 @@
         <v>11</v>
       </c>
       <c r="G146" s="9" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="H146" s="10"/>
     </row>
     <row r="147" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="11" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B147" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/design-add-and-search-words-data-structure/", "211")</f>
@@ -5226,13 +5241,13 @@
         <v>11</v>
       </c>
       <c r="G147" s="16" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="H147" s="17"/>
     </row>
     <row r="148" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B148" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search-ii/", "212")</f>
@@ -5252,13 +5267,13 @@
         <v>11</v>
       </c>
       <c r="G148" s="9" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="H148" s="10"/>
     </row>
     <row r="149" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B149" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/replace-words/", "648")</f>
@@ -5278,13 +5293,13 @@
         <v>11</v>
       </c>
       <c r="G149" s="16" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="H149" s="17"/>
     </row>
     <row r="150" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B150" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/map-sum-pairs/", "677")</f>
@@ -5304,13 +5319,13 @@
         <v>11</v>
       </c>
       <c r="G150" s="9" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="H150" s="10"/>
     </row>
     <row r="151" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="11" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B151" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-suggestions-system/", "1268")</f>
@@ -5330,13 +5345,13 @@
         <v>11</v>
       </c>
       <c r="G151" s="16" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="H151" s="17"/>
     </row>
     <row r="152" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B152" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number/", "136")</f>
@@ -5347,7 +5362,7 @@
         <v>Single Number</v>
       </c>
       <c r="D152" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E152" s="8" t="s">
         <v>11</v>
@@ -5356,13 +5371,13 @@
         <v>11</v>
       </c>
       <c r="G152" s="9" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="H152" s="10"/>
     </row>
     <row r="153" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="11" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B153" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number-ii/", "137")</f>
@@ -5382,13 +5397,13 @@
         <v>11</v>
       </c>
       <c r="G153" s="16" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="H153" s="17"/>
     </row>
     <row r="154" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B154" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-1-bits/", "191")</f>
@@ -5399,7 +5414,7 @@
         <v>Number of 1 Bits</v>
       </c>
       <c r="D154" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E154" s="8" t="s">
         <v>11</v>
@@ -5408,13 +5423,13 @@
         <v>11</v>
       </c>
       <c r="G154" s="9" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="H154" s="10"/>
     </row>
     <row r="155" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="11" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B155" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/counting-bits/", "338")</f>
@@ -5425,7 +5440,7 @@
         <v>Counting Bits</v>
       </c>
       <c r="D155" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E155" s="15" t="s">
         <v>11</v>
@@ -5434,13 +5449,13 @@
         <v>11</v>
       </c>
       <c r="G155" s="16" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="H155" s="17"/>
     </row>
     <row r="156" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B156" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/missing-number/", "268")</f>
@@ -5451,7 +5466,7 @@
         <v>Missing Number</v>
       </c>
       <c r="D156" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E156" s="8" t="s">
         <v>11</v>
@@ -5460,13 +5475,13 @@
         <v>11</v>
       </c>
       <c r="G156" s="9" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="H156" s="10"/>
     </row>
     <row r="157" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="11" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B157" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-bits/", "190")</f>
@@ -5477,7 +5492,7 @@
         <v>Reverse Bits</v>
       </c>
       <c r="D157" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E157" s="15" t="s">
         <v>11</v>
@@ -5486,13 +5501,13 @@
         <v>11</v>
       </c>
       <c r="G157" s="16" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="H157" s="17"/>
     </row>
     <row r="158" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B158" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/climbing-stairs/", "70")</f>
@@ -5503,7 +5518,7 @@
         <v>Climbing Stairs</v>
       </c>
       <c r="D158" s="18" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E158" s="8" t="s">
         <v>11</v>
@@ -5512,13 +5527,13 @@
         <v>11</v>
       </c>
       <c r="G158" s="9" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="H158" s="10"/>
     </row>
     <row r="159" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="11" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B159" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber/", "198")</f>
@@ -5538,13 +5553,13 @@
         <v>11</v>
       </c>
       <c r="G159" s="16" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="H159" s="17"/>
     </row>
     <row r="160" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B160" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber-ii/", "213")</f>
@@ -5564,13 +5579,13 @@
         <v>11</v>
       </c>
       <c r="G160" s="9" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="H160" s="10"/>
     </row>
     <row r="161" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="11" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B161" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change/", "322")</f>
@@ -5590,13 +5605,13 @@
         <v>11</v>
       </c>
       <c r="G161" s="16" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="H161" s="17"/>
     </row>
     <row r="162" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B162" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/perfect-squares/", "279")</f>
@@ -5616,13 +5631,13 @@
         <v>11</v>
       </c>
       <c r="G162" s="9" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="H162" s="10"/>
     </row>
     <row r="163" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="11" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B163" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-increasing-subsequence/", "300")</f>
@@ -5642,13 +5657,13 @@
         <v>11</v>
       </c>
       <c r="G163" s="16" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="H163" s="17"/>
     </row>
     <row r="164" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B164" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-equal-subset-sum/", "416")</f>
@@ -5668,13 +5683,13 @@
         <v>11</v>
       </c>
       <c r="G164" s="9" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="H164" s="10"/>
     </row>
     <row r="165" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="11" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B165" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/target-sum/", "494")</f>
@@ -5694,13 +5709,13 @@
         <v>11</v>
       </c>
       <c r="G165" s="16" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="H165" s="17"/>
     </row>
     <row r="166" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B166" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change-ii/", "518")</f>
@@ -5720,13 +5735,13 @@
         <v>11</v>
       </c>
       <c r="G166" s="9" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="H166" s="10"/>
     </row>
     <row r="167" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="11" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B167" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/ones-and-zeroes/", "474")</f>
@@ -5746,13 +5761,13 @@
         <v>11</v>
       </c>
       <c r="G167" s="16" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="H167" s="17"/>
     </row>
     <row r="168" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="3" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B168" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight-ii/", "1049")</f>
@@ -5772,13 +5787,13 @@
         <v>11</v>
       </c>
       <c r="G168" s="9" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="H168" s="10"/>
     </row>
     <row r="169" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="11" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B169" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/profitable-schemes/", "879")</f>
@@ -5798,13 +5813,13 @@
         <v>11</v>
       </c>
       <c r="G169" s="16" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="H169" s="17"/>
     </row>
     <row r="170" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="3" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B170" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths/", "62")</f>
@@ -5824,13 +5839,13 @@
         <v>11</v>
       </c>
       <c r="G170" s="9" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="H170" s="10"/>
     </row>
     <row r="171" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B171" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths-ii/", "63")</f>
@@ -5850,13 +5865,13 @@
         <v>11</v>
       </c>
       <c r="G171" s="16" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="H171" s="17"/>
     </row>
     <row r="172" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="3" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B172" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-path-sum/", "64")</f>
@@ -5876,13 +5891,13 @@
         <v>11</v>
       </c>
       <c r="G172" s="9" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="H172" s="10"/>
     </row>
     <row r="173" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="11" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B173" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-square/", "221")</f>
@@ -5902,13 +5917,13 @@
         <v>11</v>
       </c>
       <c r="G173" s="16" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="H173" s="17"/>
     </row>
     <row r="174" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B174" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-falling-path-sum/", "931")</f>
@@ -5928,13 +5943,13 @@
         <v>11</v>
       </c>
       <c r="G174" s="9" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="H174" s="10"/>
     </row>
     <row r="175" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="11" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B175" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/triangle/", "120")</f>
@@ -5954,13 +5969,13 @@
         <v>11</v>
       </c>
       <c r="G175" s="16" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="H175" s="17"/>
     </row>
     <row r="176" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B176" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-common-subsequence/", "1143")</f>
@@ -5980,13 +5995,13 @@
         <v>11</v>
       </c>
       <c r="G176" s="9" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="H176" s="10"/>
     </row>
     <row r="177" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="11" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B177" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/edit-distance/", "72")</f>
@@ -6006,13 +6021,13 @@
         <v>11</v>
       </c>
       <c r="G177" s="16" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="H177" s="17"/>
     </row>
     <row r="178" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B178" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/distinct-subsequences/", "115")</f>
@@ -6032,13 +6047,13 @@
         <v>11</v>
       </c>
       <c r="G178" s="9" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="H178" s="10"/>
     </row>
     <row r="179" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="11" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B179" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-operation-for-two-strings/", "583")</f>
@@ -6058,13 +6073,13 @@
         <v>11</v>
       </c>
       <c r="G179" s="16" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="H179" s="17"/>
     </row>
     <row r="180" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="3" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B180" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/interleaving-string/", "97")</f>
@@ -6084,13 +6099,13 @@
         <v>11</v>
       </c>
       <c r="G180" s="9" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="H180" s="10"/>
     </row>
     <row r="181" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="11" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B181" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-insertion-steps-to-make-a-string-palindrome/", "1312")</f>
@@ -6110,7 +6125,7 @@
         <v>11</v>
       </c>
       <c r="G181" s="16" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="H181" s="17"/>
     </row>

</xml_diff>

<commit_message>
solved 3 binary search problems
</commit_message>
<xml_diff>
--- a/leetcode_roadmap.xlsx
+++ b/leetcode_roadmap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="930" uniqueCount="238">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -148,9 +148,15 @@
     <t xml:space="preserve">https://leetcode.com/problems/remove-nth-node-from-end-of-list/</t>
   </si>
   <si>
+    <t xml:space="preserve">convert the problem into deleting the nth node from the start of the linked list (easier for me)</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/middle-of-the-linked-list/</t>
   </si>
   <si>
+    <t xml:space="preserve">Tortoise-hair algo. Once finished, slow is always going to be at the middle of the linked list.</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/intersection-of-two-linked-lists/</t>
   </si>
   <si>
@@ -163,10 +169,19 @@
     <t xml:space="preserve">https://leetcode.com/problems/search-in-rotated-sorted-array/</t>
   </si>
   <si>
+    <t xml:space="preserve">find pivot using normal binary search. Then apply binary search based on if target is greater than or less than pivot</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/</t>
   </si>
   <si>
+    <t xml:space="preserve">two separate binary searches. One for the first instance, other for last instance. When you find target, DON’T STOP!</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/search-insert-position/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">normal binary search. Once completed, left pointer will always be either equal to target or neighboring it.</t>
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/</t>
@@ -1382,11 +1397,11 @@
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="48.12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="95.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="98.71"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1823,7 +1838,9 @@
       <c r="G16" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="H16" s="10"/>
+      <c r="H16" s="10" t="s">
+        <v>41</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
@@ -1847,9 +1864,11 @@
         <v>11</v>
       </c>
       <c r="G17" s="16" t="s">
-        <v>41</v>
-      </c>
-      <c r="H17" s="17"/>
+        <v>42</v>
+      </c>
+      <c r="H17" s="17" t="s">
+        <v>43</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
@@ -1873,7 +1892,7 @@
         <v>11</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H18" s="10"/>
     </row>
@@ -1899,13 +1918,13 @@
         <v>11</v>
       </c>
       <c r="G19" s="16" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H19" s="17"/>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B20" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-rotated-sorted-array/", "33")</f>
@@ -1918,20 +1937,22 @@
       <c r="D20" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E20" s="8" t="s">
-        <v>11</v>
+      <c r="E20" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F20" s="8" t="s">
         <v>11</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="H20" s="10"/>
+        <v>47</v>
+      </c>
+      <c r="H20" s="0" t="s">
+        <v>48</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B21" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-first-and-last-position-of-element-in-sorted-array/", "34")</f>
@@ -1944,20 +1965,22 @@
       <c r="D21" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E21" s="15" t="s">
-        <v>11</v>
+      <c r="E21" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F21" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G21" s="16" t="s">
-        <v>46</v>
-      </c>
-      <c r="H21" s="17"/>
+        <v>49</v>
+      </c>
+      <c r="H21" s="17" t="s">
+        <v>50</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B22" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-insert-position/", "35")</f>
@@ -1970,20 +1993,22 @@
       <c r="D22" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E22" s="8" t="s">
-        <v>11</v>
+      <c r="E22" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F22" s="8" t="s">
         <v>11</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="H22" s="10"/>
+        <v>51</v>
+      </c>
+      <c r="H22" s="10" t="s">
+        <v>52</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B23" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/", "153")</f>
@@ -2003,13 +2028,13 @@
         <v>11</v>
       </c>
       <c r="G23" s="16" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="H23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B24" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-peak-element/", "162")</f>
@@ -2029,13 +2054,13 @@
         <v>11</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="H24" s="10"/>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B25" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-search/", "704")</f>
@@ -2055,13 +2080,13 @@
         <v>11</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="H25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B26" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/koko-eating-bananas/", "875")</f>
@@ -2081,13 +2106,13 @@
         <v>11</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="H26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B27" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/capacity-to-ship-packages-within-d-days/", "1011")</f>
@@ -2107,13 +2132,13 @@
         <v>11</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="H27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B28" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/split-array-largest-sum/", "410")</f>
@@ -2133,13 +2158,13 @@
         <v>11</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="H28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B29" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimize-max-distance-to-gas-station/", "774")</f>
@@ -2159,15 +2184,15 @@
         <v>11</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="H29" s="19" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B30" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-smallest-divisor-given-a-threshold/", "1283")</f>
@@ -2187,13 +2212,13 @@
         <v>11</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="H30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B31" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-days-to-make-m-bouquets/", "1482")</f>
@@ -2213,13 +2238,13 @@
         <v>11</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="H31" s="17"/>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B32" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/two-sum/", "1")</f>
@@ -2239,13 +2264,13 @@
         <v>11</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="H32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B33" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/group-anagrams/", "49")</f>
@@ -2265,13 +2290,13 @@
         <v>11</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="H33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B34" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-consecutive-sequence/", "128")</f>
@@ -2291,13 +2316,13 @@
         <v>11</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="H34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B35" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/contains-duplicate/", "217")</f>
@@ -2317,13 +2342,13 @@
         <v>11</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="H35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B36" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/valid-anagram/", "242")</f>
@@ -2343,13 +2368,13 @@
         <v>11</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="H36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B37" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -2369,13 +2394,13 @@
         <v>11</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="H37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B38" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-sum-query-immutable/", "303")</f>
@@ -2395,13 +2420,13 @@
         <v>11</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="H38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B39" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sum-equals-k/", "560")</f>
@@ -2421,13 +2446,13 @@
         <v>11</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="H39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B40" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-pivot-index/", "724")</f>
@@ -2447,13 +2472,13 @@
         <v>11</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="H40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B41" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-subarrays-with-sum/", "930")</f>
@@ -2473,13 +2498,13 @@
         <v>11</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="H41" s="17"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B42" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sums-divisible-by-k/", "974")</f>
@@ -2499,13 +2524,13 @@
         <v>11</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="H42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B43" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/continuous-subarray-sum/", "523")</f>
@@ -2525,13 +2550,13 @@
         <v>11</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="H43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B44" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-addition/", "370")</f>
@@ -2551,15 +2576,15 @@
         <v>11</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="H44" s="20" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B45" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/car-pooling/", "1094")</f>
@@ -2579,13 +2604,13 @@
         <v>11</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="H45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B46" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/corporate-flight-bookings/", "1109")</f>
@@ -2605,13 +2630,13 @@
         <v>11</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B47" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/check-if-all-the-integers-in-a-range-are-covered/", "1893")</f>
@@ -2631,13 +2656,13 @@
         <v>11</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B48" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/describe-the-painting/", "1943")</f>
@@ -2657,13 +2682,13 @@
         <v>11</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="H48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B49" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shifting-letters-ii/", "2381")</f>
@@ -2683,13 +2708,13 @@
         <v>11</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="H49" s="17"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B50" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/daily-temperatures/", "739")</f>
@@ -2709,13 +2734,13 @@
         <v>11</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="H50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B51" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-i/", "496")</f>
@@ -2735,13 +2760,13 @@
         <v>11</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="H51" s="17"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B52" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-ii/", "503")</f>
@@ -2761,13 +2786,13 @@
         <v>11</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="H52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B53" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/largest-rectangle-in-histogram/", "84")</f>
@@ -2787,13 +2812,13 @@
         <v>11</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="H53" s="17"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B54" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-rectangle/", "85")</f>
@@ -2813,13 +2838,13 @@
         <v>11</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="H54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B55" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/online-stock-span/", "901")</f>
@@ -2839,13 +2864,13 @@
         <v>11</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="H55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B56" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sliding-window-maximum/", "239")</f>
@@ -2865,13 +2890,13 @@
         <v>11</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B57" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-subarray-with-sum-at-least-k/", "862")</f>
@@ -2891,13 +2916,13 @@
         <v>11</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="H57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B58" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/constrained-subsequence-sum/", "1425")</f>
@@ -2917,13 +2942,13 @@
         <v>11</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="H58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B59" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-continuous-subarray-with-absolute-diff-less-than-or-equal-to-limit/", "1438")</f>
@@ -2943,13 +2968,13 @@
         <v>11</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="H59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B60" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-value-of-equation/", "1499")</f>
@@ -2969,13 +2994,13 @@
         <v>11</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="H60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B61" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-vi/", "1696")</f>
@@ -2995,13 +3020,13 @@
         <v>11</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="H61" s="17"/>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B62" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-an-array/", "215")</f>
@@ -3021,13 +3046,13 @@
         <v>11</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="H62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B63" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -3047,13 +3072,13 @@
         <v>11</v>
       </c>
       <c r="G63" s="16" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="H63" s="17"/>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B64" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-words/", "692")</f>
@@ -3073,13 +3098,13 @@
         <v>11</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="H64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B65" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-a-stream/", "703")</f>
@@ -3099,13 +3124,13 @@
         <v>11</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="H65" s="17"/>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B66" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/k-closest-points-to-origin/", "973")</f>
@@ -3125,13 +3150,13 @@
         <v>11</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="H66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B67" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight/", "1046")</f>
@@ -3151,13 +3176,13 @@
         <v>11</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="H67" s="17"/>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B68" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-intervals/", "56")</f>
@@ -3177,13 +3202,13 @@
         <v>11</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="H68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B69" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/insert-interval/", "57")</f>
@@ -3203,13 +3228,13 @@
         <v>11</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H69" s="17"/>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B70" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms/", "252")</f>
@@ -3229,15 +3254,15 @@
         <v>11</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="H70" s="20" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B71" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms-ii/", "253")</f>
@@ -3257,15 +3282,15 @@
         <v>11</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="H71" s="19" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B72" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/non-overlapping-intervals/", "435")</f>
@@ -3285,13 +3310,13 @@
         <v>11</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="H72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B73" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-arrows-to-burst-balloons/", "452")</f>
@@ -3311,13 +3336,13 @@
         <v>11</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H73" s="17"/>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B74" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-ii/", "45")</f>
@@ -3337,13 +3362,13 @@
         <v>11</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="H74" s="10"/>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="11" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B75" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game/", "55")</f>
@@ -3363,13 +3388,13 @@
         <v>11</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H75" s="17"/>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B76" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/queue-reconstruction-by-height/", "406")</f>
@@ -3389,13 +3414,13 @@
         <v>11</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="H76" s="10"/>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B77" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/task-scheduler/", "621")</f>
@@ -3415,13 +3440,13 @@
         <v>11</v>
       </c>
       <c r="G77" s="16" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="H77" s="17"/>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B78" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-labels/", "763")</f>
@@ -3441,13 +3466,13 @@
         <v>11</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="H78" s="10"/>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B79" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/gas-station/", "134")</f>
@@ -3467,13 +3492,13 @@
         <v>11</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="H79" s="17"/>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B80" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/", "21")</f>
@@ -3493,13 +3518,13 @@
         <v>11</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H80" s="10"/>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B81" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-k-sorted-lists/", "23")</f>
@@ -3519,13 +3544,13 @@
         <v>11</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="H81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B82" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swap-nodes-in-pairs/", "24")</f>
@@ -3545,13 +3570,13 @@
         <v>11</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="H82" s="10"/>
     </row>
     <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B83" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-nodes-in-k-group/", "25")</f>
@@ -3571,13 +3596,13 @@
         <v>11</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="H83" s="17"/>
     </row>
     <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B84" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-linked-list-ii/", "92")</f>
@@ -3597,13 +3622,13 @@
         <v>11</v>
       </c>
       <c r="G84" s="9" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="H84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B85" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/copy-list-with-random-pointer/", "138")</f>
@@ -3623,13 +3648,13 @@
         <v>11</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="H85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B86" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximum-depth-of-binary-tree/", "104")</f>
@@ -3649,13 +3674,13 @@
         <v>11</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="H86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B87" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum/", "112")</f>
@@ -3675,13 +3700,13 @@
         <v>11</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="H87" s="17"/>
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B88" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum-ii/", "113")</f>
@@ -3701,13 +3726,13 @@
         <v>11</v>
       </c>
       <c r="G88" s="9" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="H88" s="10"/>
     </row>
     <row r="89" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B89" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/diameter-of-binary-tree/", "543")</f>
@@ -3727,13 +3752,13 @@
         <v>11</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="H89" s="17"/>
     </row>
     <row r="90" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B90" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-maximum-path-sum/", "124")</f>
@@ -3753,13 +3778,13 @@
         <v>11</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="H90" s="10"/>
     </row>
     <row r="91" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B91" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/invert-binary-tree/", "226")</f>
@@ -3779,13 +3804,13 @@
         <v>11</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="H91" s="17"/>
     </row>
     <row r="92" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B92" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-level-order-traversal/", "102")</f>
@@ -3805,13 +3830,13 @@
         <v>11</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="H92" s="10"/>
     </row>
     <row r="93" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B93" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/", "103")</f>
@@ -3831,13 +3856,13 @@
         <v>11</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="H93" s="17"/>
     </row>
     <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B94" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-right-side-view/", "199")</f>
@@ -3857,13 +3882,13 @@
         <v>11</v>
       </c>
       <c r="G94" s="9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="H94" s="10"/>
     </row>
     <row r="95" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B95" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-largest-value-in-each-tree-row/", "515")</f>
@@ -3883,13 +3908,13 @@
         <v>11</v>
       </c>
       <c r="G95" s="16" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="H95" s="17"/>
     </row>
     <row r="96" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B96" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/average-of-levels-in-binary-tree/", "637")</f>
@@ -3909,13 +3934,13 @@
         <v>11</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="H96" s="10"/>
     </row>
     <row r="97" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="B97" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/populating-next-right-pointers-in-each-node/", "116")</f>
@@ -3935,13 +3960,13 @@
         <v>11</v>
       </c>
       <c r="G97" s="16" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="H97" s="17"/>
     </row>
     <row r="98" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B98" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/validate-binary-search-tree/", "98")</f>
@@ -3961,13 +3986,13 @@
         <v>11</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="H98" s="10"/>
     </row>
     <row r="99" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B99" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/recover-binary-search-tree/", "99")</f>
@@ -3987,13 +4012,13 @@
         <v>11</v>
       </c>
       <c r="G99" s="16" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="H99" s="17"/>
     </row>
     <row r="100" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B100" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-smallest-element-in-a-bst/", "230")</f>
@@ -4013,13 +4038,13 @@
         <v>11</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="H100" s="10"/>
     </row>
     <row r="101" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B101" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/", "235")</f>
@@ -4039,13 +4064,13 @@
         <v>11</v>
       </c>
       <c r="G101" s="16" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="H101" s="17"/>
     </row>
     <row r="102" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B102" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-node-in-a-bst/", "450")</f>
@@ -4065,13 +4090,13 @@
         <v>11</v>
       </c>
       <c r="G102" s="9" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="H102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="B103" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-a-binary-search-tree/", "700")</f>
@@ -4091,13 +4116,13 @@
         <v>11</v>
       </c>
       <c r="G103" s="16" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="H103" s="17"/>
     </row>
     <row r="104" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B104" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations/", "46")</f>
@@ -4117,13 +4142,13 @@
         <v>11</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="H104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B105" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations-ii/", "47")</f>
@@ -4143,13 +4168,13 @@
         <v>11</v>
       </c>
       <c r="G105" s="16" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="H105" s="17"/>
     </row>
     <row r="106" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B106" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combinations/", "77")</f>
@@ -4169,13 +4194,13 @@
         <v>11</v>
       </c>
       <c r="G106" s="9" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="H106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B107" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets/", "78")</f>
@@ -4195,13 +4220,13 @@
         <v>11</v>
       </c>
       <c r="G107" s="16" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="H107" s="17"/>
     </row>
     <row r="108" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B108" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets-ii/", "90")</f>
@@ -4221,13 +4246,13 @@
         <v>11</v>
       </c>
       <c r="G108" s="9" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="H108" s="10"/>
     </row>
     <row r="109" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="11" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="B109" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum/", "39")</f>
@@ -4247,13 +4272,13 @@
         <v>11</v>
       </c>
       <c r="G109" s="16" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="H109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B110" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum-ii/", "40")</f>
@@ -4273,13 +4298,13 @@
         <v>11</v>
       </c>
       <c r="G110" s="9" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="H110" s="10"/>
     </row>
     <row r="111" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B111" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/letter-combinations-of-a-phone-number/", "17")</f>
@@ -4299,13 +4324,13 @@
         <v>11</v>
       </c>
       <c r="G111" s="16" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="H111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B112" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search/", "79")</f>
@@ -4325,13 +4350,13 @@
         <v>11</v>
       </c>
       <c r="G112" s="9" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="H112" s="10"/>
     </row>
     <row r="113" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B113" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/palindrome-partitioning/", "131")</f>
@@ -4351,13 +4376,13 @@
         <v>11</v>
       </c>
       <c r="G113" s="16" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="H113" s="17"/>
     </row>
     <row r="114" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B114" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens/", "51")</f>
@@ -4377,13 +4402,13 @@
         <v>11</v>
       </c>
       <c r="G114" s="9" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="H114" s="10"/>
     </row>
     <row r="115" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="B115" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens-ii/", "52")</f>
@@ -4403,13 +4428,13 @@
         <v>11</v>
       </c>
       <c r="G115" s="16" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="H115" s="17"/>
     </row>
     <row r="116" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B116" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-islands/", "200")</f>
@@ -4429,13 +4454,13 @@
         <v>11</v>
       </c>
       <c r="G116" s="9" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="H116" s="10"/>
     </row>
     <row r="117" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="11" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B117" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-area-of-island/", "695")</f>
@@ -4455,13 +4480,13 @@
         <v>11</v>
       </c>
       <c r="G117" s="16" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="H117" s="17"/>
     </row>
     <row r="118" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B118" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/flood-fill/", "733")</f>
@@ -4481,13 +4506,13 @@
         <v>11</v>
       </c>
       <c r="G118" s="9" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="H118" s="10"/>
     </row>
     <row r="119" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B119" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/rotting-oranges/", "994")</f>
@@ -4507,13 +4532,13 @@
         <v>11</v>
       </c>
       <c r="G119" s="16" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="H119" s="17"/>
     </row>
     <row r="120" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B120" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-path-in-binary-matrix/", "1091")</f>
@@ -4533,13 +4558,13 @@
         <v>11</v>
       </c>
       <c r="G120" s="9" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="H120" s="10"/>
     </row>
     <row r="121" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="11" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="B121" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-closed-islands/", "1254")</f>
@@ -4559,13 +4584,13 @@
         <v>11</v>
       </c>
       <c r="G121" s="16" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="H121" s="17"/>
     </row>
     <row r="122" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B122" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule/", "207")</f>
@@ -4585,13 +4610,13 @@
         <v>11</v>
       </c>
       <c r="G122" s="9" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="H122" s="10"/>
     </row>
     <row r="123" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B123" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-ii/", "210")</f>
@@ -4611,13 +4636,13 @@
         <v>11</v>
       </c>
       <c r="G123" s="16" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="H123" s="17"/>
     </row>
     <row r="124" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B124" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-eventual-safe-states/", "802")</f>
@@ -4637,13 +4662,13 @@
         <v>11</v>
       </c>
       <c r="G124" s="9" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="H124" s="10"/>
     </row>
     <row r="125" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B125" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-iv/", "1462")</f>
@@ -4663,13 +4688,13 @@
         <v>11</v>
       </c>
       <c r="G125" s="16" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="H125" s="17"/>
     </row>
     <row r="126" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B126" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sort-items-by-groups-respecting-dependencies/", "1203")</f>
@@ -4689,13 +4714,13 @@
         <v>11</v>
       </c>
       <c r="G126" s="9" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="H126" s="10"/>
     </row>
     <row r="127" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="11" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B127" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-all-possible-recipes-from-given-supplies/", "2115")</f>
@@ -4715,13 +4740,13 @@
         <v>11</v>
       </c>
       <c r="G127" s="16" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="H127" s="17"/>
     </row>
     <row r="128" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B128" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-provinces/", "547")</f>
@@ -4741,13 +4766,13 @@
         <v>11</v>
       </c>
       <c r="G128" s="9" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="H128" s="10"/>
     </row>
     <row r="129" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="11" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B129" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/redundant-connection/", "684")</f>
@@ -4767,13 +4792,13 @@
         <v>11</v>
       </c>
       <c r="G129" s="16" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="H129" s="17"/>
     </row>
     <row r="130" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B130" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-operations-to-make-network-connected/", "1319")</f>
@@ -4793,13 +4818,13 @@
         <v>11</v>
       </c>
       <c r="G130" s="9" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="H130" s="10"/>
     </row>
     <row r="131" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="11" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B131" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/remove-max-number-of-edges-to-keep-graph-fully-traversable/", "1579")</f>
@@ -4819,13 +4844,13 @@
         <v>11</v>
       </c>
       <c r="G131" s="16" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="H131" s="17"/>
     </row>
     <row r="132" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B132" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/satisfiability-of-equality-equations/", "990")</f>
@@ -4845,13 +4870,13 @@
         <v>11</v>
       </c>
       <c r="G132" s="9" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H132" s="10"/>
     </row>
     <row r="133" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="11" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="B133" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/smallest-string-with-swaps/", "1202")</f>
@@ -4871,13 +4896,13 @@
         <v>11</v>
       </c>
       <c r="G133" s="16" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H133" s="17"/>
     </row>
     <row r="134" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B134" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/network-delay-time/", "743")</f>
@@ -4897,13 +4922,13 @@
         <v>11</v>
       </c>
       <c r="G134" s="9" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="H134" s="10"/>
     </row>
     <row r="135" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="11" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B135" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/cheapest-flights-within-k-stops/", "787")</f>
@@ -4923,13 +4948,13 @@
         <v>11</v>
       </c>
       <c r="G135" s="16" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="H135" s="17"/>
     </row>
     <row r="136" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B136" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-probability/", "1514")</f>
@@ -4949,13 +4974,13 @@
         <v>11</v>
       </c>
       <c r="G136" s="9" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="H136" s="10"/>
     </row>
     <row r="137" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="11" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B137" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-minimum-effort/", "1631")</f>
@@ -4975,13 +5000,13 @@
         <v>11</v>
       </c>
       <c r="G137" s="16" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="H137" s="17"/>
     </row>
     <row r="138" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B138" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/", "1334")</f>
@@ -5001,13 +5026,13 @@
         <v>11</v>
       </c>
       <c r="G138" s="9" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="H138" s="10"/>
     </row>
     <row r="139" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="11" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="B139" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-ways-to-arrive-at-destination/", "1976")</f>
@@ -5027,13 +5052,13 @@
         <v>11</v>
       </c>
       <c r="G139" s="16" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="H139" s="17"/>
     </row>
     <row r="140" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B140" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/min-cost-to-connect-all-points/", "1584")</f>
@@ -5053,13 +5078,13 @@
         <v>11</v>
       </c>
       <c r="G140" s="9" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="H140" s="10"/>
     </row>
     <row r="141" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="11" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B141" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/connecting-cities-with-minimum-cost/", "1135")</f>
@@ -5079,15 +5104,15 @@
         <v>11</v>
       </c>
       <c r="G141" s="16" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="H141" s="19" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B142" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/optimize-water-distribution-in-a-village/", "1168")</f>
@@ -5107,15 +5132,15 @@
         <v>11</v>
       </c>
       <c r="G142" s="9" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="H142" s="20" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="11" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B143" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-critical-and-pseudo-critical-edges-in-minimum-spanning-tree/", "1489")</f>
@@ -5135,13 +5160,13 @@
         <v>11</v>
       </c>
       <c r="G143" s="16" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="H143" s="17"/>
     </row>
     <row r="144" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B144" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swim-in-rising-water/", "778")</f>
@@ -5161,13 +5186,13 @@
         <v>11</v>
       </c>
       <c r="G144" s="9" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="H144" s="10"/>
     </row>
     <row r="145" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="11" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="B145" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-minimum-value/", "1102")</f>
@@ -5187,15 +5212,15 @@
         <v>11</v>
       </c>
       <c r="G145" s="16" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="H145" s="19" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B146" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/implement-trie-prefix-tree/", "208")</f>
@@ -5215,13 +5240,13 @@
         <v>11</v>
       </c>
       <c r="G146" s="9" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="H146" s="10"/>
     </row>
     <row r="147" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="11" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B147" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/design-add-and-search-words-data-structure/", "211")</f>
@@ -5241,13 +5266,13 @@
         <v>11</v>
       </c>
       <c r="G147" s="16" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="H147" s="17"/>
     </row>
     <row r="148" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B148" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search-ii/", "212")</f>
@@ -5267,13 +5292,13 @@
         <v>11</v>
       </c>
       <c r="G148" s="9" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="H148" s="10"/>
     </row>
     <row r="149" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B149" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/replace-words/", "648")</f>
@@ -5293,13 +5318,13 @@
         <v>11</v>
       </c>
       <c r="G149" s="16" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="H149" s="17"/>
     </row>
     <row r="150" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B150" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/map-sum-pairs/", "677")</f>
@@ -5319,13 +5344,13 @@
         <v>11</v>
       </c>
       <c r="G150" s="9" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="H150" s="10"/>
     </row>
     <row r="151" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="11" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="B151" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-suggestions-system/", "1268")</f>
@@ -5345,13 +5370,13 @@
         <v>11</v>
       </c>
       <c r="G151" s="16" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="H151" s="17"/>
     </row>
     <row r="152" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="B152" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number/", "136")</f>
@@ -5371,13 +5396,13 @@
         <v>11</v>
       </c>
       <c r="G152" s="9" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="H152" s="10"/>
     </row>
     <row r="153" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="11" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="B153" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number-ii/", "137")</f>
@@ -5397,13 +5422,13 @@
         <v>11</v>
       </c>
       <c r="G153" s="16" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="H153" s="17"/>
     </row>
     <row r="154" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="B154" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-1-bits/", "191")</f>
@@ -5423,13 +5448,13 @@
         <v>11</v>
       </c>
       <c r="G154" s="9" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="H154" s="10"/>
     </row>
     <row r="155" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="11" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="B155" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/counting-bits/", "338")</f>
@@ -5449,13 +5474,13 @@
         <v>11</v>
       </c>
       <c r="G155" s="16" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="H155" s="17"/>
     </row>
     <row r="156" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="B156" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/missing-number/", "268")</f>
@@ -5475,13 +5500,13 @@
         <v>11</v>
       </c>
       <c r="G156" s="9" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="H156" s="10"/>
     </row>
     <row r="157" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="11" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="B157" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-bits/", "190")</f>
@@ -5501,13 +5526,13 @@
         <v>11</v>
       </c>
       <c r="G157" s="16" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="H157" s="17"/>
     </row>
     <row r="158" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B158" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/climbing-stairs/", "70")</f>
@@ -5527,13 +5552,13 @@
         <v>11</v>
       </c>
       <c r="G158" s="9" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="H158" s="10"/>
     </row>
     <row r="159" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="11" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B159" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber/", "198")</f>
@@ -5553,13 +5578,13 @@
         <v>11</v>
       </c>
       <c r="G159" s="16" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="H159" s="17"/>
     </row>
     <row r="160" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B160" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber-ii/", "213")</f>
@@ -5579,13 +5604,13 @@
         <v>11</v>
       </c>
       <c r="G160" s="9" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="H160" s="10"/>
     </row>
     <row r="161" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="11" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B161" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change/", "322")</f>
@@ -5605,13 +5630,13 @@
         <v>11</v>
       </c>
       <c r="G161" s="16" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="H161" s="17"/>
     </row>
     <row r="162" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B162" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/perfect-squares/", "279")</f>
@@ -5631,13 +5656,13 @@
         <v>11</v>
       </c>
       <c r="G162" s="9" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="H162" s="10"/>
     </row>
     <row r="163" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="11" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="B163" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-increasing-subsequence/", "300")</f>
@@ -5657,13 +5682,13 @@
         <v>11</v>
       </c>
       <c r="G163" s="16" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="H163" s="17"/>
     </row>
     <row r="164" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B164" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-equal-subset-sum/", "416")</f>
@@ -5683,13 +5708,13 @@
         <v>11</v>
       </c>
       <c r="G164" s="9" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="H164" s="10"/>
     </row>
     <row r="165" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="11" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B165" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/target-sum/", "494")</f>
@@ -5709,13 +5734,13 @@
         <v>11</v>
       </c>
       <c r="G165" s="16" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="H165" s="17"/>
     </row>
     <row r="166" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B166" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change-ii/", "518")</f>
@@ -5735,13 +5760,13 @@
         <v>11</v>
       </c>
       <c r="G166" s="9" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="H166" s="10"/>
     </row>
     <row r="167" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="11" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B167" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/ones-and-zeroes/", "474")</f>
@@ -5761,13 +5786,13 @@
         <v>11</v>
       </c>
       <c r="G167" s="16" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="H167" s="17"/>
     </row>
     <row r="168" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="3" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B168" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight-ii/", "1049")</f>
@@ -5787,13 +5812,13 @@
         <v>11</v>
       </c>
       <c r="G168" s="9" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="H168" s="10"/>
     </row>
     <row r="169" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="11" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="B169" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/profitable-schemes/", "879")</f>
@@ -5813,13 +5838,13 @@
         <v>11</v>
       </c>
       <c r="G169" s="16" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="H169" s="17"/>
     </row>
     <row r="170" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B170" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths/", "62")</f>
@@ -5839,13 +5864,13 @@
         <v>11</v>
       </c>
       <c r="G170" s="9" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="H170" s="10"/>
     </row>
     <row r="171" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B171" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths-ii/", "63")</f>
@@ -5865,13 +5890,13 @@
         <v>11</v>
       </c>
       <c r="G171" s="16" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="H171" s="17"/>
     </row>
     <row r="172" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B172" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-path-sum/", "64")</f>
@@ -5891,13 +5916,13 @@
         <v>11</v>
       </c>
       <c r="G172" s="9" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="H172" s="10"/>
     </row>
     <row r="173" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="11" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B173" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-square/", "221")</f>
@@ -5917,13 +5942,13 @@
         <v>11</v>
       </c>
       <c r="G173" s="16" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="H173" s="17"/>
     </row>
     <row r="174" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B174" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-falling-path-sum/", "931")</f>
@@ -5943,13 +5968,13 @@
         <v>11</v>
       </c>
       <c r="G174" s="9" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="H174" s="10"/>
     </row>
     <row r="175" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="11" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B175" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/triangle/", "120")</f>
@@ -5969,13 +5994,13 @@
         <v>11</v>
       </c>
       <c r="G175" s="16" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="H175" s="17"/>
     </row>
     <row r="176" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="3" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B176" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-common-subsequence/", "1143")</f>
@@ -5995,13 +6020,13 @@
         <v>11</v>
       </c>
       <c r="G176" s="9" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="H176" s="10"/>
     </row>
     <row r="177" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="11" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B177" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/edit-distance/", "72")</f>
@@ -6021,13 +6046,13 @@
         <v>11</v>
       </c>
       <c r="G177" s="16" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="H177" s="17"/>
     </row>
     <row r="178" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="3" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B178" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/distinct-subsequences/", "115")</f>
@@ -6047,13 +6072,13 @@
         <v>11</v>
       </c>
       <c r="G178" s="9" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="H178" s="10"/>
     </row>
     <row r="179" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="11" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B179" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-operation-for-two-strings/", "583")</f>
@@ -6073,13 +6098,13 @@
         <v>11</v>
       </c>
       <c r="G179" s="16" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="H179" s="17"/>
     </row>
     <row r="180" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="3" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B180" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/interleaving-string/", "97")</f>
@@ -6099,13 +6124,13 @@
         <v>11</v>
       </c>
       <c r="G180" s="9" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="H180" s="10"/>
     </row>
     <row r="181" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="11" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="B181" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-insertion-steps-to-make-a-string-palindrome/", "1312")</f>
@@ -6125,7 +6150,7 @@
         <v>11</v>
       </c>
       <c r="G181" s="16" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="H181" s="17"/>
     </row>

</xml_diff>

<commit_message>
added notes.md for linked list
</commit_message>
<xml_diff>
--- a/leetcode_roadmap.xlsx
+++ b/leetcode_roadmap.xlsx
@@ -1401,7 +1401,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="12"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="60"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="98.71"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="98.7"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1946,7 +1946,7 @@
       <c r="G20" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H20" s="0" t="s">
+      <c r="H20" s="1" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>

<commit_message>
finished bs problems on sorted data.
</commit_message>
<xml_diff>
--- a/leetcode_roadmap.xlsx
+++ b/leetcode_roadmap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="930" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="239">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -185,6 +185,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/find-minimum-in-rotated-sorted-array/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">same as problem 33 minus the target search. find the pivot using binary search. The pivot is the smallest in the array.</t>
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/find-peak-element/</t>
@@ -746,7 +749,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -829,6 +832,13 @@
       <color rgb="FF166534"/>
       <name val="Calibri"/>
       <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
     <font>
@@ -938,7 +948,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1015,11 +1025,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1946,7 +1960,7 @@
       <c r="G20" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="H20" s="1" t="s">
+      <c r="H20" s="19" t="s">
         <v>48</v>
       </c>
     </row>
@@ -2021,8 +2035,8 @@
       <c r="D23" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E23" s="15" t="s">
-        <v>11</v>
+      <c r="E23" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F23" s="15" t="s">
         <v>11</v>
@@ -2030,7 +2044,9 @@
       <c r="G23" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="H23" s="17"/>
+      <c r="H23" s="17" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
@@ -2054,7 +2070,7 @@
         <v>11</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H24" s="10"/>
     </row>
@@ -2080,13 +2096,13 @@
         <v>11</v>
       </c>
       <c r="G25" s="16" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="H25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B26" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/koko-eating-bananas/", "875")</f>
@@ -2106,13 +2122,13 @@
         <v>11</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H26" s="10"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B27" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/capacity-to-ship-packages-within-d-days/", "1011")</f>
@@ -2132,13 +2148,13 @@
         <v>11</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H27" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B28" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/split-array-largest-sum/", "410")</f>
@@ -2158,13 +2174,13 @@
         <v>11</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H28" s="10"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B29" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimize-max-distance-to-gas-station/", "774")</f>
@@ -2184,15 +2200,15 @@
         <v>11</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>60</v>
-      </c>
-      <c r="H29" s="19" t="s">
         <v>61</v>
+      </c>
+      <c r="H29" s="20" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B30" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-smallest-divisor-given-a-threshold/", "1283")</f>
@@ -2212,13 +2228,13 @@
         <v>11</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="H30" s="10"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B31" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-days-to-make-m-bouquets/", "1482")</f>
@@ -2238,13 +2254,13 @@
         <v>11</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="H31" s="17"/>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B32" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/two-sum/", "1")</f>
@@ -2264,13 +2280,13 @@
         <v>11</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="H32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B33" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/group-anagrams/", "49")</f>
@@ -2290,13 +2306,13 @@
         <v>11</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="H33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B34" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-consecutive-sequence/", "128")</f>
@@ -2316,13 +2332,13 @@
         <v>11</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B35" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/contains-duplicate/", "217")</f>
@@ -2342,13 +2358,13 @@
         <v>11</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="H35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B36" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/valid-anagram/", "242")</f>
@@ -2368,13 +2384,13 @@
         <v>11</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="H36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B37" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -2394,13 +2410,13 @@
         <v>11</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B38" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-sum-query-immutable/", "303")</f>
@@ -2420,13 +2436,13 @@
         <v>11</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="H38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B39" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sum-equals-k/", "560")</f>
@@ -2446,13 +2462,13 @@
         <v>11</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B40" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-pivot-index/", "724")</f>
@@ -2472,13 +2488,13 @@
         <v>11</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="H40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B41" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-subarrays-with-sum/", "930")</f>
@@ -2498,13 +2514,13 @@
         <v>11</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H41" s="17"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B42" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sums-divisible-by-k/", "974")</f>
@@ -2524,13 +2540,13 @@
         <v>11</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B43" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/continuous-subarray-sum/", "523")</f>
@@ -2550,13 +2566,13 @@
         <v>11</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="H43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B44" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-addition/", "370")</f>
@@ -2576,15 +2592,15 @@
         <v>11</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="H44" s="20" t="s">
-        <v>61</v>
+        <v>80</v>
+      </c>
+      <c r="H44" s="21" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B45" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/car-pooling/", "1094")</f>
@@ -2604,13 +2620,13 @@
         <v>11</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="H45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B46" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/corporate-flight-bookings/", "1109")</f>
@@ -2630,13 +2646,13 @@
         <v>11</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B47" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/check-if-all-the-integers-in-a-range-are-covered/", "1893")</f>
@@ -2656,13 +2672,13 @@
         <v>11</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B48" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/describe-the-painting/", "1943")</f>
@@ -2682,13 +2698,13 @@
         <v>11</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B49" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shifting-letters-ii/", "2381")</f>
@@ -2708,13 +2724,13 @@
         <v>11</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H49" s="17"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B50" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/daily-temperatures/", "739")</f>
@@ -2734,13 +2750,13 @@
         <v>11</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B51" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-i/", "496")</f>
@@ -2760,13 +2776,13 @@
         <v>11</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="H51" s="17"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B52" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-ii/", "503")</f>
@@ -2786,13 +2802,13 @@
         <v>11</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B53" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/largest-rectangle-in-histogram/", "84")</f>
@@ -2812,13 +2828,13 @@
         <v>11</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="H53" s="17"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B54" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-rectangle/", "85")</f>
@@ -2838,13 +2854,13 @@
         <v>11</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="H54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B55" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/online-stock-span/", "901")</f>
@@ -2864,13 +2880,13 @@
         <v>11</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B56" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sliding-window-maximum/", "239")</f>
@@ -2890,13 +2906,13 @@
         <v>11</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="H56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B57" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-subarray-with-sum-at-least-k/", "862")</f>
@@ -2916,13 +2932,13 @@
         <v>11</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B58" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/constrained-subsequence-sum/", "1425")</f>
@@ -2942,13 +2958,13 @@
         <v>11</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="H58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B59" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-continuous-subarray-with-absolute-diff-less-than-or-equal-to-limit/", "1438")</f>
@@ -2968,13 +2984,13 @@
         <v>11</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B60" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-value-of-equation/", "1499")</f>
@@ -2994,13 +3010,13 @@
         <v>11</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B61" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-vi/", "1696")</f>
@@ -3020,13 +3036,13 @@
         <v>11</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H61" s="17"/>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B62" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-an-array/", "215")</f>
@@ -3046,13 +3062,13 @@
         <v>11</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B63" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -3072,13 +3088,13 @@
         <v>11</v>
       </c>
       <c r="G63" s="16" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="H63" s="17"/>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B64" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-words/", "692")</f>
@@ -3098,13 +3114,13 @@
         <v>11</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="H64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B65" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-a-stream/", "703")</f>
@@ -3124,13 +3140,13 @@
         <v>11</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="H65" s="17"/>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B66" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/k-closest-points-to-origin/", "973")</f>
@@ -3150,13 +3166,13 @@
         <v>11</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B67" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight/", "1046")</f>
@@ -3176,13 +3192,13 @@
         <v>11</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H67" s="17"/>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B68" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-intervals/", "56")</f>
@@ -3202,13 +3218,13 @@
         <v>11</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="H68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B69" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/insert-interval/", "57")</f>
@@ -3228,13 +3244,13 @@
         <v>11</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H69" s="17"/>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B70" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms/", "252")</f>
@@ -3254,15 +3270,15 @@
         <v>11</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>108</v>
-      </c>
-      <c r="H70" s="20" t="s">
-        <v>61</v>
+        <v>109</v>
+      </c>
+      <c r="H70" s="21" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B71" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms-ii/", "253")</f>
@@ -3282,15 +3298,15 @@
         <v>11</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>109</v>
-      </c>
-      <c r="H71" s="19" t="s">
-        <v>61</v>
+        <v>110</v>
+      </c>
+      <c r="H71" s="20" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B72" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/non-overlapping-intervals/", "435")</f>
@@ -3310,13 +3326,13 @@
         <v>11</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="H72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B73" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-arrows-to-burst-balloons/", "452")</f>
@@ -3336,13 +3352,13 @@
         <v>11</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H73" s="17"/>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B74" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-ii/", "45")</f>
@@ -3362,13 +3378,13 @@
         <v>11</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H74" s="10"/>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B75" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game/", "55")</f>
@@ -3388,13 +3404,13 @@
         <v>11</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="H75" s="17"/>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B76" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/queue-reconstruction-by-height/", "406")</f>
@@ -3414,13 +3430,13 @@
         <v>11</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="H76" s="10"/>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B77" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/task-scheduler/", "621")</f>
@@ -3440,13 +3456,13 @@
         <v>11</v>
       </c>
       <c r="G77" s="16" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H77" s="17"/>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B78" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-labels/", "763")</f>
@@ -3466,13 +3482,13 @@
         <v>11</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H78" s="10"/>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B79" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/gas-station/", "134")</f>
@@ -3492,13 +3508,13 @@
         <v>11</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="H79" s="17"/>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B80" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/", "21")</f>
@@ -3518,13 +3534,13 @@
         <v>11</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="H80" s="10"/>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B81" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-k-sorted-lists/", "23")</f>
@@ -3544,13 +3560,13 @@
         <v>11</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B82" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swap-nodes-in-pairs/", "24")</f>
@@ -3570,13 +3586,13 @@
         <v>11</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="H82" s="10"/>
     </row>
     <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B83" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-nodes-in-k-group/", "25")</f>
@@ -3596,13 +3612,13 @@
         <v>11</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="H83" s="17"/>
     </row>
     <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B84" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-linked-list-ii/", "92")</f>
@@ -3622,13 +3638,13 @@
         <v>11</v>
       </c>
       <c r="G84" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B85" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/copy-list-with-random-pointer/", "138")</f>
@@ -3648,13 +3664,13 @@
         <v>11</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="H85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B86" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximum-depth-of-binary-tree/", "104")</f>
@@ -3674,13 +3690,13 @@
         <v>11</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="H86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B87" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum/", "112")</f>
@@ -3700,13 +3716,13 @@
         <v>11</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H87" s="17"/>
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B88" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum-ii/", "113")</f>
@@ -3726,13 +3742,13 @@
         <v>11</v>
       </c>
       <c r="G88" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="H88" s="10"/>
     </row>
     <row r="89" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B89" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/diameter-of-binary-tree/", "543")</f>
@@ -3752,13 +3768,13 @@
         <v>11</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H89" s="17"/>
     </row>
     <row r="90" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B90" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-maximum-path-sum/", "124")</f>
@@ -3778,13 +3794,13 @@
         <v>11</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="H90" s="10"/>
     </row>
     <row r="91" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B91" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/invert-binary-tree/", "226")</f>
@@ -3804,13 +3820,13 @@
         <v>11</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H91" s="17"/>
     </row>
     <row r="92" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B92" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-level-order-traversal/", "102")</f>
@@ -3830,13 +3846,13 @@
         <v>11</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="H92" s="10"/>
     </row>
     <row r="93" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B93" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/", "103")</f>
@@ -3856,13 +3872,13 @@
         <v>11</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="H93" s="17"/>
     </row>
     <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B94" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-right-side-view/", "199")</f>
@@ -3882,13 +3898,13 @@
         <v>11</v>
       </c>
       <c r="G94" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="H94" s="10"/>
     </row>
     <row r="95" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B95" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-largest-value-in-each-tree-row/", "515")</f>
@@ -3908,13 +3924,13 @@
         <v>11</v>
       </c>
       <c r="G95" s="16" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H95" s="17"/>
     </row>
     <row r="96" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B96" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/average-of-levels-in-binary-tree/", "637")</f>
@@ -3934,13 +3950,13 @@
         <v>11</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H96" s="10"/>
     </row>
     <row r="97" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B97" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/populating-next-right-pointers-in-each-node/", "116")</f>
@@ -3960,13 +3976,13 @@
         <v>11</v>
       </c>
       <c r="G97" s="16" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="H97" s="17"/>
     </row>
     <row r="98" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B98" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/validate-binary-search-tree/", "98")</f>
@@ -3986,13 +4002,13 @@
         <v>11</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="H98" s="10"/>
     </row>
     <row r="99" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B99" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/recover-binary-search-tree/", "99")</f>
@@ -4012,13 +4028,13 @@
         <v>11</v>
       </c>
       <c r="G99" s="16" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="H99" s="17"/>
     </row>
     <row r="100" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B100" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-smallest-element-in-a-bst/", "230")</f>
@@ -4038,13 +4054,13 @@
         <v>11</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="H100" s="10"/>
     </row>
     <row r="101" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B101" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/", "235")</f>
@@ -4064,13 +4080,13 @@
         <v>11</v>
       </c>
       <c r="G101" s="16" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H101" s="17"/>
     </row>
     <row r="102" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B102" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-node-in-a-bst/", "450")</f>
@@ -4090,13 +4106,13 @@
         <v>11</v>
       </c>
       <c r="G102" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="H102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="B103" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-a-binary-search-tree/", "700")</f>
@@ -4116,13 +4132,13 @@
         <v>11</v>
       </c>
       <c r="G103" s="16" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H103" s="17"/>
     </row>
     <row r="104" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B104" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations/", "46")</f>
@@ -4142,13 +4158,13 @@
         <v>11</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B105" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations-ii/", "47")</f>
@@ -4168,13 +4184,13 @@
         <v>11</v>
       </c>
       <c r="G105" s="16" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H105" s="17"/>
     </row>
     <row r="106" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B106" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combinations/", "77")</f>
@@ -4194,13 +4210,13 @@
         <v>11</v>
       </c>
       <c r="G106" s="9" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="H106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B107" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets/", "78")</f>
@@ -4220,13 +4236,13 @@
         <v>11</v>
       </c>
       <c r="G107" s="16" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="H107" s="17"/>
     </row>
     <row r="108" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B108" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets-ii/", "90")</f>
@@ -4246,13 +4262,13 @@
         <v>11</v>
       </c>
       <c r="G108" s="9" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="H108" s="10"/>
     </row>
     <row r="109" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="11" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B109" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum/", "39")</f>
@@ -4272,13 +4288,13 @@
         <v>11</v>
       </c>
       <c r="G109" s="16" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="H109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B110" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum-ii/", "40")</f>
@@ -4298,13 +4314,13 @@
         <v>11</v>
       </c>
       <c r="G110" s="9" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="H110" s="10"/>
     </row>
     <row r="111" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B111" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/letter-combinations-of-a-phone-number/", "17")</f>
@@ -4324,13 +4340,13 @@
         <v>11</v>
       </c>
       <c r="G111" s="16" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="H111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B112" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search/", "79")</f>
@@ -4350,13 +4366,13 @@
         <v>11</v>
       </c>
       <c r="G112" s="9" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="H112" s="10"/>
     </row>
     <row r="113" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B113" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/palindrome-partitioning/", "131")</f>
@@ -4376,13 +4392,13 @@
         <v>11</v>
       </c>
       <c r="G113" s="16" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="H113" s="17"/>
     </row>
     <row r="114" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B114" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens/", "51")</f>
@@ -4402,13 +4418,13 @@
         <v>11</v>
       </c>
       <c r="G114" s="9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="H114" s="10"/>
     </row>
     <row r="115" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B115" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens-ii/", "52")</f>
@@ -4428,13 +4444,13 @@
         <v>11</v>
       </c>
       <c r="G115" s="16" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H115" s="17"/>
     </row>
     <row r="116" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B116" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-islands/", "200")</f>
@@ -4454,13 +4470,13 @@
         <v>11</v>
       </c>
       <c r="G116" s="9" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="H116" s="10"/>
     </row>
     <row r="117" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B117" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-area-of-island/", "695")</f>
@@ -4480,13 +4496,13 @@
         <v>11</v>
       </c>
       <c r="G117" s="16" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="H117" s="17"/>
     </row>
     <row r="118" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B118" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/flood-fill/", "733")</f>
@@ -4506,13 +4522,13 @@
         <v>11</v>
       </c>
       <c r="G118" s="9" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="H118" s="10"/>
     </row>
     <row r="119" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B119" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/rotting-oranges/", "994")</f>
@@ -4532,13 +4548,13 @@
         <v>11</v>
       </c>
       <c r="G119" s="16" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H119" s="17"/>
     </row>
     <row r="120" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B120" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-path-in-binary-matrix/", "1091")</f>
@@ -4558,13 +4574,13 @@
         <v>11</v>
       </c>
       <c r="G120" s="9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="H120" s="10"/>
     </row>
     <row r="121" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="11" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B121" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-closed-islands/", "1254")</f>
@@ -4584,13 +4600,13 @@
         <v>11</v>
       </c>
       <c r="G121" s="16" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="H121" s="17"/>
     </row>
     <row r="122" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B122" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule/", "207")</f>
@@ -4610,13 +4626,13 @@
         <v>11</v>
       </c>
       <c r="G122" s="9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H122" s="10"/>
     </row>
     <row r="123" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B123" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-ii/", "210")</f>
@@ -4636,13 +4652,13 @@
         <v>11</v>
       </c>
       <c r="G123" s="16" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H123" s="17"/>
     </row>
     <row r="124" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B124" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-eventual-safe-states/", "802")</f>
@@ -4662,13 +4678,13 @@
         <v>11</v>
       </c>
       <c r="G124" s="9" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="H124" s="10"/>
     </row>
     <row r="125" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B125" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-iv/", "1462")</f>
@@ -4688,13 +4704,13 @@
         <v>11</v>
       </c>
       <c r="G125" s="16" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="H125" s="17"/>
     </row>
     <row r="126" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B126" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sort-items-by-groups-respecting-dependencies/", "1203")</f>
@@ -4714,13 +4730,13 @@
         <v>11</v>
       </c>
       <c r="G126" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="H126" s="10"/>
     </row>
     <row r="127" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="11" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B127" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-all-possible-recipes-from-given-supplies/", "2115")</f>
@@ -4740,13 +4756,13 @@
         <v>11</v>
       </c>
       <c r="G127" s="16" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="H127" s="17"/>
     </row>
     <row r="128" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B128" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-provinces/", "547")</f>
@@ -4766,13 +4782,13 @@
         <v>11</v>
       </c>
       <c r="G128" s="9" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H128" s="10"/>
     </row>
     <row r="129" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B129" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/redundant-connection/", "684")</f>
@@ -4792,13 +4808,13 @@
         <v>11</v>
       </c>
       <c r="G129" s="16" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="H129" s="17"/>
     </row>
     <row r="130" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B130" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-operations-to-make-network-connected/", "1319")</f>
@@ -4818,13 +4834,13 @@
         <v>11</v>
       </c>
       <c r="G130" s="9" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="H130" s="10"/>
     </row>
     <row r="131" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B131" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/remove-max-number-of-edges-to-keep-graph-fully-traversable/", "1579")</f>
@@ -4844,13 +4860,13 @@
         <v>11</v>
       </c>
       <c r="G131" s="16" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="H131" s="17"/>
     </row>
     <row r="132" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B132" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/satisfiability-of-equality-equations/", "990")</f>
@@ -4870,13 +4886,13 @@
         <v>11</v>
       </c>
       <c r="G132" s="9" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="H132" s="10"/>
     </row>
     <row r="133" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="11" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="B133" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/smallest-string-with-swaps/", "1202")</f>
@@ -4896,13 +4912,13 @@
         <v>11</v>
       </c>
       <c r="G133" s="16" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="H133" s="17"/>
     </row>
     <row r="134" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B134" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/network-delay-time/", "743")</f>
@@ -4922,13 +4938,13 @@
         <v>11</v>
       </c>
       <c r="G134" s="9" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H134" s="10"/>
     </row>
     <row r="135" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B135" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/cheapest-flights-within-k-stops/", "787")</f>
@@ -4948,13 +4964,13 @@
         <v>11</v>
       </c>
       <c r="G135" s="16" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="H135" s="17"/>
     </row>
     <row r="136" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B136" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-probability/", "1514")</f>
@@ -4974,13 +4990,13 @@
         <v>11</v>
       </c>
       <c r="G136" s="9" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="H136" s="10"/>
     </row>
     <row r="137" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B137" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-minimum-effort/", "1631")</f>
@@ -5000,13 +5016,13 @@
         <v>11</v>
       </c>
       <c r="G137" s="16" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="H137" s="17"/>
     </row>
     <row r="138" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B138" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/", "1334")</f>
@@ -5026,13 +5042,13 @@
         <v>11</v>
       </c>
       <c r="G138" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H138" s="10"/>
     </row>
     <row r="139" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="11" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B139" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-ways-to-arrive-at-destination/", "1976")</f>
@@ -5052,13 +5068,13 @@
         <v>11</v>
       </c>
       <c r="G139" s="16" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="H139" s="17"/>
     </row>
     <row r="140" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B140" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/min-cost-to-connect-all-points/", "1584")</f>
@@ -5078,13 +5094,13 @@
         <v>11</v>
       </c>
       <c r="G140" s="9" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="H140" s="10"/>
     </row>
     <row r="141" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B141" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/connecting-cities-with-minimum-cost/", "1135")</f>
@@ -5104,15 +5120,15 @@
         <v>11</v>
       </c>
       <c r="G141" s="16" t="s">
-        <v>191</v>
-      </c>
-      <c r="H141" s="19" t="s">
-        <v>61</v>
+        <v>192</v>
+      </c>
+      <c r="H141" s="20" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B142" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/optimize-water-distribution-in-a-village/", "1168")</f>
@@ -5132,15 +5148,15 @@
         <v>11</v>
       </c>
       <c r="G142" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="H142" s="20" t="s">
-        <v>61</v>
+        <v>193</v>
+      </c>
+      <c r="H142" s="21" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B143" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-critical-and-pseudo-critical-edges-in-minimum-spanning-tree/", "1489")</f>
@@ -5160,13 +5176,13 @@
         <v>11</v>
       </c>
       <c r="G143" s="16" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H143" s="17"/>
     </row>
     <row r="144" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B144" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swim-in-rising-water/", "778")</f>
@@ -5186,13 +5202,13 @@
         <v>11</v>
       </c>
       <c r="G144" s="9" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="H144" s="10"/>
     </row>
     <row r="145" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="11" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="B145" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-minimum-value/", "1102")</f>
@@ -5212,15 +5228,15 @@
         <v>11</v>
       </c>
       <c r="G145" s="16" t="s">
-        <v>195</v>
-      </c>
-      <c r="H145" s="19" t="s">
-        <v>61</v>
+        <v>196</v>
+      </c>
+      <c r="H145" s="20" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B146" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/implement-trie-prefix-tree/", "208")</f>
@@ -5240,13 +5256,13 @@
         <v>11</v>
       </c>
       <c r="G146" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H146" s="10"/>
     </row>
     <row r="147" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B147" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/design-add-and-search-words-data-structure/", "211")</f>
@@ -5266,13 +5282,13 @@
         <v>11</v>
       </c>
       <c r="G147" s="16" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="H147" s="17"/>
     </row>
     <row r="148" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B148" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search-ii/", "212")</f>
@@ -5292,13 +5308,13 @@
         <v>11</v>
       </c>
       <c r="G148" s="9" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="H148" s="10"/>
     </row>
     <row r="149" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B149" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/replace-words/", "648")</f>
@@ -5318,13 +5334,13 @@
         <v>11</v>
       </c>
       <c r="G149" s="16" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H149" s="17"/>
     </row>
     <row r="150" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B150" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/map-sum-pairs/", "677")</f>
@@ -5344,13 +5360,13 @@
         <v>11</v>
       </c>
       <c r="G150" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="H150" s="10"/>
     </row>
     <row r="151" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="11" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B151" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-suggestions-system/", "1268")</f>
@@ -5370,13 +5386,13 @@
         <v>11</v>
       </c>
       <c r="G151" s="16" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="H151" s="17"/>
     </row>
     <row r="152" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B152" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number/", "136")</f>
@@ -5396,13 +5412,13 @@
         <v>11</v>
       </c>
       <c r="G152" s="9" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="H152" s="10"/>
     </row>
     <row r="153" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B153" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number-ii/", "137")</f>
@@ -5422,13 +5438,13 @@
         <v>11</v>
       </c>
       <c r="G153" s="16" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H153" s="17"/>
     </row>
     <row r="154" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B154" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-1-bits/", "191")</f>
@@ -5448,13 +5464,13 @@
         <v>11</v>
       </c>
       <c r="G154" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="H154" s="10"/>
     </row>
     <row r="155" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B155" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/counting-bits/", "338")</f>
@@ -5474,13 +5490,13 @@
         <v>11</v>
       </c>
       <c r="G155" s="16" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="H155" s="17"/>
     </row>
     <row r="156" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B156" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/missing-number/", "268")</f>
@@ -5500,13 +5516,13 @@
         <v>11</v>
       </c>
       <c r="G156" s="9" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H156" s="10"/>
     </row>
     <row r="157" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="11" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B157" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-bits/", "190")</f>
@@ -5526,13 +5542,13 @@
         <v>11</v>
       </c>
       <c r="G157" s="16" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="H157" s="17"/>
     </row>
     <row r="158" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B158" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/climbing-stairs/", "70")</f>
@@ -5552,13 +5568,13 @@
         <v>11</v>
       </c>
       <c r="G158" s="9" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="H158" s="10"/>
     </row>
     <row r="159" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B159" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber/", "198")</f>
@@ -5578,13 +5594,13 @@
         <v>11</v>
       </c>
       <c r="G159" s="16" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="H159" s="17"/>
     </row>
     <row r="160" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B160" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber-ii/", "213")</f>
@@ -5604,13 +5620,13 @@
         <v>11</v>
       </c>
       <c r="G160" s="9" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="H160" s="10"/>
     </row>
     <row r="161" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B161" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change/", "322")</f>
@@ -5630,13 +5646,13 @@
         <v>11</v>
       </c>
       <c r="G161" s="16" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H161" s="17"/>
     </row>
     <row r="162" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B162" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/perfect-squares/", "279")</f>
@@ -5656,13 +5672,13 @@
         <v>11</v>
       </c>
       <c r="G162" s="9" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="H162" s="10"/>
     </row>
     <row r="163" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="11" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="B163" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-increasing-subsequence/", "300")</f>
@@ -5682,13 +5698,13 @@
         <v>11</v>
       </c>
       <c r="G163" s="16" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="H163" s="17"/>
     </row>
     <row r="164" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B164" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-equal-subset-sum/", "416")</f>
@@ -5708,13 +5724,13 @@
         <v>11</v>
       </c>
       <c r="G164" s="9" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="H164" s="10"/>
     </row>
     <row r="165" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B165" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/target-sum/", "494")</f>
@@ -5734,13 +5750,13 @@
         <v>11</v>
       </c>
       <c r="G165" s="16" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H165" s="17"/>
     </row>
     <row r="166" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B166" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change-ii/", "518")</f>
@@ -5760,13 +5776,13 @@
         <v>11</v>
       </c>
       <c r="G166" s="9" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="H166" s="10"/>
     </row>
     <row r="167" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B167" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/ones-and-zeroes/", "474")</f>
@@ -5786,13 +5802,13 @@
         <v>11</v>
       </c>
       <c r="G167" s="16" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="H167" s="17"/>
     </row>
     <row r="168" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="3" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B168" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight-ii/", "1049")</f>
@@ -5812,13 +5828,13 @@
         <v>11</v>
       </c>
       <c r="G168" s="9" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="H168" s="10"/>
     </row>
     <row r="169" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="11" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B169" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/profitable-schemes/", "879")</f>
@@ -5838,13 +5854,13 @@
         <v>11</v>
       </c>
       <c r="G169" s="16" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="H169" s="17"/>
     </row>
     <row r="170" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B170" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths/", "62")</f>
@@ -5864,13 +5880,13 @@
         <v>11</v>
       </c>
       <c r="G170" s="9" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="H170" s="10"/>
     </row>
     <row r="171" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B171" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths-ii/", "63")</f>
@@ -5890,13 +5906,13 @@
         <v>11</v>
       </c>
       <c r="G171" s="16" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="H171" s="17"/>
     </row>
     <row r="172" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B172" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-path-sum/", "64")</f>
@@ -5916,13 +5932,13 @@
         <v>11</v>
       </c>
       <c r="G172" s="9" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="H172" s="10"/>
     </row>
     <row r="173" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B173" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-square/", "221")</f>
@@ -5942,13 +5958,13 @@
         <v>11</v>
       </c>
       <c r="G173" s="16" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="H173" s="17"/>
     </row>
     <row r="174" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B174" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-falling-path-sum/", "931")</f>
@@ -5968,13 +5984,13 @@
         <v>11</v>
       </c>
       <c r="G174" s="9" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H174" s="10"/>
     </row>
     <row r="175" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="11" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="B175" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/triangle/", "120")</f>
@@ -5994,13 +6010,13 @@
         <v>11</v>
       </c>
       <c r="G175" s="16" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="H175" s="17"/>
     </row>
     <row r="176" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B176" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-common-subsequence/", "1143")</f>
@@ -6020,13 +6036,13 @@
         <v>11</v>
       </c>
       <c r="G176" s="9" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="H176" s="10"/>
     </row>
     <row r="177" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B177" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/edit-distance/", "72")</f>
@@ -6046,13 +6062,13 @@
         <v>11</v>
       </c>
       <c r="G177" s="16" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="H177" s="17"/>
     </row>
     <row r="178" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B178" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/distinct-subsequences/", "115")</f>
@@ -6072,13 +6088,13 @@
         <v>11</v>
       </c>
       <c r="G178" s="9" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H178" s="10"/>
     </row>
     <row r="179" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B179" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-operation-for-two-strings/", "583")</f>
@@ -6098,13 +6114,13 @@
         <v>11</v>
       </c>
       <c r="G179" s="16" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="H179" s="17"/>
     </row>
     <row r="180" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="3" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B180" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/interleaving-string/", "97")</f>
@@ -6124,13 +6140,13 @@
         <v>11</v>
       </c>
       <c r="G180" s="9" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="H180" s="10"/>
     </row>
     <row r="181" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="11" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="B181" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-insertion-steps-to-make-a-string-palindrome/", "1312")</f>
@@ -6150,7 +6166,7 @@
         <v>11</v>
       </c>
       <c r="G181" s="16" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="H181" s="17"/>
     </row>

</xml_diff>

<commit_message>
finished more binary search problems. updated spreadsheet.
</commit_message>
<xml_diff>
--- a/leetcode_roadmap.xlsx
+++ b/leetcode_roadmap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="931" uniqueCount="239">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="243">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -202,70 +202,82 @@
     <t xml:space="preserve">https://leetcode.com/problems/koko-eating-bananas/</t>
   </si>
   <si>
+    <t xml:space="preserve">apply binary search on the [min,max]  range of the input array and not the input array itself</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/capacity-to-ship-packages-within-d-days/</t>
   </si>
   <si>
+    <t xml:space="preserve">same as above problem. [max] is going to be the sum of all weights.</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/split-array-largest-sum/</t>
   </si>
   <si>
+    <t xml:space="preserve">similar to above. Creating “k” subarrays such that the values in them is less than or equal to “mid”.</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/minimize-max-distance-to-gas-station/</t>
   </si>
   <si>
+    <t xml:space="preserve">again, try finding the [min,max] range. Tricky part is to not cause decimal overflow (can lead to TLE). Avoid by checking (high – low) &gt; 1e-x (where x is the lower limit).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/find-the-smallest-divisor-given-a-threshold/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/minimum-number-of-days-to-make-m-bouquets/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hashing / Frequency Maps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/two-sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/group-anagrams/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/longest-consecutive-sequence/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/contains-duplicate/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/valid-anagram/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/top-k-frequent-elements/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prefix Sum / Running Sum</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/range-sum-query-immutable/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/subarray-sum-equals-k/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/find-pivot-index/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/binary-subarrays-with-sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/subarray-sums-divisible-by-k/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/continuous-subarray-sum/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difference Array / Range Updates</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://leetcode.com/problems/range-addition/</t>
+  </si>
+  <si>
     <t xml:space="preserve">Premium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/find-the-smallest-divisor-given-a-threshold/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/minimum-number-of-days-to-make-m-bouquets/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hashing / Frequency Maps</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/two-sum/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/group-anagrams/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/longest-consecutive-sequence/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/contains-duplicate/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/valid-anagram/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/top-k-frequent-elements/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prefix Sum / Running Sum</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/range-sum-query-immutable/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/subarray-sum-equals-k/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/find-pivot-index/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/binary-subarrays-with-sum/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/subarray-sums-divisible-by-k/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/continuous-subarray-sum/</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Difference Array / Range Updates</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://leetcode.com/problems/range-addition/</t>
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/car-pooling/</t>
@@ -1029,11 +1041,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="13" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2115,8 +2127,8 @@
       <c r="D26" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E26" s="8" t="s">
-        <v>11</v>
+      <c r="E26" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F26" s="8" t="s">
         <v>11</v>
@@ -2124,7 +2136,9 @@
       <c r="G26" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="H26" s="10"/>
+      <c r="H26" s="10" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
@@ -2141,16 +2155,18 @@
       <c r="D27" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E27" s="15" t="s">
-        <v>11</v>
+      <c r="E27" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F27" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G27" s="16" t="s">
-        <v>59</v>
-      </c>
-      <c r="H27" s="17"/>
+        <v>60</v>
+      </c>
+      <c r="H27" s="17" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
@@ -2167,16 +2183,18 @@
       <c r="D28" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="E28" s="8" t="s">
-        <v>11</v>
+      <c r="E28" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F28" s="8" t="s">
         <v>11</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="H28" s="10"/>
+        <v>62</v>
+      </c>
+      <c r="H28" s="10" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="11" t="s">
@@ -2193,17 +2211,17 @@
       <c r="D29" s="14" t="s">
         <v>14</v>
       </c>
-      <c r="E29" s="15" t="s">
-        <v>11</v>
+      <c r="E29" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F29" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G29" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="H29" s="20" t="s">
-        <v>62</v>
+        <v>64</v>
+      </c>
+      <c r="H29" s="17" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2228,7 +2246,7 @@
         <v>11</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H30" s="10"/>
     </row>
@@ -2254,13 +2272,13 @@
         <v>11</v>
       </c>
       <c r="G31" s="16" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H31" s="17"/>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B32" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/two-sum/", "1")</f>
@@ -2280,13 +2298,13 @@
         <v>11</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="H32" s="10"/>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B33" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/group-anagrams/", "49")</f>
@@ -2306,13 +2324,13 @@
         <v>11</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H33" s="17"/>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B34" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-consecutive-sequence/", "128")</f>
@@ -2332,13 +2350,13 @@
         <v>11</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H34" s="10"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B35" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/contains-duplicate/", "217")</f>
@@ -2358,13 +2376,13 @@
         <v>11</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="H35" s="17"/>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B36" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/valid-anagram/", "242")</f>
@@ -2384,13 +2402,13 @@
         <v>11</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="H36" s="10"/>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="B37" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -2410,13 +2428,13 @@
         <v>11</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H37" s="17"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B38" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-sum-query-immutable/", "303")</f>
@@ -2436,13 +2454,13 @@
         <v>11</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="H38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B39" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sum-equals-k/", "560")</f>
@@ -2462,13 +2480,13 @@
         <v>11</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="H39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B40" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-pivot-index/", "724")</f>
@@ -2488,13 +2506,13 @@
         <v>11</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="H40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B41" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-subarrays-with-sum/", "930")</f>
@@ -2514,13 +2532,13 @@
         <v>11</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H41" s="17"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B42" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sums-divisible-by-k/", "974")</f>
@@ -2540,13 +2558,13 @@
         <v>11</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="H42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B43" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/continuous-subarray-sum/", "523")</f>
@@ -2566,13 +2584,13 @@
         <v>11</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="H43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B44" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-addition/", "370")</f>
@@ -2592,15 +2610,15 @@
         <v>11</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="H44" s="21" t="s">
-        <v>62</v>
+        <v>83</v>
+      </c>
+      <c r="H44" s="20" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B45" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/car-pooling/", "1094")</f>
@@ -2620,13 +2638,13 @@
         <v>11</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="H45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B46" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/corporate-flight-bookings/", "1109")</f>
@@ -2646,13 +2664,13 @@
         <v>11</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="H46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B47" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/check-if-all-the-integers-in-a-range-are-covered/", "1893")</f>
@@ -2672,13 +2690,13 @@
         <v>11</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="H47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B48" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/describe-the-painting/", "1943")</f>
@@ -2698,13 +2716,13 @@
         <v>11</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="H48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="B49" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shifting-letters-ii/", "2381")</f>
@@ -2724,13 +2742,13 @@
         <v>11</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H49" s="17"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B50" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/daily-temperatures/", "739")</f>
@@ -2750,13 +2768,13 @@
         <v>11</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B51" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-i/", "496")</f>
@@ -2776,13 +2794,13 @@
         <v>11</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="H51" s="17"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B52" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-ii/", "503")</f>
@@ -2802,13 +2820,13 @@
         <v>11</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B53" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/largest-rectangle-in-histogram/", "84")</f>
@@ -2828,13 +2846,13 @@
         <v>11</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="H53" s="17"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B54" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-rectangle/", "85")</f>
@@ -2854,13 +2872,13 @@
         <v>11</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="B55" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/online-stock-span/", "901")</f>
@@ -2880,13 +2898,13 @@
         <v>11</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B56" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sliding-window-maximum/", "239")</f>
@@ -2906,13 +2924,13 @@
         <v>11</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="H56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B57" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-subarray-with-sum-at-least-k/", "862")</f>
@@ -2932,13 +2950,13 @@
         <v>11</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="H57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B58" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/constrained-subsequence-sum/", "1425")</f>
@@ -2958,13 +2976,13 @@
         <v>11</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="H58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B59" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-continuous-subarray-with-absolute-diff-less-than-or-equal-to-limit/", "1438")</f>
@@ -2984,13 +3002,13 @@
         <v>11</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="H59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B60" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-value-of-equation/", "1499")</f>
@@ -3010,13 +3028,13 @@
         <v>11</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="H60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="B61" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-vi/", "1696")</f>
@@ -3036,13 +3054,13 @@
         <v>11</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="H61" s="17"/>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B62" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-an-array/", "215")</f>
@@ -3062,13 +3080,13 @@
         <v>11</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B63" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -3088,13 +3106,13 @@
         <v>11</v>
       </c>
       <c r="G63" s="16" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="H63" s="17"/>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B64" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-words/", "692")</f>
@@ -3114,13 +3132,13 @@
         <v>11</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="H64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B65" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-a-stream/", "703")</f>
@@ -3140,13 +3158,13 @@
         <v>11</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="H65" s="17"/>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B66" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/k-closest-points-to-origin/", "973")</f>
@@ -3166,13 +3184,13 @@
         <v>11</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="B67" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight/", "1046")</f>
@@ -3192,13 +3210,13 @@
         <v>11</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="H67" s="17"/>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B68" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-intervals/", "56")</f>
@@ -3218,13 +3236,13 @@
         <v>11</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="H68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B69" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/insert-interval/", "57")</f>
@@ -3244,13 +3262,13 @@
         <v>11</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="H69" s="17"/>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B70" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms/", "252")</f>
@@ -3270,15 +3288,15 @@
         <v>11</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>109</v>
-      </c>
-      <c r="H70" s="21" t="s">
-        <v>62</v>
+        <v>113</v>
+      </c>
+      <c r="H70" s="20" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B71" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms-ii/", "253")</f>
@@ -3298,15 +3316,15 @@
         <v>11</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>110</v>
-      </c>
-      <c r="H71" s="20" t="s">
-        <v>62</v>
+        <v>114</v>
+      </c>
+      <c r="H71" s="21" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B72" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/non-overlapping-intervals/", "435")</f>
@@ -3326,13 +3344,13 @@
         <v>11</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="B73" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-arrows-to-burst-balloons/", "452")</f>
@@ -3352,13 +3370,13 @@
         <v>11</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="H73" s="17"/>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B74" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-ii/", "45")</f>
@@ -3378,13 +3396,13 @@
         <v>11</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="H74" s="10"/>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="11" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B75" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game/", "55")</f>
@@ -3404,13 +3422,13 @@
         <v>11</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="H75" s="17"/>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B76" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/queue-reconstruction-by-height/", "406")</f>
@@ -3430,13 +3448,13 @@
         <v>11</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H76" s="10"/>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B77" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/task-scheduler/", "621")</f>
@@ -3456,13 +3474,13 @@
         <v>11</v>
       </c>
       <c r="G77" s="16" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="H77" s="17"/>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B78" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-labels/", "763")</f>
@@ -3482,13 +3500,13 @@
         <v>11</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="H78" s="10"/>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B79" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/gas-station/", "134")</f>
@@ -3508,13 +3526,13 @@
         <v>11</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="H79" s="17"/>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B80" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/", "21")</f>
@@ -3534,13 +3552,13 @@
         <v>11</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H80" s="10"/>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B81" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-k-sorted-lists/", "23")</f>
@@ -3560,13 +3578,13 @@
         <v>11</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="H81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B82" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swap-nodes-in-pairs/", "24")</f>
@@ -3586,13 +3604,13 @@
         <v>11</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="H82" s="10"/>
     </row>
     <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B83" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-nodes-in-k-group/", "25")</f>
@@ -3612,13 +3630,13 @@
         <v>11</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="H83" s="17"/>
     </row>
     <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B84" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-linked-list-ii/", "92")</f>
@@ -3638,13 +3656,13 @@
         <v>11</v>
       </c>
       <c r="G84" s="9" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="H84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="B85" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/copy-list-with-random-pointer/", "138")</f>
@@ -3664,13 +3682,13 @@
         <v>11</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="H85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B86" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximum-depth-of-binary-tree/", "104")</f>
@@ -3690,13 +3708,13 @@
         <v>11</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="H86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B87" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum/", "112")</f>
@@ -3716,13 +3734,13 @@
         <v>11</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="H87" s="17"/>
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B88" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum-ii/", "113")</f>
@@ -3742,13 +3760,13 @@
         <v>11</v>
       </c>
       <c r="G88" s="9" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="H88" s="10"/>
     </row>
     <row r="89" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B89" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/diameter-of-binary-tree/", "543")</f>
@@ -3768,13 +3786,13 @@
         <v>11</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="H89" s="17"/>
     </row>
     <row r="90" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B90" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-maximum-path-sum/", "124")</f>
@@ -3794,13 +3812,13 @@
         <v>11</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="H90" s="10"/>
     </row>
     <row r="91" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B91" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/invert-binary-tree/", "226")</f>
@@ -3820,13 +3838,13 @@
         <v>11</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="H91" s="17"/>
     </row>
     <row r="92" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B92" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-level-order-traversal/", "102")</f>
@@ -3846,13 +3864,13 @@
         <v>11</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="H92" s="10"/>
     </row>
     <row r="93" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B93" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/", "103")</f>
@@ -3872,13 +3890,13 @@
         <v>11</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="H93" s="17"/>
     </row>
     <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B94" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-right-side-view/", "199")</f>
@@ -3898,13 +3916,13 @@
         <v>11</v>
       </c>
       <c r="G94" s="9" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="H94" s="10"/>
     </row>
     <row r="95" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B95" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-largest-value-in-each-tree-row/", "515")</f>
@@ -3924,13 +3942,13 @@
         <v>11</v>
       </c>
       <c r="G95" s="16" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="H95" s="17"/>
     </row>
     <row r="96" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B96" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/average-of-levels-in-binary-tree/", "637")</f>
@@ -3950,13 +3968,13 @@
         <v>11</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H96" s="10"/>
     </row>
     <row r="97" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="B97" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/populating-next-right-pointers-in-each-node/", "116")</f>
@@ -3976,13 +3994,13 @@
         <v>11</v>
       </c>
       <c r="G97" s="16" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="H97" s="17"/>
     </row>
     <row r="98" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B98" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/validate-binary-search-tree/", "98")</f>
@@ -4002,13 +4020,13 @@
         <v>11</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="H98" s="10"/>
     </row>
     <row r="99" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B99" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/recover-binary-search-tree/", "99")</f>
@@ -4028,13 +4046,13 @@
         <v>11</v>
       </c>
       <c r="G99" s="16" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="H99" s="17"/>
     </row>
     <row r="100" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B100" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-smallest-element-in-a-bst/", "230")</f>
@@ -4054,13 +4072,13 @@
         <v>11</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="H100" s="10"/>
     </row>
     <row r="101" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B101" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/", "235")</f>
@@ -4080,13 +4098,13 @@
         <v>11</v>
       </c>
       <c r="G101" s="16" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="H101" s="17"/>
     </row>
     <row r="102" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B102" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-node-in-a-bst/", "450")</f>
@@ -4106,13 +4124,13 @@
         <v>11</v>
       </c>
       <c r="G102" s="9" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="H102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B103" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-a-binary-search-tree/", "700")</f>
@@ -4132,13 +4150,13 @@
         <v>11</v>
       </c>
       <c r="G103" s="16" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="H103" s="17"/>
     </row>
     <row r="104" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B104" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations/", "46")</f>
@@ -4158,13 +4176,13 @@
         <v>11</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="H104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B105" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations-ii/", "47")</f>
@@ -4184,13 +4202,13 @@
         <v>11</v>
       </c>
       <c r="G105" s="16" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="H105" s="17"/>
     </row>
     <row r="106" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B106" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combinations/", "77")</f>
@@ -4210,13 +4228,13 @@
         <v>11</v>
       </c>
       <c r="G106" s="9" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="H106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B107" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets/", "78")</f>
@@ -4236,13 +4254,13 @@
         <v>11</v>
       </c>
       <c r="G107" s="16" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="H107" s="17"/>
     </row>
     <row r="108" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B108" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets-ii/", "90")</f>
@@ -4262,13 +4280,13 @@
         <v>11</v>
       </c>
       <c r="G108" s="9" t="s">
-        <v>153</v>
+        <v>157</v>
       </c>
       <c r="H108" s="10"/>
     </row>
     <row r="109" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="11" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="B109" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum/", "39")</f>
@@ -4288,13 +4306,13 @@
         <v>11</v>
       </c>
       <c r="G109" s="16" t="s">
-        <v>154</v>
+        <v>158</v>
       </c>
       <c r="H109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B110" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum-ii/", "40")</f>
@@ -4314,13 +4332,13 @@
         <v>11</v>
       </c>
       <c r="G110" s="9" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="H110" s="10"/>
     </row>
     <row r="111" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B111" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/letter-combinations-of-a-phone-number/", "17")</f>
@@ -4340,13 +4358,13 @@
         <v>11</v>
       </c>
       <c r="G111" s="16" t="s">
-        <v>157</v>
+        <v>161</v>
       </c>
       <c r="H111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B112" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search/", "79")</f>
@@ -4366,13 +4384,13 @@
         <v>11</v>
       </c>
       <c r="G112" s="9" t="s">
-        <v>158</v>
+        <v>162</v>
       </c>
       <c r="H112" s="10"/>
     </row>
     <row r="113" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B113" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/palindrome-partitioning/", "131")</f>
@@ -4392,13 +4410,13 @@
         <v>11</v>
       </c>
       <c r="G113" s="16" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="H113" s="17"/>
     </row>
     <row r="114" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B114" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens/", "51")</f>
@@ -4418,13 +4436,13 @@
         <v>11</v>
       </c>
       <c r="G114" s="9" t="s">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="H114" s="10"/>
     </row>
     <row r="115" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="s">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="B115" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens-ii/", "52")</f>
@@ -4444,13 +4462,13 @@
         <v>11</v>
       </c>
       <c r="G115" s="16" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="H115" s="17"/>
     </row>
     <row r="116" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B116" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-islands/", "200")</f>
@@ -4470,13 +4488,13 @@
         <v>11</v>
       </c>
       <c r="G116" s="9" t="s">
-        <v>163</v>
+        <v>167</v>
       </c>
       <c r="H116" s="10"/>
     </row>
     <row r="117" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="11" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B117" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-area-of-island/", "695")</f>
@@ -4496,13 +4514,13 @@
         <v>11</v>
       </c>
       <c r="G117" s="16" t="s">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="H117" s="17"/>
     </row>
     <row r="118" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B118" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/flood-fill/", "733")</f>
@@ -4522,13 +4540,13 @@
         <v>11</v>
       </c>
       <c r="G118" s="9" t="s">
-        <v>165</v>
+        <v>169</v>
       </c>
       <c r="H118" s="10"/>
     </row>
     <row r="119" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B119" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/rotting-oranges/", "994")</f>
@@ -4548,13 +4566,13 @@
         <v>11</v>
       </c>
       <c r="G119" s="16" t="s">
-        <v>166</v>
+        <v>170</v>
       </c>
       <c r="H119" s="17"/>
     </row>
     <row r="120" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B120" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-path-in-binary-matrix/", "1091")</f>
@@ -4574,13 +4592,13 @@
         <v>11</v>
       </c>
       <c r="G120" s="9" t="s">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="H120" s="10"/>
     </row>
     <row r="121" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="11" t="s">
-        <v>162</v>
+        <v>166</v>
       </c>
       <c r="B121" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-closed-islands/", "1254")</f>
@@ -4600,13 +4618,13 @@
         <v>11</v>
       </c>
       <c r="G121" s="16" t="s">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="H121" s="17"/>
     </row>
     <row r="122" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B122" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule/", "207")</f>
@@ -4626,13 +4644,13 @@
         <v>11</v>
       </c>
       <c r="G122" s="9" t="s">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="H122" s="10"/>
     </row>
     <row r="123" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B123" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-ii/", "210")</f>
@@ -4652,13 +4670,13 @@
         <v>11</v>
       </c>
       <c r="G123" s="16" t="s">
-        <v>171</v>
+        <v>175</v>
       </c>
       <c r="H123" s="17"/>
     </row>
     <row r="124" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B124" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-eventual-safe-states/", "802")</f>
@@ -4678,13 +4696,13 @@
         <v>11</v>
       </c>
       <c r="G124" s="9" t="s">
-        <v>172</v>
+        <v>176</v>
       </c>
       <c r="H124" s="10"/>
     </row>
     <row r="125" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B125" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-iv/", "1462")</f>
@@ -4704,13 +4722,13 @@
         <v>11</v>
       </c>
       <c r="G125" s="16" t="s">
-        <v>173</v>
+        <v>177</v>
       </c>
       <c r="H125" s="17"/>
     </row>
     <row r="126" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B126" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sort-items-by-groups-respecting-dependencies/", "1203")</f>
@@ -4730,13 +4748,13 @@
         <v>11</v>
       </c>
       <c r="G126" s="9" t="s">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="H126" s="10"/>
     </row>
     <row r="127" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="11" t="s">
-        <v>169</v>
+        <v>173</v>
       </c>
       <c r="B127" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-all-possible-recipes-from-given-supplies/", "2115")</f>
@@ -4756,13 +4774,13 @@
         <v>11</v>
       </c>
       <c r="G127" s="16" t="s">
-        <v>175</v>
+        <v>179</v>
       </c>
       <c r="H127" s="17"/>
     </row>
     <row r="128" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B128" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-provinces/", "547")</f>
@@ -4782,13 +4800,13 @@
         <v>11</v>
       </c>
       <c r="G128" s="9" t="s">
-        <v>177</v>
+        <v>181</v>
       </c>
       <c r="H128" s="10"/>
     </row>
     <row r="129" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="11" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B129" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/redundant-connection/", "684")</f>
@@ -4808,13 +4826,13 @@
         <v>11</v>
       </c>
       <c r="G129" s="16" t="s">
-        <v>178</v>
+        <v>182</v>
       </c>
       <c r="H129" s="17"/>
     </row>
     <row r="130" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B130" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-operations-to-make-network-connected/", "1319")</f>
@@ -4834,13 +4852,13 @@
         <v>11</v>
       </c>
       <c r="G130" s="9" t="s">
-        <v>179</v>
+        <v>183</v>
       </c>
       <c r="H130" s="10"/>
     </row>
     <row r="131" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="11" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B131" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/remove-max-number-of-edges-to-keep-graph-fully-traversable/", "1579")</f>
@@ -4860,13 +4878,13 @@
         <v>11</v>
       </c>
       <c r="G131" s="16" t="s">
-        <v>180</v>
+        <v>184</v>
       </c>
       <c r="H131" s="17"/>
     </row>
     <row r="132" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B132" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/satisfiability-of-equality-equations/", "990")</f>
@@ -4886,13 +4904,13 @@
         <v>11</v>
       </c>
       <c r="G132" s="9" t="s">
-        <v>181</v>
+        <v>185</v>
       </c>
       <c r="H132" s="10"/>
     </row>
     <row r="133" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="11" t="s">
-        <v>176</v>
+        <v>180</v>
       </c>
       <c r="B133" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/smallest-string-with-swaps/", "1202")</f>
@@ -4912,13 +4930,13 @@
         <v>11</v>
       </c>
       <c r="G133" s="16" t="s">
-        <v>182</v>
+        <v>186</v>
       </c>
       <c r="H133" s="17"/>
     </row>
     <row r="134" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B134" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/network-delay-time/", "743")</f>
@@ -4938,13 +4956,13 @@
         <v>11</v>
       </c>
       <c r="G134" s="9" t="s">
-        <v>184</v>
+        <v>188</v>
       </c>
       <c r="H134" s="10"/>
     </row>
     <row r="135" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="11" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B135" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/cheapest-flights-within-k-stops/", "787")</f>
@@ -4964,13 +4982,13 @@
         <v>11</v>
       </c>
       <c r="G135" s="16" t="s">
-        <v>185</v>
+        <v>189</v>
       </c>
       <c r="H135" s="17"/>
     </row>
     <row r="136" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B136" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-probability/", "1514")</f>
@@ -4990,13 +5008,13 @@
         <v>11</v>
       </c>
       <c r="G136" s="9" t="s">
-        <v>186</v>
+        <v>190</v>
       </c>
       <c r="H136" s="10"/>
     </row>
     <row r="137" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="11" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B137" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-minimum-effort/", "1631")</f>
@@ -5016,13 +5034,13 @@
         <v>11</v>
       </c>
       <c r="G137" s="16" t="s">
-        <v>187</v>
+        <v>191</v>
       </c>
       <c r="H137" s="17"/>
     </row>
     <row r="138" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B138" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/", "1334")</f>
@@ -5042,13 +5060,13 @@
         <v>11</v>
       </c>
       <c r="G138" s="9" t="s">
-        <v>188</v>
+        <v>192</v>
       </c>
       <c r="H138" s="10"/>
     </row>
     <row r="139" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="11" t="s">
-        <v>183</v>
+        <v>187</v>
       </c>
       <c r="B139" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-ways-to-arrive-at-destination/", "1976")</f>
@@ -5068,13 +5086,13 @@
         <v>11</v>
       </c>
       <c r="G139" s="16" t="s">
-        <v>189</v>
+        <v>193</v>
       </c>
       <c r="H139" s="17"/>
     </row>
     <row r="140" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B140" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/min-cost-to-connect-all-points/", "1584")</f>
@@ -5094,13 +5112,13 @@
         <v>11</v>
       </c>
       <c r="G140" s="9" t="s">
-        <v>191</v>
+        <v>195</v>
       </c>
       <c r="H140" s="10"/>
     </row>
     <row r="141" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B141" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/connecting-cities-with-minimum-cost/", "1135")</f>
@@ -5120,15 +5138,15 @@
         <v>11</v>
       </c>
       <c r="G141" s="16" t="s">
-        <v>192</v>
-      </c>
-      <c r="H141" s="20" t="s">
-        <v>62</v>
+        <v>196</v>
+      </c>
+      <c r="H141" s="21" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B142" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/optimize-water-distribution-in-a-village/", "1168")</f>
@@ -5148,15 +5166,15 @@
         <v>11</v>
       </c>
       <c r="G142" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="H142" s="21" t="s">
-        <v>62</v>
+        <v>197</v>
+      </c>
+      <c r="H142" s="20" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B143" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-critical-and-pseudo-critical-edges-in-minimum-spanning-tree/", "1489")</f>
@@ -5176,13 +5194,13 @@
         <v>11</v>
       </c>
       <c r="G143" s="16" t="s">
-        <v>194</v>
+        <v>198</v>
       </c>
       <c r="H143" s="17"/>
     </row>
     <row r="144" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B144" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swim-in-rising-water/", "778")</f>
@@ -5202,13 +5220,13 @@
         <v>11</v>
       </c>
       <c r="G144" s="9" t="s">
-        <v>195</v>
+        <v>199</v>
       </c>
       <c r="H144" s="10"/>
     </row>
     <row r="145" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="11" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B145" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-minimum-value/", "1102")</f>
@@ -5228,15 +5246,15 @@
         <v>11</v>
       </c>
       <c r="G145" s="16" t="s">
-        <v>196</v>
-      </c>
-      <c r="H145" s="20" t="s">
-        <v>62</v>
+        <v>200</v>
+      </c>
+      <c r="H145" s="21" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B146" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/implement-trie-prefix-tree/", "208")</f>
@@ -5256,13 +5274,13 @@
         <v>11</v>
       </c>
       <c r="G146" s="9" t="s">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="H146" s="10"/>
     </row>
     <row r="147" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="11" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B147" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/design-add-and-search-words-data-structure/", "211")</f>
@@ -5282,13 +5300,13 @@
         <v>11</v>
       </c>
       <c r="G147" s="16" t="s">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="H147" s="17"/>
     </row>
     <row r="148" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B148" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search-ii/", "212")</f>
@@ -5308,13 +5326,13 @@
         <v>11</v>
       </c>
       <c r="G148" s="9" t="s">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="H148" s="10"/>
     </row>
     <row r="149" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B149" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/replace-words/", "648")</f>
@@ -5334,13 +5352,13 @@
         <v>11</v>
       </c>
       <c r="G149" s="16" t="s">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="H149" s="17"/>
     </row>
     <row r="150" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B150" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/map-sum-pairs/", "677")</f>
@@ -5360,13 +5378,13 @@
         <v>11</v>
       </c>
       <c r="G150" s="9" t="s">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="H150" s="10"/>
     </row>
     <row r="151" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="11" t="s">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="B151" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-suggestions-system/", "1268")</f>
@@ -5386,13 +5404,13 @@
         <v>11</v>
       </c>
       <c r="G151" s="16" t="s">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="H151" s="17"/>
     </row>
     <row r="152" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B152" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number/", "136")</f>
@@ -5412,13 +5430,13 @@
         <v>11</v>
       </c>
       <c r="G152" s="9" t="s">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="H152" s="10"/>
     </row>
     <row r="153" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="11" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B153" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number-ii/", "137")</f>
@@ -5438,13 +5456,13 @@
         <v>11</v>
       </c>
       <c r="G153" s="16" t="s">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="H153" s="17"/>
     </row>
     <row r="154" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B154" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-1-bits/", "191")</f>
@@ -5464,13 +5482,13 @@
         <v>11</v>
       </c>
       <c r="G154" s="9" t="s">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="H154" s="10"/>
     </row>
     <row r="155" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="11" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B155" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/counting-bits/", "338")</f>
@@ -5490,13 +5508,13 @@
         <v>11</v>
       </c>
       <c r="G155" s="16" t="s">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="H155" s="17"/>
     </row>
     <row r="156" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B156" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/missing-number/", "268")</f>
@@ -5516,13 +5534,13 @@
         <v>11</v>
       </c>
       <c r="G156" s="9" t="s">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="H156" s="10"/>
     </row>
     <row r="157" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="11" t="s">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="B157" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-bits/", "190")</f>
@@ -5542,13 +5560,13 @@
         <v>11</v>
       </c>
       <c r="G157" s="16" t="s">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="H157" s="17"/>
     </row>
     <row r="158" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B158" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/climbing-stairs/", "70")</f>
@@ -5568,13 +5586,13 @@
         <v>11</v>
       </c>
       <c r="G158" s="9" t="s">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="H158" s="10"/>
     </row>
     <row r="159" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="11" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B159" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber/", "198")</f>
@@ -5594,13 +5612,13 @@
         <v>11</v>
       </c>
       <c r="G159" s="16" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="H159" s="17"/>
     </row>
     <row r="160" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B160" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber-ii/", "213")</f>
@@ -5620,13 +5638,13 @@
         <v>11</v>
       </c>
       <c r="G160" s="9" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="H160" s="10"/>
     </row>
     <row r="161" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="11" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B161" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change/", "322")</f>
@@ -5646,13 +5664,13 @@
         <v>11</v>
       </c>
       <c r="G161" s="16" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="H161" s="17"/>
     </row>
     <row r="162" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B162" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/perfect-squares/", "279")</f>
@@ -5672,13 +5690,13 @@
         <v>11</v>
       </c>
       <c r="G162" s="9" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="H162" s="10"/>
     </row>
     <row r="163" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="11" t="s">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="B163" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-increasing-subsequence/", "300")</f>
@@ -5698,13 +5716,13 @@
         <v>11</v>
       </c>
       <c r="G163" s="16" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="H163" s="17"/>
     </row>
     <row r="164" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B164" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-equal-subset-sum/", "416")</f>
@@ -5724,13 +5742,13 @@
         <v>11</v>
       </c>
       <c r="G164" s="9" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="H164" s="10"/>
     </row>
     <row r="165" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="11" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B165" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/target-sum/", "494")</f>
@@ -5750,13 +5768,13 @@
         <v>11</v>
       </c>
       <c r="G165" s="16" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="H165" s="17"/>
     </row>
     <row r="166" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B166" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change-ii/", "518")</f>
@@ -5776,13 +5794,13 @@
         <v>11</v>
       </c>
       <c r="G166" s="9" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="H166" s="10"/>
     </row>
     <row r="167" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="11" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B167" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/ones-and-zeroes/", "474")</f>
@@ -5802,13 +5820,13 @@
         <v>11</v>
       </c>
       <c r="G167" s="16" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="H167" s="17"/>
     </row>
     <row r="168" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="3" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B168" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight-ii/", "1049")</f>
@@ -5828,13 +5846,13 @@
         <v>11</v>
       </c>
       <c r="G168" s="9" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="H168" s="10"/>
     </row>
     <row r="169" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="11" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="B169" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/profitable-schemes/", "879")</f>
@@ -5854,13 +5872,13 @@
         <v>11</v>
       </c>
       <c r="G169" s="16" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="H169" s="17"/>
     </row>
     <row r="170" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="3" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B170" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths/", "62")</f>
@@ -5880,13 +5898,13 @@
         <v>11</v>
       </c>
       <c r="G170" s="9" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="H170" s="10"/>
     </row>
     <row r="171" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B171" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths-ii/", "63")</f>
@@ -5906,13 +5924,13 @@
         <v>11</v>
       </c>
       <c r="G171" s="16" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="H171" s="17"/>
     </row>
     <row r="172" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="3" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B172" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-path-sum/", "64")</f>
@@ -5932,13 +5950,13 @@
         <v>11</v>
       </c>
       <c r="G172" s="9" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="H172" s="10"/>
     </row>
     <row r="173" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="11" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B173" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-square/", "221")</f>
@@ -5958,13 +5976,13 @@
         <v>11</v>
       </c>
       <c r="G173" s="16" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="H173" s="17"/>
     </row>
     <row r="174" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B174" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-falling-path-sum/", "931")</f>
@@ -5984,13 +6002,13 @@
         <v>11</v>
       </c>
       <c r="G174" s="9" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="H174" s="10"/>
     </row>
     <row r="175" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="11" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="B175" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/triangle/", "120")</f>
@@ -6010,13 +6028,13 @@
         <v>11</v>
       </c>
       <c r="G175" s="16" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="H175" s="17"/>
     </row>
     <row r="176" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="3" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B176" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-common-subsequence/", "1143")</f>
@@ -6036,13 +6054,13 @@
         <v>11</v>
       </c>
       <c r="G176" s="9" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="H176" s="10"/>
     </row>
     <row r="177" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="11" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B177" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/edit-distance/", "72")</f>
@@ -6062,13 +6080,13 @@
         <v>11</v>
       </c>
       <c r="G177" s="16" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="H177" s="17"/>
     </row>
     <row r="178" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="3" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B178" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/distinct-subsequences/", "115")</f>
@@ -6088,13 +6106,13 @@
         <v>11</v>
       </c>
       <c r="G178" s="9" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="H178" s="10"/>
     </row>
     <row r="179" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="11" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B179" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-operation-for-two-strings/", "583")</f>
@@ -6114,13 +6132,13 @@
         <v>11</v>
       </c>
       <c r="G179" s="16" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="H179" s="17"/>
     </row>
     <row r="180" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="3" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B180" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/interleaving-string/", "97")</f>
@@ -6140,13 +6158,13 @@
         <v>11</v>
       </c>
       <c r="G180" s="9" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="H180" s="10"/>
     </row>
     <row r="181" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="11" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="B181" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-insertion-steps-to-make-a-string-palindrome/", "1312")</f>
@@ -6166,7 +6184,7 @@
         <v>11</v>
       </c>
       <c r="G181" s="16" t="s">
-        <v>238</v>
+        <v>242</v>
       </c>
       <c r="H181" s="17"/>
     </row>

</xml_diff>

<commit_message>
finished all hash map problems. updated spreadsheet.
</commit_message>
<xml_diff>
--- a/leetcode_roadmap.xlsx
+++ b/leetcode_roadmap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="934" uniqueCount="243">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="249">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -235,19 +235,37 @@
     <t xml:space="preserve">https://leetcode.com/problems/two-sum/</t>
   </si>
   <si>
+    <t xml:space="preserve">very simple. Don’t overcompicate. Create a hashmap and add to it if the current val isn’t present.</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/group-anagrams/</t>
   </si>
   <si>
+    <t xml:space="preserve">sorting each string and hashing</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/longest-consecutive-sequence/</t>
   </si>
   <si>
+    <t xml:space="preserve">find the start of the streak and check if following consecutive numbers exist in the lookup table and count the streak.</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/contains-duplicate/</t>
   </si>
   <si>
+    <t xml:space="preserve">store in a hash table (set). Compare size of the set to the size of the input array.</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/valid-anagram/</t>
   </si>
   <si>
+    <t xml:space="preserve">create a hash table. Calc frequency of chars of string a. Negate freq of chars of string b. If final hash table has 0 for all, then it is an anagram</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/top-k-frequent-elements/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">using a priority queue will make this easier but you don’t have to.</t>
   </si>
   <si>
     <t xml:space="preserve">Prefix Sum / Running Sum</t>
@@ -2291,8 +2309,8 @@
       <c r="D32" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E32" s="8" t="s">
-        <v>11</v>
+      <c r="E32" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F32" s="8" t="s">
         <v>11</v>
@@ -2300,7 +2318,9 @@
       <c r="G32" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="H32" s="10"/>
+      <c r="H32" s="10" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="s">
@@ -2317,16 +2337,18 @@
       <c r="D33" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E33" s="15" t="s">
-        <v>11</v>
+      <c r="E33" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F33" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G33" s="16" t="s">
-        <v>70</v>
-      </c>
-      <c r="H33" s="17"/>
+        <v>71</v>
+      </c>
+      <c r="H33" s="17" t="s">
+        <v>72</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
@@ -2343,16 +2365,18 @@
       <c r="D34" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E34" s="8" t="s">
-        <v>11</v>
+      <c r="E34" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F34" s="8" t="s">
         <v>11</v>
       </c>
       <c r="G34" s="9" t="s">
-        <v>71</v>
-      </c>
-      <c r="H34" s="10"/>
+        <v>73</v>
+      </c>
+      <c r="H34" s="10" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="s">
@@ -2369,16 +2393,18 @@
       <c r="D35" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E35" s="15" t="s">
-        <v>11</v>
+      <c r="E35" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F35" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G35" s="16" t="s">
-        <v>72</v>
-      </c>
-      <c r="H35" s="17"/>
+        <v>75</v>
+      </c>
+      <c r="H35" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="3" t="s">
@@ -2395,16 +2421,18 @@
       <c r="D36" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E36" s="8" t="s">
-        <v>11</v>
+      <c r="E36" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F36" s="8" t="s">
         <v>11</v>
       </c>
       <c r="G36" s="9" t="s">
-        <v>73</v>
-      </c>
-      <c r="H36" s="10"/>
+        <v>77</v>
+      </c>
+      <c r="H36" s="10" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
@@ -2421,20 +2449,22 @@
       <c r="D37" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E37" s="15" t="s">
-        <v>11</v>
+      <c r="E37" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F37" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G37" s="16" t="s">
-        <v>74</v>
-      </c>
-      <c r="H37" s="17"/>
+        <v>79</v>
+      </c>
+      <c r="H37" s="17" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="3" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B38" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-sum-query-immutable/", "303")</f>
@@ -2454,13 +2484,13 @@
         <v>11</v>
       </c>
       <c r="G38" s="9" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="H38" s="10"/>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B39" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sum-equals-k/", "560")</f>
@@ -2480,13 +2510,13 @@
         <v>11</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="H39" s="17"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B40" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-pivot-index/", "724")</f>
@@ -2506,13 +2536,13 @@
         <v>11</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="H40" s="10"/>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B41" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-subarrays-with-sum/", "930")</f>
@@ -2532,13 +2562,13 @@
         <v>11</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="H41" s="17"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B42" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subarray-sums-divisible-by-k/", "974")</f>
@@ -2558,13 +2588,13 @@
         <v>11</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="H42" s="10"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B43" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/continuous-subarray-sum/", "523")</f>
@@ -2584,13 +2614,13 @@
         <v>11</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="H43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B44" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-addition/", "370")</f>
@@ -2610,15 +2640,15 @@
         <v>11</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="H44" s="20" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B45" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/car-pooling/", "1094")</f>
@@ -2638,13 +2668,13 @@
         <v>11</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="H45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B46" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/corporate-flight-bookings/", "1109")</f>
@@ -2664,13 +2694,13 @@
         <v>11</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>86</v>
+        <v>92</v>
       </c>
       <c r="H46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B47" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/check-if-all-the-integers-in-a-range-are-covered/", "1893")</f>
@@ -2690,13 +2720,13 @@
         <v>11</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="H47" s="17"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B48" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/describe-the-painting/", "1943")</f>
@@ -2716,13 +2746,13 @@
         <v>11</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>88</v>
+        <v>94</v>
       </c>
       <c r="H48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B49" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shifting-letters-ii/", "2381")</f>
@@ -2742,13 +2772,13 @@
         <v>11</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>89</v>
+        <v>95</v>
       </c>
       <c r="H49" s="17"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B50" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/daily-temperatures/", "739")</f>
@@ -2768,13 +2798,13 @@
         <v>11</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="H50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B51" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-i/", "496")</f>
@@ -2794,13 +2824,13 @@
         <v>11</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="H51" s="17"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B52" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-ii/", "503")</f>
@@ -2820,13 +2850,13 @@
         <v>11</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="H52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B53" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/largest-rectangle-in-histogram/", "84")</f>
@@ -2846,13 +2876,13 @@
         <v>11</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="H53" s="17"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B54" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-rectangle/", "85")</f>
@@ -2872,13 +2902,13 @@
         <v>11</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="H54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="B55" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/online-stock-span/", "901")</f>
@@ -2898,13 +2928,13 @@
         <v>11</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="H55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B56" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sliding-window-maximum/", "239")</f>
@@ -2924,13 +2954,13 @@
         <v>11</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="H56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B57" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-subarray-with-sum-at-least-k/", "862")</f>
@@ -2950,13 +2980,13 @@
         <v>11</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="H57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B58" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/constrained-subsequence-sum/", "1425")</f>
@@ -2976,13 +3006,13 @@
         <v>11</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="H58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B59" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-continuous-subarray-with-absolute-diff-less-than-or-equal-to-limit/", "1438")</f>
@@ -3002,13 +3032,13 @@
         <v>11</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="H59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B60" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-value-of-equation/", "1499")</f>
@@ -3028,13 +3058,13 @@
         <v>11</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="H60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="B61" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-vi/", "1696")</f>
@@ -3054,13 +3084,13 @@
         <v>11</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="H61" s="17"/>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B62" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-an-array/", "215")</f>
@@ -3080,13 +3110,13 @@
         <v>11</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="H62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B63" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -3106,13 +3136,13 @@
         <v>11</v>
       </c>
       <c r="G63" s="16" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="H63" s="17"/>
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B64" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-words/", "692")</f>
@@ -3132,13 +3162,13 @@
         <v>11</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="H64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B65" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-a-stream/", "703")</f>
@@ -3158,13 +3188,13 @@
         <v>11</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="H65" s="17"/>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B66" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/k-closest-points-to-origin/", "973")</f>
@@ -3184,13 +3214,13 @@
         <v>11</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="H66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="B67" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight/", "1046")</f>
@@ -3210,13 +3240,13 @@
         <v>11</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="H67" s="17"/>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B68" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-intervals/", "56")</f>
@@ -3236,13 +3266,13 @@
         <v>11</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="H68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B69" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/insert-interval/", "57")</f>
@@ -3262,13 +3292,13 @@
         <v>11</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="H69" s="17"/>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B70" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms/", "252")</f>
@@ -3288,15 +3318,15 @@
         <v>11</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="H70" s="20" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B71" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms-ii/", "253")</f>
@@ -3316,15 +3346,15 @@
         <v>11</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="H71" s="21" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B72" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/non-overlapping-intervals/", "435")</f>
@@ -3344,13 +3374,13 @@
         <v>11</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="H72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="B73" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-arrows-to-burst-balloons/", "452")</f>
@@ -3370,13 +3400,13 @@
         <v>11</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="H73" s="17"/>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B74" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-ii/", "45")</f>
@@ -3396,13 +3426,13 @@
         <v>11</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="H74" s="10"/>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="11" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B75" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game/", "55")</f>
@@ -3422,13 +3452,13 @@
         <v>11</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="H75" s="17"/>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B76" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/queue-reconstruction-by-height/", "406")</f>
@@ -3448,13 +3478,13 @@
         <v>11</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="H76" s="10"/>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B77" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/task-scheduler/", "621")</f>
@@ -3474,13 +3504,13 @@
         <v>11</v>
       </c>
       <c r="G77" s="16" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="H77" s="17"/>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B78" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-labels/", "763")</f>
@@ -3500,13 +3530,13 @@
         <v>11</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="H78" s="10"/>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="B79" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/gas-station/", "134")</f>
@@ -3526,13 +3556,13 @@
         <v>11</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="H79" s="17"/>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B80" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/", "21")</f>
@@ -3552,13 +3582,13 @@
         <v>11</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="H80" s="10"/>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B81" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-k-sorted-lists/", "23")</f>
@@ -3578,13 +3608,13 @@
         <v>11</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="H81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B82" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swap-nodes-in-pairs/", "24")</f>
@@ -3604,13 +3634,13 @@
         <v>11</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="H82" s="10"/>
     </row>
     <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B83" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-nodes-in-k-group/", "25")</f>
@@ -3630,13 +3660,13 @@
         <v>11</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>128</v>
+        <v>134</v>
       </c>
       <c r="H83" s="17"/>
     </row>
     <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B84" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-linked-list-ii/", "92")</f>
@@ -3656,13 +3686,13 @@
         <v>11</v>
       </c>
       <c r="G84" s="9" t="s">
-        <v>129</v>
+        <v>135</v>
       </c>
       <c r="H84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="B85" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/copy-list-with-random-pointer/", "138")</f>
@@ -3682,13 +3712,13 @@
         <v>11</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>130</v>
+        <v>136</v>
       </c>
       <c r="H85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B86" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximum-depth-of-binary-tree/", "104")</f>
@@ -3708,13 +3738,13 @@
         <v>11</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="H86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B87" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum/", "112")</f>
@@ -3734,13 +3764,13 @@
         <v>11</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>133</v>
+        <v>139</v>
       </c>
       <c r="H87" s="17"/>
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B88" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum-ii/", "113")</f>
@@ -3760,13 +3790,13 @@
         <v>11</v>
       </c>
       <c r="G88" s="9" t="s">
-        <v>134</v>
+        <v>140</v>
       </c>
       <c r="H88" s="10"/>
     </row>
     <row r="89" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B89" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/diameter-of-binary-tree/", "543")</f>
@@ -3786,13 +3816,13 @@
         <v>11</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="H89" s="17"/>
     </row>
     <row r="90" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B90" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-maximum-path-sum/", "124")</f>
@@ -3812,13 +3842,13 @@
         <v>11</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="H90" s="10"/>
     </row>
     <row r="91" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>131</v>
+        <v>137</v>
       </c>
       <c r="B91" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/invert-binary-tree/", "226")</f>
@@ -3838,13 +3868,13 @@
         <v>11</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>137</v>
+        <v>143</v>
       </c>
       <c r="H91" s="17"/>
     </row>
     <row r="92" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B92" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-level-order-traversal/", "102")</f>
@@ -3864,13 +3894,13 @@
         <v>11</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>139</v>
+        <v>145</v>
       </c>
       <c r="H92" s="10"/>
     </row>
     <row r="93" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B93" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/", "103")</f>
@@ -3890,13 +3920,13 @@
         <v>11</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="H93" s="17"/>
     </row>
     <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B94" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-right-side-view/", "199")</f>
@@ -3916,13 +3946,13 @@
         <v>11</v>
       </c>
       <c r="G94" s="9" t="s">
-        <v>141</v>
+        <v>147</v>
       </c>
       <c r="H94" s="10"/>
     </row>
     <row r="95" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B95" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-largest-value-in-each-tree-row/", "515")</f>
@@ -3942,13 +3972,13 @@
         <v>11</v>
       </c>
       <c r="G95" s="16" t="s">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="H95" s="17"/>
     </row>
     <row r="96" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B96" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/average-of-levels-in-binary-tree/", "637")</f>
@@ -3968,13 +3998,13 @@
         <v>11</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>143</v>
+        <v>149</v>
       </c>
       <c r="H96" s="10"/>
     </row>
     <row r="97" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="B97" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/populating-next-right-pointers-in-each-node/", "116")</f>
@@ -3994,13 +4024,13 @@
         <v>11</v>
       </c>
       <c r="G97" s="16" t="s">
-        <v>144</v>
+        <v>150</v>
       </c>
       <c r="H97" s="17"/>
     </row>
     <row r="98" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B98" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/validate-binary-search-tree/", "98")</f>
@@ -4020,13 +4050,13 @@
         <v>11</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>146</v>
+        <v>152</v>
       </c>
       <c r="H98" s="10"/>
     </row>
     <row r="99" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B99" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/recover-binary-search-tree/", "99")</f>
@@ -4046,13 +4076,13 @@
         <v>11</v>
       </c>
       <c r="G99" s="16" t="s">
-        <v>147</v>
+        <v>153</v>
       </c>
       <c r="H99" s="17"/>
     </row>
     <row r="100" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B100" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-smallest-element-in-a-bst/", "230")</f>
@@ -4072,13 +4102,13 @@
         <v>11</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="H100" s="10"/>
     </row>
     <row r="101" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B101" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/", "235")</f>
@@ -4098,13 +4128,13 @@
         <v>11</v>
       </c>
       <c r="G101" s="16" t="s">
-        <v>149</v>
+        <v>155</v>
       </c>
       <c r="H101" s="17"/>
     </row>
     <row r="102" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B102" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-node-in-a-bst/", "450")</f>
@@ -4124,13 +4154,13 @@
         <v>11</v>
       </c>
       <c r="G102" s="9" t="s">
-        <v>150</v>
+        <v>156</v>
       </c>
       <c r="H102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="s">
-        <v>145</v>
+        <v>151</v>
       </c>
       <c r="B103" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-a-binary-search-tree/", "700")</f>
@@ -4150,13 +4180,13 @@
         <v>11</v>
       </c>
       <c r="G103" s="16" t="s">
-        <v>151</v>
+        <v>157</v>
       </c>
       <c r="H103" s="17"/>
     </row>
     <row r="104" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B104" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations/", "46")</f>
@@ -4176,13 +4206,13 @@
         <v>11</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>153</v>
+        <v>159</v>
       </c>
       <c r="H104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B105" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations-ii/", "47")</f>
@@ -4202,13 +4232,13 @@
         <v>11</v>
       </c>
       <c r="G105" s="16" t="s">
-        <v>154</v>
+        <v>160</v>
       </c>
       <c r="H105" s="17"/>
     </row>
     <row r="106" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B106" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combinations/", "77")</f>
@@ -4228,13 +4258,13 @@
         <v>11</v>
       </c>
       <c r="G106" s="9" t="s">
-        <v>155</v>
+        <v>161</v>
       </c>
       <c r="H106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B107" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets/", "78")</f>
@@ -4254,13 +4284,13 @@
         <v>11</v>
       </c>
       <c r="G107" s="16" t="s">
-        <v>156</v>
+        <v>162</v>
       </c>
       <c r="H107" s="17"/>
     </row>
     <row r="108" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B108" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets-ii/", "90")</f>
@@ -4280,13 +4310,13 @@
         <v>11</v>
       </c>
       <c r="G108" s="9" t="s">
-        <v>157</v>
+        <v>163</v>
       </c>
       <c r="H108" s="10"/>
     </row>
     <row r="109" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="11" t="s">
-        <v>152</v>
+        <v>158</v>
       </c>
       <c r="B109" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum/", "39")</f>
@@ -4306,13 +4336,13 @@
         <v>11</v>
       </c>
       <c r="G109" s="16" t="s">
-        <v>158</v>
+        <v>164</v>
       </c>
       <c r="H109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B110" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum-ii/", "40")</f>
@@ -4332,13 +4362,13 @@
         <v>11</v>
       </c>
       <c r="G110" s="9" t="s">
-        <v>160</v>
+        <v>166</v>
       </c>
       <c r="H110" s="10"/>
     </row>
     <row r="111" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B111" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/letter-combinations-of-a-phone-number/", "17")</f>
@@ -4358,13 +4388,13 @@
         <v>11</v>
       </c>
       <c r="G111" s="16" t="s">
-        <v>161</v>
+        <v>167</v>
       </c>
       <c r="H111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B112" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search/", "79")</f>
@@ -4384,13 +4414,13 @@
         <v>11</v>
       </c>
       <c r="G112" s="9" t="s">
-        <v>162</v>
+        <v>168</v>
       </c>
       <c r="H112" s="10"/>
     </row>
     <row r="113" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B113" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/palindrome-partitioning/", "131")</f>
@@ -4410,13 +4440,13 @@
         <v>11</v>
       </c>
       <c r="G113" s="16" t="s">
-        <v>163</v>
+        <v>169</v>
       </c>
       <c r="H113" s="17"/>
     </row>
     <row r="114" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B114" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens/", "51")</f>
@@ -4436,13 +4466,13 @@
         <v>11</v>
       </c>
       <c r="G114" s="9" t="s">
-        <v>164</v>
+        <v>170</v>
       </c>
       <c r="H114" s="10"/>
     </row>
     <row r="115" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="s">
-        <v>159</v>
+        <v>165</v>
       </c>
       <c r="B115" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens-ii/", "52")</f>
@@ -4462,13 +4492,13 @@
         <v>11</v>
       </c>
       <c r="G115" s="16" t="s">
-        <v>165</v>
+        <v>171</v>
       </c>
       <c r="H115" s="17"/>
     </row>
     <row r="116" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B116" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-islands/", "200")</f>
@@ -4488,13 +4518,13 @@
         <v>11</v>
       </c>
       <c r="G116" s="9" t="s">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="H116" s="10"/>
     </row>
     <row r="117" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="11" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B117" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-area-of-island/", "695")</f>
@@ -4514,13 +4544,13 @@
         <v>11</v>
       </c>
       <c r="G117" s="16" t="s">
-        <v>168</v>
+        <v>174</v>
       </c>
       <c r="H117" s="17"/>
     </row>
     <row r="118" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B118" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/flood-fill/", "733")</f>
@@ -4540,13 +4570,13 @@
         <v>11</v>
       </c>
       <c r="G118" s="9" t="s">
-        <v>169</v>
+        <v>175</v>
       </c>
       <c r="H118" s="10"/>
     </row>
     <row r="119" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B119" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/rotting-oranges/", "994")</f>
@@ -4566,13 +4596,13 @@
         <v>11</v>
       </c>
       <c r="G119" s="16" t="s">
-        <v>170</v>
+        <v>176</v>
       </c>
       <c r="H119" s="17"/>
     </row>
     <row r="120" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B120" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-path-in-binary-matrix/", "1091")</f>
@@ -4592,13 +4622,13 @@
         <v>11</v>
       </c>
       <c r="G120" s="9" t="s">
-        <v>171</v>
+        <v>177</v>
       </c>
       <c r="H120" s="10"/>
     </row>
     <row r="121" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="11" t="s">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="B121" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-closed-islands/", "1254")</f>
@@ -4618,13 +4648,13 @@
         <v>11</v>
       </c>
       <c r="G121" s="16" t="s">
-        <v>172</v>
+        <v>178</v>
       </c>
       <c r="H121" s="17"/>
     </row>
     <row r="122" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B122" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule/", "207")</f>
@@ -4644,13 +4674,13 @@
         <v>11</v>
       </c>
       <c r="G122" s="9" t="s">
-        <v>174</v>
+        <v>180</v>
       </c>
       <c r="H122" s="10"/>
     </row>
     <row r="123" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B123" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-ii/", "210")</f>
@@ -4670,13 +4700,13 @@
         <v>11</v>
       </c>
       <c r="G123" s="16" t="s">
-        <v>175</v>
+        <v>181</v>
       </c>
       <c r="H123" s="17"/>
     </row>
     <row r="124" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B124" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-eventual-safe-states/", "802")</f>
@@ -4696,13 +4726,13 @@
         <v>11</v>
       </c>
       <c r="G124" s="9" t="s">
-        <v>176</v>
+        <v>182</v>
       </c>
       <c r="H124" s="10"/>
     </row>
     <row r="125" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B125" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-iv/", "1462")</f>
@@ -4722,13 +4752,13 @@
         <v>11</v>
       </c>
       <c r="G125" s="16" t="s">
-        <v>177</v>
+        <v>183</v>
       </c>
       <c r="H125" s="17"/>
     </row>
     <row r="126" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B126" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sort-items-by-groups-respecting-dependencies/", "1203")</f>
@@ -4748,13 +4778,13 @@
         <v>11</v>
       </c>
       <c r="G126" s="9" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="H126" s="10"/>
     </row>
     <row r="127" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="11" t="s">
-        <v>173</v>
+        <v>179</v>
       </c>
       <c r="B127" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-all-possible-recipes-from-given-supplies/", "2115")</f>
@@ -4774,13 +4804,13 @@
         <v>11</v>
       </c>
       <c r="G127" s="16" t="s">
-        <v>179</v>
+        <v>185</v>
       </c>
       <c r="H127" s="17"/>
     </row>
     <row r="128" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B128" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-provinces/", "547")</f>
@@ -4800,13 +4830,13 @@
         <v>11</v>
       </c>
       <c r="G128" s="9" t="s">
-        <v>181</v>
+        <v>187</v>
       </c>
       <c r="H128" s="10"/>
     </row>
     <row r="129" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="11" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B129" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/redundant-connection/", "684")</f>
@@ -4826,13 +4856,13 @@
         <v>11</v>
       </c>
       <c r="G129" s="16" t="s">
-        <v>182</v>
+        <v>188</v>
       </c>
       <c r="H129" s="17"/>
     </row>
     <row r="130" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B130" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-operations-to-make-network-connected/", "1319")</f>
@@ -4852,13 +4882,13 @@
         <v>11</v>
       </c>
       <c r="G130" s="9" t="s">
-        <v>183</v>
+        <v>189</v>
       </c>
       <c r="H130" s="10"/>
     </row>
     <row r="131" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="11" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B131" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/remove-max-number-of-edges-to-keep-graph-fully-traversable/", "1579")</f>
@@ -4878,13 +4908,13 @@
         <v>11</v>
       </c>
       <c r="G131" s="16" t="s">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="H131" s="17"/>
     </row>
     <row r="132" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B132" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/satisfiability-of-equality-equations/", "990")</f>
@@ -4904,13 +4934,13 @@
         <v>11</v>
       </c>
       <c r="G132" s="9" t="s">
-        <v>185</v>
+        <v>191</v>
       </c>
       <c r="H132" s="10"/>
     </row>
     <row r="133" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="11" t="s">
-        <v>180</v>
+        <v>186</v>
       </c>
       <c r="B133" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/smallest-string-with-swaps/", "1202")</f>
@@ -4930,13 +4960,13 @@
         <v>11</v>
       </c>
       <c r="G133" s="16" t="s">
-        <v>186</v>
+        <v>192</v>
       </c>
       <c r="H133" s="17"/>
     </row>
     <row r="134" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B134" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/network-delay-time/", "743")</f>
@@ -4956,13 +4986,13 @@
         <v>11</v>
       </c>
       <c r="G134" s="9" t="s">
-        <v>188</v>
+        <v>194</v>
       </c>
       <c r="H134" s="10"/>
     </row>
     <row r="135" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="11" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B135" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/cheapest-flights-within-k-stops/", "787")</f>
@@ -4982,13 +5012,13 @@
         <v>11</v>
       </c>
       <c r="G135" s="16" t="s">
-        <v>189</v>
+        <v>195</v>
       </c>
       <c r="H135" s="17"/>
     </row>
     <row r="136" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B136" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-probability/", "1514")</f>
@@ -5008,13 +5038,13 @@
         <v>11</v>
       </c>
       <c r="G136" s="9" t="s">
-        <v>190</v>
+        <v>196</v>
       </c>
       <c r="H136" s="10"/>
     </row>
     <row r="137" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="11" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B137" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-minimum-effort/", "1631")</f>
@@ -5034,13 +5064,13 @@
         <v>11</v>
       </c>
       <c r="G137" s="16" t="s">
-        <v>191</v>
+        <v>197</v>
       </c>
       <c r="H137" s="17"/>
     </row>
     <row r="138" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B138" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/", "1334")</f>
@@ -5060,13 +5090,13 @@
         <v>11</v>
       </c>
       <c r="G138" s="9" t="s">
-        <v>192</v>
+        <v>198</v>
       </c>
       <c r="H138" s="10"/>
     </row>
     <row r="139" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="11" t="s">
-        <v>187</v>
+        <v>193</v>
       </c>
       <c r="B139" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-ways-to-arrive-at-destination/", "1976")</f>
@@ -5086,13 +5116,13 @@
         <v>11</v>
       </c>
       <c r="G139" s="16" t="s">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="H139" s="17"/>
     </row>
     <row r="140" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B140" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/min-cost-to-connect-all-points/", "1584")</f>
@@ -5112,13 +5142,13 @@
         <v>11</v>
       </c>
       <c r="G140" s="9" t="s">
-        <v>195</v>
+        <v>201</v>
       </c>
       <c r="H140" s="10"/>
     </row>
     <row r="141" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="11" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B141" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/connecting-cities-with-minimum-cost/", "1135")</f>
@@ -5138,15 +5168,15 @@
         <v>11</v>
       </c>
       <c r="G141" s="16" t="s">
-        <v>196</v>
+        <v>202</v>
       </c>
       <c r="H141" s="21" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B142" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/optimize-water-distribution-in-a-village/", "1168")</f>
@@ -5166,15 +5196,15 @@
         <v>11</v>
       </c>
       <c r="G142" s="9" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
       <c r="H142" s="20" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="11" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B143" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-critical-and-pseudo-critical-edges-in-minimum-spanning-tree/", "1489")</f>
@@ -5194,13 +5224,13 @@
         <v>11</v>
       </c>
       <c r="G143" s="16" t="s">
-        <v>198</v>
+        <v>204</v>
       </c>
       <c r="H143" s="17"/>
     </row>
     <row r="144" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B144" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swim-in-rising-water/", "778")</f>
@@ -5220,13 +5250,13 @@
         <v>11</v>
       </c>
       <c r="G144" s="9" t="s">
-        <v>199</v>
+        <v>205</v>
       </c>
       <c r="H144" s="10"/>
     </row>
     <row r="145" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="11" t="s">
-        <v>194</v>
+        <v>200</v>
       </c>
       <c r="B145" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-minimum-value/", "1102")</f>
@@ -5246,15 +5276,15 @@
         <v>11</v>
       </c>
       <c r="G145" s="16" t="s">
-        <v>200</v>
+        <v>206</v>
       </c>
       <c r="H145" s="21" t="s">
-        <v>84</v>
+        <v>90</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B146" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/implement-trie-prefix-tree/", "208")</f>
@@ -5274,13 +5304,13 @@
         <v>11</v>
       </c>
       <c r="G146" s="9" t="s">
-        <v>202</v>
+        <v>208</v>
       </c>
       <c r="H146" s="10"/>
     </row>
     <row r="147" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="11" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B147" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/design-add-and-search-words-data-structure/", "211")</f>
@@ -5300,13 +5330,13 @@
         <v>11</v>
       </c>
       <c r="G147" s="16" t="s">
-        <v>203</v>
+        <v>209</v>
       </c>
       <c r="H147" s="17"/>
     </row>
     <row r="148" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B148" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search-ii/", "212")</f>
@@ -5326,13 +5356,13 @@
         <v>11</v>
       </c>
       <c r="G148" s="9" t="s">
-        <v>204</v>
+        <v>210</v>
       </c>
       <c r="H148" s="10"/>
     </row>
     <row r="149" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B149" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/replace-words/", "648")</f>
@@ -5352,13 +5382,13 @@
         <v>11</v>
       </c>
       <c r="G149" s="16" t="s">
-        <v>205</v>
+        <v>211</v>
       </c>
       <c r="H149" s="17"/>
     </row>
     <row r="150" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B150" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/map-sum-pairs/", "677")</f>
@@ -5378,13 +5408,13 @@
         <v>11</v>
       </c>
       <c r="G150" s="9" t="s">
-        <v>206</v>
+        <v>212</v>
       </c>
       <c r="H150" s="10"/>
     </row>
     <row r="151" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="11" t="s">
-        <v>201</v>
+        <v>207</v>
       </c>
       <c r="B151" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-suggestions-system/", "1268")</f>
@@ -5404,13 +5434,13 @@
         <v>11</v>
       </c>
       <c r="G151" s="16" t="s">
-        <v>207</v>
+        <v>213</v>
       </c>
       <c r="H151" s="17"/>
     </row>
     <row r="152" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B152" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number/", "136")</f>
@@ -5430,13 +5460,13 @@
         <v>11</v>
       </c>
       <c r="G152" s="9" t="s">
-        <v>209</v>
+        <v>215</v>
       </c>
       <c r="H152" s="10"/>
     </row>
     <row r="153" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="11" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B153" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number-ii/", "137")</f>
@@ -5456,13 +5486,13 @@
         <v>11</v>
       </c>
       <c r="G153" s="16" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="H153" s="17"/>
     </row>
     <row r="154" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B154" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-1-bits/", "191")</f>
@@ -5482,13 +5512,13 @@
         <v>11</v>
       </c>
       <c r="G154" s="9" t="s">
-        <v>211</v>
+        <v>217</v>
       </c>
       <c r="H154" s="10"/>
     </row>
     <row r="155" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="11" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B155" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/counting-bits/", "338")</f>
@@ -5508,13 +5538,13 @@
         <v>11</v>
       </c>
       <c r="G155" s="16" t="s">
-        <v>212</v>
+        <v>218</v>
       </c>
       <c r="H155" s="17"/>
     </row>
     <row r="156" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B156" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/missing-number/", "268")</f>
@@ -5534,13 +5564,13 @@
         <v>11</v>
       </c>
       <c r="G156" s="9" t="s">
-        <v>213</v>
+        <v>219</v>
       </c>
       <c r="H156" s="10"/>
     </row>
     <row r="157" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="11" t="s">
-        <v>208</v>
+        <v>214</v>
       </c>
       <c r="B157" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-bits/", "190")</f>
@@ -5560,13 +5590,13 @@
         <v>11</v>
       </c>
       <c r="G157" s="16" t="s">
-        <v>214</v>
+        <v>220</v>
       </c>
       <c r="H157" s="17"/>
     </row>
     <row r="158" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B158" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/climbing-stairs/", "70")</f>
@@ -5586,13 +5616,13 @@
         <v>11</v>
       </c>
       <c r="G158" s="9" t="s">
-        <v>216</v>
+        <v>222</v>
       </c>
       <c r="H158" s="10"/>
     </row>
     <row r="159" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="11" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B159" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber/", "198")</f>
@@ -5612,13 +5642,13 @@
         <v>11</v>
       </c>
       <c r="G159" s="16" t="s">
-        <v>217</v>
+        <v>223</v>
       </c>
       <c r="H159" s="17"/>
     </row>
     <row r="160" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B160" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber-ii/", "213")</f>
@@ -5638,13 +5668,13 @@
         <v>11</v>
       </c>
       <c r="G160" s="9" t="s">
-        <v>218</v>
+        <v>224</v>
       </c>
       <c r="H160" s="10"/>
     </row>
     <row r="161" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="11" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B161" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change/", "322")</f>
@@ -5664,13 +5694,13 @@
         <v>11</v>
       </c>
       <c r="G161" s="16" t="s">
-        <v>219</v>
+        <v>225</v>
       </c>
       <c r="H161" s="17"/>
     </row>
     <row r="162" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B162" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/perfect-squares/", "279")</f>
@@ -5690,13 +5720,13 @@
         <v>11</v>
       </c>
       <c r="G162" s="9" t="s">
-        <v>220</v>
+        <v>226</v>
       </c>
       <c r="H162" s="10"/>
     </row>
     <row r="163" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="11" t="s">
-        <v>215</v>
+        <v>221</v>
       </c>
       <c r="B163" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-increasing-subsequence/", "300")</f>
@@ -5716,13 +5746,13 @@
         <v>11</v>
       </c>
       <c r="G163" s="16" t="s">
-        <v>221</v>
+        <v>227</v>
       </c>
       <c r="H163" s="17"/>
     </row>
     <row r="164" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B164" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-equal-subset-sum/", "416")</f>
@@ -5742,13 +5772,13 @@
         <v>11</v>
       </c>
       <c r="G164" s="9" t="s">
-        <v>223</v>
+        <v>229</v>
       </c>
       <c r="H164" s="10"/>
     </row>
     <row r="165" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="11" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B165" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/target-sum/", "494")</f>
@@ -5768,13 +5798,13 @@
         <v>11</v>
       </c>
       <c r="G165" s="16" t="s">
-        <v>224</v>
+        <v>230</v>
       </c>
       <c r="H165" s="17"/>
     </row>
     <row r="166" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B166" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change-ii/", "518")</f>
@@ -5794,13 +5824,13 @@
         <v>11</v>
       </c>
       <c r="G166" s="9" t="s">
-        <v>225</v>
+        <v>231</v>
       </c>
       <c r="H166" s="10"/>
     </row>
     <row r="167" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="11" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B167" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/ones-and-zeroes/", "474")</f>
@@ -5820,13 +5850,13 @@
         <v>11</v>
       </c>
       <c r="G167" s="16" t="s">
-        <v>226</v>
+        <v>232</v>
       </c>
       <c r="H167" s="17"/>
     </row>
     <row r="168" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="3" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B168" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight-ii/", "1049")</f>
@@ -5846,13 +5876,13 @@
         <v>11</v>
       </c>
       <c r="G168" s="9" t="s">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="H168" s="10"/>
     </row>
     <row r="169" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="11" t="s">
-        <v>222</v>
+        <v>228</v>
       </c>
       <c r="B169" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/profitable-schemes/", "879")</f>
@@ -5872,13 +5902,13 @@
         <v>11</v>
       </c>
       <c r="G169" s="16" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
       <c r="H169" s="17"/>
     </row>
     <row r="170" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="3" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B170" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths/", "62")</f>
@@ -5898,13 +5928,13 @@
         <v>11</v>
       </c>
       <c r="G170" s="9" t="s">
-        <v>230</v>
+        <v>236</v>
       </c>
       <c r="H170" s="10"/>
     </row>
     <row r="171" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B171" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths-ii/", "63")</f>
@@ -5924,13 +5954,13 @@
         <v>11</v>
       </c>
       <c r="G171" s="16" t="s">
-        <v>231</v>
+        <v>237</v>
       </c>
       <c r="H171" s="17"/>
     </row>
     <row r="172" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="3" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B172" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-path-sum/", "64")</f>
@@ -5950,13 +5980,13 @@
         <v>11</v>
       </c>
       <c r="G172" s="9" t="s">
-        <v>232</v>
+        <v>238</v>
       </c>
       <c r="H172" s="10"/>
     </row>
     <row r="173" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="11" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B173" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-square/", "221")</f>
@@ -5976,13 +6006,13 @@
         <v>11</v>
       </c>
       <c r="G173" s="16" t="s">
-        <v>233</v>
+        <v>239</v>
       </c>
       <c r="H173" s="17"/>
     </row>
     <row r="174" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B174" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-falling-path-sum/", "931")</f>
@@ -6002,13 +6032,13 @@
         <v>11</v>
       </c>
       <c r="G174" s="9" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="H174" s="10"/>
     </row>
     <row r="175" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="11" t="s">
-        <v>229</v>
+        <v>235</v>
       </c>
       <c r="B175" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/triangle/", "120")</f>
@@ -6028,13 +6058,13 @@
         <v>11</v>
       </c>
       <c r="G175" s="16" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="H175" s="17"/>
     </row>
     <row r="176" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="3" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B176" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-common-subsequence/", "1143")</f>
@@ -6054,13 +6084,13 @@
         <v>11</v>
       </c>
       <c r="G176" s="9" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="H176" s="10"/>
     </row>
     <row r="177" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="11" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B177" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/edit-distance/", "72")</f>
@@ -6080,13 +6110,13 @@
         <v>11</v>
       </c>
       <c r="G177" s="16" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="H177" s="17"/>
     </row>
     <row r="178" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="3" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B178" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/distinct-subsequences/", "115")</f>
@@ -6106,13 +6136,13 @@
         <v>11</v>
       </c>
       <c r="G178" s="9" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="H178" s="10"/>
     </row>
     <row r="179" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="11" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B179" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-operation-for-two-strings/", "583")</f>
@@ -6132,13 +6162,13 @@
         <v>11</v>
       </c>
       <c r="G179" s="16" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="H179" s="17"/>
     </row>
     <row r="180" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="3" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B180" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/interleaving-string/", "97")</f>
@@ -6158,13 +6188,13 @@
         <v>11</v>
       </c>
       <c r="G180" s="9" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="H180" s="10"/>
     </row>
     <row r="181" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="11" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="B181" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-insertion-steps-to-make-a-string-palindrome/", "1312")</f>
@@ -6184,7 +6214,7 @@
         <v>11</v>
       </c>
       <c r="G181" s="16" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="H181" s="17"/>
     </row>

</xml_diff>

<commit_message>
solved prefix sum problems and 1 diff array problem.
</commit_message>
<xml_diff>
--- a/leetcode_roadmap.xlsx
+++ b/leetcode_roadmap.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="249">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="254">
   <si>
     <t xml:space="preserve">Category</t>
   </si>
@@ -274,15 +274,27 @@
     <t xml:space="preserve">https://leetcode.com/problems/range-sum-query-immutable/</t>
   </si>
   <si>
+    <t xml:space="preserve">create prefix sum array. Simple arithmetic right after</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/subarray-sum-equals-k/</t>
   </si>
   <si>
+    <t xml:space="preserve">should be categorized as hard. Calculcate prefix sum simultaneously with calculating the number of subarrays (use hashmap).</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/find-pivot-index/</t>
   </si>
   <si>
+    <t xml:space="preserve">calculate forward and backward prefix sums</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/binary-subarrays-with-sum/</t>
   </si>
   <si>
+    <t xml:space="preserve">same solution as “subarray sum equal to k” problem. But can also be solved using sliding window</t>
+  </si>
+  <si>
     <t xml:space="preserve">https://leetcode.com/problems/subarray-sums-divisible-by-k/</t>
   </si>
   <si>
@@ -305,6 +317,9 @@
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/check-if-all-the-integers-in-a-range-are-covered/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difference sum is little tricky but useful once you get it. Remember the analogy of boarding and leaving a bus at different stops.</t>
   </si>
   <si>
     <t xml:space="preserve">https://leetcode.com/problems/describe-the-painting/</t>
@@ -2477,8 +2492,8 @@
       <c r="D38" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E38" s="8" t="s">
-        <v>11</v>
+      <c r="E38" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F38" s="8" t="s">
         <v>11</v>
@@ -2486,7 +2501,9 @@
       <c r="G38" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="H38" s="10"/>
+      <c r="H38" s="10" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="11" t="s">
@@ -2503,16 +2520,18 @@
       <c r="D39" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E39" s="15" t="s">
-        <v>11</v>
+      <c r="E39" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F39" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G39" s="16" t="s">
-        <v>83</v>
-      </c>
-      <c r="H39" s="17"/>
+        <v>84</v>
+      </c>
+      <c r="H39" s="17" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="3" t="s">
@@ -2529,16 +2548,18 @@
       <c r="D40" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E40" s="8" t="s">
-        <v>11</v>
+      <c r="E40" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F40" s="8" t="s">
         <v>11</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>84</v>
-      </c>
-      <c r="H40" s="10"/>
+        <v>86</v>
+      </c>
+      <c r="H40" s="10" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="s">
@@ -2555,16 +2576,18 @@
       <c r="D41" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="E41" s="15" t="s">
-        <v>11</v>
+      <c r="E41" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F41" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G41" s="16" t="s">
-        <v>85</v>
-      </c>
-      <c r="H41" s="17"/>
+        <v>88</v>
+      </c>
+      <c r="H41" s="17" t="s">
+        <v>89</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="3" t="s">
@@ -2588,7 +2611,7 @@
         <v>11</v>
       </c>
       <c r="G42" s="9" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="H42" s="10"/>
     </row>
@@ -2614,13 +2637,13 @@
         <v>11</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="H43" s="17"/>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B44" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/range-addition/", "370")</f>
@@ -2640,15 +2663,15 @@
         <v>11</v>
       </c>
       <c r="G44" s="9" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="H44" s="20" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B45" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/car-pooling/", "1094")</f>
@@ -2668,13 +2691,13 @@
         <v>11</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="H45" s="17"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B46" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/corporate-flight-bookings/", "1109")</f>
@@ -2694,13 +2717,13 @@
         <v>11</v>
       </c>
       <c r="G46" s="9" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="H46" s="10"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="11" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B47" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/check-if-all-the-integers-in-a-range-are-covered/", "1893")</f>
@@ -2713,20 +2736,22 @@
       <c r="D47" s="18" t="s">
         <v>35</v>
       </c>
-      <c r="E47" s="15" t="s">
-        <v>11</v>
+      <c r="E47" s="7" t="s">
+        <v>10</v>
       </c>
       <c r="F47" s="15" t="s">
         <v>11</v>
       </c>
       <c r="G47" s="16" t="s">
-        <v>93</v>
-      </c>
-      <c r="H47" s="17"/>
+        <v>97</v>
+      </c>
+      <c r="H47" s="17" t="s">
+        <v>98</v>
+      </c>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B48" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/describe-the-painting/", "1943")</f>
@@ -2746,13 +2771,13 @@
         <v>11</v>
       </c>
       <c r="G48" s="9" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="H48" s="10"/>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="11" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="B49" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shifting-letters-ii/", "2381")</f>
@@ -2772,13 +2797,13 @@
         <v>11</v>
       </c>
       <c r="G49" s="16" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="H49" s="17"/>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B50" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/daily-temperatures/", "739")</f>
@@ -2798,13 +2823,13 @@
         <v>11</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="H50" s="10"/>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B51" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-i/", "496")</f>
@@ -2824,13 +2849,13 @@
         <v>11</v>
       </c>
       <c r="G51" s="16" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="H51" s="17"/>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B52" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/next-greater-element-ii/", "503")</f>
@@ -2850,13 +2875,13 @@
         <v>11</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="H52" s="10"/>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B53" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/largest-rectangle-in-histogram/", "84")</f>
@@ -2876,13 +2901,13 @@
         <v>11</v>
       </c>
       <c r="G53" s="16" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="H53" s="17"/>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="3" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B54" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-rectangle/", "85")</f>
@@ -2902,13 +2927,13 @@
         <v>11</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="H54" s="10"/>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B55" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/online-stock-span/", "901")</f>
@@ -2928,13 +2953,13 @@
         <v>11</v>
       </c>
       <c r="G55" s="16" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="H55" s="17"/>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B56" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sliding-window-maximum/", "239")</f>
@@ -2954,13 +2979,13 @@
         <v>11</v>
       </c>
       <c r="G56" s="9" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="H56" s="10"/>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B57" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-subarray-with-sum-at-least-k/", "862")</f>
@@ -2980,13 +3005,13 @@
         <v>11</v>
       </c>
       <c r="G57" s="16" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="H57" s="17"/>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B58" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/constrained-subsequence-sum/", "1425")</f>
@@ -3006,13 +3031,13 @@
         <v>11</v>
       </c>
       <c r="G58" s="9" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="H58" s="10"/>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B59" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-continuous-subarray-with-absolute-diff-less-than-or-equal-to-limit/", "1438")</f>
@@ -3032,13 +3057,13 @@
         <v>11</v>
       </c>
       <c r="G59" s="16" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="H59" s="17"/>
     </row>
     <row r="60" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="3" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B60" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-value-of-equation/", "1499")</f>
@@ -3058,13 +3083,13 @@
         <v>11</v>
       </c>
       <c r="G60" s="9" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="H60" s="10"/>
     </row>
     <row r="61" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B61" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-vi/", "1696")</f>
@@ -3084,13 +3109,13 @@
         <v>11</v>
       </c>
       <c r="G61" s="16" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="H61" s="17"/>
     </row>
     <row r="62" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B62" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-an-array/", "215")</f>
@@ -3110,13 +3135,13 @@
         <v>11</v>
       </c>
       <c r="G62" s="9" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="H62" s="10"/>
     </row>
     <row r="63" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B63" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-elements/", "347")</f>
@@ -3142,7 +3167,7 @@
     </row>
     <row r="64" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B64" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/top-k-frequent-words/", "692")</f>
@@ -3162,13 +3187,13 @@
         <v>11</v>
       </c>
       <c r="G64" s="9" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="H64" s="10"/>
     </row>
     <row r="65" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B65" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-largest-element-in-a-stream/", "703")</f>
@@ -3188,13 +3213,13 @@
         <v>11</v>
       </c>
       <c r="G65" s="16" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="H65" s="17"/>
     </row>
     <row r="66" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="3" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B66" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/k-closest-points-to-origin/", "973")</f>
@@ -3214,13 +3239,13 @@
         <v>11</v>
       </c>
       <c r="G66" s="9" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="H66" s="10"/>
     </row>
     <row r="67" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="11" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B67" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight/", "1046")</f>
@@ -3240,13 +3265,13 @@
         <v>11</v>
       </c>
       <c r="G67" s="16" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="H67" s="17"/>
     </row>
     <row r="68" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B68" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-intervals/", "56")</f>
@@ -3266,13 +3291,13 @@
         <v>11</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="H68" s="10"/>
     </row>
     <row r="69" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="11" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B69" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/insert-interval/", "57")</f>
@@ -3292,13 +3317,13 @@
         <v>11</v>
       </c>
       <c r="G69" s="16" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="H69" s="17"/>
     </row>
     <row r="70" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B70" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms/", "252")</f>
@@ -3318,15 +3343,15 @@
         <v>11</v>
       </c>
       <c r="G70" s="9" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="H70" s="20" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="71" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="11" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B71" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/meeting-rooms-ii/", "253")</f>
@@ -3346,15 +3371,15 @@
         <v>11</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="H71" s="21" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="72" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="3" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B72" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/non-overlapping-intervals/", "435")</f>
@@ -3374,13 +3399,13 @@
         <v>11</v>
       </c>
       <c r="G72" s="9" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="H72" s="10"/>
     </row>
     <row r="73" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="11" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B73" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-number-of-arrows-to-burst-balloons/", "452")</f>
@@ -3400,13 +3425,13 @@
         <v>11</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="H73" s="17"/>
     </row>
     <row r="74" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="3" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B74" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game-ii/", "45")</f>
@@ -3426,13 +3451,13 @@
         <v>11</v>
       </c>
       <c r="G74" s="9" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="H74" s="10"/>
     </row>
     <row r="75" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="11" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B75" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/jump-game/", "55")</f>
@@ -3452,13 +3477,13 @@
         <v>11</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="H75" s="17"/>
     </row>
     <row r="76" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="3" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B76" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/queue-reconstruction-by-height/", "406")</f>
@@ -3478,13 +3503,13 @@
         <v>11</v>
       </c>
       <c r="G76" s="9" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="H76" s="10"/>
     </row>
     <row r="77" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="11" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B77" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/task-scheduler/", "621")</f>
@@ -3504,13 +3529,13 @@
         <v>11</v>
       </c>
       <c r="G77" s="16" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="H77" s="17"/>
     </row>
     <row r="78" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="3" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B78" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-labels/", "763")</f>
@@ -3530,13 +3555,13 @@
         <v>11</v>
       </c>
       <c r="G78" s="9" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="H78" s="10"/>
     </row>
     <row r="79" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="11" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B79" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/gas-station/", "134")</f>
@@ -3556,13 +3581,13 @@
         <v>11</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="H79" s="17"/>
     </row>
     <row r="80" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="3" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B80" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-two-sorted-lists/", "21")</f>
@@ -3582,13 +3607,13 @@
         <v>11</v>
       </c>
       <c r="G80" s="9" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="H80" s="10"/>
     </row>
     <row r="81" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="11" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B81" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/merge-k-sorted-lists/", "23")</f>
@@ -3608,13 +3633,13 @@
         <v>11</v>
       </c>
       <c r="G81" s="16" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="H81" s="17"/>
     </row>
     <row r="82" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="3" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B82" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swap-nodes-in-pairs/", "24")</f>
@@ -3634,13 +3659,13 @@
         <v>11</v>
       </c>
       <c r="G82" s="9" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="H82" s="10"/>
     </row>
     <row r="83" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="11" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B83" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-nodes-in-k-group/", "25")</f>
@@ -3660,13 +3685,13 @@
         <v>11</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="H83" s="17"/>
     </row>
     <row r="84" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="3" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B84" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-linked-list-ii/", "92")</f>
@@ -3686,13 +3711,13 @@
         <v>11</v>
       </c>
       <c r="G84" s="9" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="H84" s="10"/>
     </row>
     <row r="85" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="11" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="B85" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/copy-list-with-random-pointer/", "138")</f>
@@ -3712,13 +3737,13 @@
         <v>11</v>
       </c>
       <c r="G85" s="16" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="H85" s="17"/>
     </row>
     <row r="86" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B86" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximum-depth-of-binary-tree/", "104")</f>
@@ -3738,13 +3763,13 @@
         <v>11</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="H86" s="10"/>
     </row>
     <row r="87" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="11" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B87" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum/", "112")</f>
@@ -3764,13 +3789,13 @@
         <v>11</v>
       </c>
       <c r="G87" s="16" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="H87" s="17"/>
     </row>
     <row r="88" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B88" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-sum-ii/", "113")</f>
@@ -3790,13 +3815,13 @@
         <v>11</v>
       </c>
       <c r="G88" s="9" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="H88" s="10"/>
     </row>
     <row r="89" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="11" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B89" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/diameter-of-binary-tree/", "543")</f>
@@ -3816,13 +3841,13 @@
         <v>11</v>
       </c>
       <c r="G89" s="16" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="H89" s="17"/>
     </row>
     <row r="90" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="3" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B90" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-maximum-path-sum/", "124")</f>
@@ -3842,13 +3867,13 @@
         <v>11</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="H90" s="10"/>
     </row>
     <row r="91" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="11" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B91" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/invert-binary-tree/", "226")</f>
@@ -3868,13 +3893,13 @@
         <v>11</v>
       </c>
       <c r="G91" s="16" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="H91" s="17"/>
     </row>
     <row r="92" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B92" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-level-order-traversal/", "102")</f>
@@ -3894,13 +3919,13 @@
         <v>11</v>
       </c>
       <c r="G92" s="9" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="H92" s="10"/>
     </row>
     <row r="93" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="11" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B93" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-zigzag-level-order-traversal/", "103")</f>
@@ -3920,13 +3945,13 @@
         <v>11</v>
       </c>
       <c r="G93" s="16" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="H93" s="17"/>
     </row>
     <row r="94" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B94" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/binary-tree-right-side-view/", "199")</f>
@@ -3946,13 +3971,13 @@
         <v>11</v>
       </c>
       <c r="G94" s="9" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="H94" s="10"/>
     </row>
     <row r="95" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="11" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B95" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-largest-value-in-each-tree-row/", "515")</f>
@@ -3972,13 +3997,13 @@
         <v>11</v>
       </c>
       <c r="G95" s="16" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="H95" s="17"/>
     </row>
     <row r="96" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="3" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B96" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/average-of-levels-in-binary-tree/", "637")</f>
@@ -3998,13 +4023,13 @@
         <v>11</v>
       </c>
       <c r="G96" s="9" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="H96" s="10"/>
     </row>
     <row r="97" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="11" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B97" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/populating-next-right-pointers-in-each-node/", "116")</f>
@@ -4024,13 +4049,13 @@
         <v>11</v>
       </c>
       <c r="G97" s="16" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="H97" s="17"/>
     </row>
     <row r="98" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="3" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B98" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/validate-binary-search-tree/", "98")</f>
@@ -4050,13 +4075,13 @@
         <v>11</v>
       </c>
       <c r="G98" s="9" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="H98" s="10"/>
     </row>
     <row r="99" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="11" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B99" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/recover-binary-search-tree/", "99")</f>
@@ -4076,13 +4101,13 @@
         <v>11</v>
       </c>
       <c r="G99" s="16" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="H99" s="17"/>
     </row>
     <row r="100" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="3" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B100" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/kth-smallest-element-in-a-bst/", "230")</f>
@@ -4102,13 +4127,13 @@
         <v>11</v>
       </c>
       <c r="G100" s="9" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="H100" s="10"/>
     </row>
     <row r="101" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="11" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B101" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/lowest-common-ancestor-of-a-binary-search-tree/", "235")</f>
@@ -4128,13 +4153,13 @@
         <v>11</v>
       </c>
       <c r="G101" s="16" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
       <c r="H101" s="17"/>
     </row>
     <row r="102" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="3" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B102" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-node-in-a-bst/", "450")</f>
@@ -4154,13 +4179,13 @@
         <v>11</v>
       </c>
       <c r="G102" s="9" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
       <c r="H102" s="10"/>
     </row>
     <row r="103" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="11" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="B103" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-in-a-binary-search-tree/", "700")</f>
@@ -4180,13 +4205,13 @@
         <v>11</v>
       </c>
       <c r="G103" s="16" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
       <c r="H103" s="17"/>
     </row>
     <row r="104" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="3" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B104" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations/", "46")</f>
@@ -4206,13 +4231,13 @@
         <v>11</v>
       </c>
       <c r="G104" s="9" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="H104" s="10"/>
     </row>
     <row r="105" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="11" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B105" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/permutations-ii/", "47")</f>
@@ -4232,13 +4257,13 @@
         <v>11</v>
       </c>
       <c r="G105" s="16" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="H105" s="17"/>
     </row>
     <row r="106" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="3" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B106" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combinations/", "77")</f>
@@ -4258,13 +4283,13 @@
         <v>11</v>
       </c>
       <c r="G106" s="9" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="H106" s="10"/>
     </row>
     <row r="107" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="11" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B107" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets/", "78")</f>
@@ -4284,13 +4309,13 @@
         <v>11</v>
       </c>
       <c r="G107" s="16" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="H107" s="17"/>
     </row>
     <row r="108" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="3" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B108" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/subsets-ii/", "90")</f>
@@ -4310,13 +4335,13 @@
         <v>11</v>
       </c>
       <c r="G108" s="9" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="H108" s="10"/>
     </row>
     <row r="109" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="11" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B109" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum/", "39")</f>
@@ -4336,13 +4361,13 @@
         <v>11</v>
       </c>
       <c r="G109" s="16" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="H109" s="17"/>
     </row>
     <row r="110" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="3" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B110" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/combination-sum-ii/", "40")</f>
@@ -4362,13 +4387,13 @@
         <v>11</v>
       </c>
       <c r="G110" s="9" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="H110" s="10"/>
     </row>
     <row r="111" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="11" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B111" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/letter-combinations-of-a-phone-number/", "17")</f>
@@ -4388,13 +4413,13 @@
         <v>11</v>
       </c>
       <c r="G111" s="16" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="H111" s="17"/>
     </row>
     <row r="112" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="3" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B112" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search/", "79")</f>
@@ -4414,13 +4439,13 @@
         <v>11</v>
       </c>
       <c r="G112" s="9" t="s">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="H112" s="10"/>
     </row>
     <row r="113" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="11" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B113" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/palindrome-partitioning/", "131")</f>
@@ -4440,13 +4465,13 @@
         <v>11</v>
       </c>
       <c r="G113" s="16" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="H113" s="17"/>
     </row>
     <row r="114" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="3" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B114" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens/", "51")</f>
@@ -4466,13 +4491,13 @@
         <v>11</v>
       </c>
       <c r="G114" s="9" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="H114" s="10"/>
     </row>
     <row r="115" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="11" t="s">
-        <v>165</v>
+        <v>170</v>
       </c>
       <c r="B115" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/n-queens-ii/", "52")</f>
@@ -4492,13 +4517,13 @@
         <v>11</v>
       </c>
       <c r="G115" s="16" t="s">
-        <v>171</v>
+        <v>176</v>
       </c>
       <c r="H115" s="17"/>
     </row>
     <row r="116" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="3" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B116" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-islands/", "200")</f>
@@ -4518,13 +4543,13 @@
         <v>11</v>
       </c>
       <c r="G116" s="9" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="H116" s="10"/>
     </row>
     <row r="117" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="11" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B117" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/max-area-of-island/", "695")</f>
@@ -4544,13 +4569,13 @@
         <v>11</v>
       </c>
       <c r="G117" s="16" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="H117" s="17"/>
     </row>
     <row r="118" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="3" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B118" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/flood-fill/", "733")</f>
@@ -4570,13 +4595,13 @@
         <v>11</v>
       </c>
       <c r="G118" s="9" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="H118" s="10"/>
     </row>
     <row r="119" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="11" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B119" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/rotting-oranges/", "994")</f>
@@ -4596,13 +4621,13 @@
         <v>11</v>
       </c>
       <c r="G119" s="16" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="H119" s="17"/>
     </row>
     <row r="120" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="3" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B120" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/shortest-path-in-binary-matrix/", "1091")</f>
@@ -4622,13 +4647,13 @@
         <v>11</v>
       </c>
       <c r="G120" s="9" t="s">
-        <v>177</v>
+        <v>182</v>
       </c>
       <c r="H120" s="10"/>
     </row>
     <row r="121" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="11" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="B121" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-closed-islands/", "1254")</f>
@@ -4648,13 +4673,13 @@
         <v>11</v>
       </c>
       <c r="G121" s="16" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="H121" s="17"/>
     </row>
     <row r="122" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B122" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule/", "207")</f>
@@ -4674,13 +4699,13 @@
         <v>11</v>
       </c>
       <c r="G122" s="9" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="H122" s="10"/>
     </row>
     <row r="123" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="11" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B123" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-ii/", "210")</f>
@@ -4700,13 +4725,13 @@
         <v>11</v>
       </c>
       <c r="G123" s="16" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="H123" s="17"/>
     </row>
     <row r="124" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A124" s="3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B124" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-eventual-safe-states/", "802")</f>
@@ -4726,13 +4751,13 @@
         <v>11</v>
       </c>
       <c r="G124" s="9" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
       <c r="H124" s="10"/>
     </row>
     <row r="125" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A125" s="11" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B125" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/course-schedule-iv/", "1462")</f>
@@ -4752,13 +4777,13 @@
         <v>11</v>
       </c>
       <c r="G125" s="16" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="H125" s="17"/>
     </row>
     <row r="126" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A126" s="3" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B126" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/sort-items-by-groups-respecting-dependencies/", "1203")</f>
@@ -4778,13 +4803,13 @@
         <v>11</v>
       </c>
       <c r="G126" s="9" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="H126" s="10"/>
     </row>
     <row r="127" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A127" s="11" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="B127" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-all-possible-recipes-from-given-supplies/", "2115")</f>
@@ -4804,13 +4829,13 @@
         <v>11</v>
       </c>
       <c r="G127" s="16" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="H127" s="17"/>
     </row>
     <row r="128" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A128" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B128" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-provinces/", "547")</f>
@@ -4830,13 +4855,13 @@
         <v>11</v>
       </c>
       <c r="G128" s="9" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
       <c r="H128" s="10"/>
     </row>
     <row r="129" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A129" s="11" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B129" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/redundant-connection/", "684")</f>
@@ -4856,13 +4881,13 @@
         <v>11</v>
       </c>
       <c r="G129" s="16" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="H129" s="17"/>
     </row>
     <row r="130" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A130" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B130" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-operations-to-make-network-connected/", "1319")</f>
@@ -4882,13 +4907,13 @@
         <v>11</v>
       </c>
       <c r="G130" s="9" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="H130" s="10"/>
     </row>
     <row r="131" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A131" s="11" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B131" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/remove-max-number-of-edges-to-keep-graph-fully-traversable/", "1579")</f>
@@ -4908,13 +4933,13 @@
         <v>11</v>
       </c>
       <c r="G131" s="16" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="H131" s="17"/>
     </row>
     <row r="132" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A132" s="3" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B132" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/satisfiability-of-equality-equations/", "990")</f>
@@ -4934,13 +4959,13 @@
         <v>11</v>
       </c>
       <c r="G132" s="9" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="H132" s="10"/>
     </row>
     <row r="133" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A133" s="11" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="B133" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/smallest-string-with-swaps/", "1202")</f>
@@ -4960,13 +4985,13 @@
         <v>11</v>
       </c>
       <c r="G133" s="16" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="H133" s="17"/>
     </row>
     <row r="134" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A134" s="3" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B134" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/network-delay-time/", "743")</f>
@@ -4986,13 +5011,13 @@
         <v>11</v>
       </c>
       <c r="G134" s="9" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="H134" s="10"/>
     </row>
     <row r="135" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A135" s="11" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B135" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/cheapest-flights-within-k-stops/", "787")</f>
@@ -5012,13 +5037,13 @@
         <v>11</v>
       </c>
       <c r="G135" s="16" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="H135" s="17"/>
     </row>
     <row r="136" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A136" s="3" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B136" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-probability/", "1514")</f>
@@ -5038,13 +5063,13 @@
         <v>11</v>
       </c>
       <c r="G136" s="9" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="H136" s="10"/>
     </row>
     <row r="137" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A137" s="11" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B137" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-minimum-effort/", "1631")</f>
@@ -5064,13 +5089,13 @@
         <v>11</v>
       </c>
       <c r="G137" s="16" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="H137" s="17"/>
     </row>
     <row r="138" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A138" s="3" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B138" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-the-city-with-the-smallest-number-of-neighbors-at-a-threshold-distance/", "1334")</f>
@@ -5090,13 +5115,13 @@
         <v>11</v>
       </c>
       <c r="G138" s="9" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="H138" s="10"/>
     </row>
     <row r="139" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A139" s="11" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="B139" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-ways-to-arrive-at-destination/", "1976")</f>
@@ -5116,13 +5141,13 @@
         <v>11</v>
       </c>
       <c r="G139" s="16" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="H139" s="17"/>
     </row>
     <row r="140" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A140" s="3" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B140" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/min-cost-to-connect-all-points/", "1584")</f>
@@ -5142,13 +5167,13 @@
         <v>11</v>
       </c>
       <c r="G140" s="9" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="H140" s="10"/>
     </row>
     <row r="141" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A141" s="11" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B141" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/connecting-cities-with-minimum-cost/", "1135")</f>
@@ -5168,15 +5193,15 @@
         <v>11</v>
       </c>
       <c r="G141" s="16" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="H141" s="21" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="142" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A142" s="3" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B142" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/optimize-water-distribution-in-a-village/", "1168")</f>
@@ -5196,15 +5221,15 @@
         <v>11</v>
       </c>
       <c r="G142" s="9" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="H142" s="20" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="143" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A143" s="11" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B143" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/find-critical-and-pseudo-critical-edges-in-minimum-spanning-tree/", "1489")</f>
@@ -5224,13 +5249,13 @@
         <v>11</v>
       </c>
       <c r="G143" s="16" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="H143" s="17"/>
     </row>
     <row r="144" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A144" s="3" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B144" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/swim-in-rising-water/", "778")</f>
@@ -5250,13 +5275,13 @@
         <v>11</v>
       </c>
       <c r="G144" s="9" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="H144" s="10"/>
     </row>
     <row r="145" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A145" s="11" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="B145" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/path-with-maximum-minimum-value/", "1102")</f>
@@ -5276,15 +5301,15 @@
         <v>11</v>
       </c>
       <c r="G145" s="16" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="H145" s="21" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
     </row>
     <row r="146" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A146" s="3" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B146" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/implement-trie-prefix-tree/", "208")</f>
@@ -5304,13 +5329,13 @@
         <v>11</v>
       </c>
       <c r="G146" s="9" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="H146" s="10"/>
     </row>
     <row r="147" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A147" s="11" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B147" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/design-add-and-search-words-data-structure/", "211")</f>
@@ -5330,13 +5355,13 @@
         <v>11</v>
       </c>
       <c r="G147" s="16" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="H147" s="17"/>
     </row>
     <row r="148" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A148" s="3" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B148" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/word-search-ii/", "212")</f>
@@ -5356,13 +5381,13 @@
         <v>11</v>
       </c>
       <c r="G148" s="9" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="H148" s="10"/>
     </row>
     <row r="149" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A149" s="11" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B149" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/replace-words/", "648")</f>
@@ -5382,13 +5407,13 @@
         <v>11</v>
       </c>
       <c r="G149" s="16" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="H149" s="17"/>
     </row>
     <row r="150" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A150" s="3" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B150" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/map-sum-pairs/", "677")</f>
@@ -5408,13 +5433,13 @@
         <v>11</v>
       </c>
       <c r="G150" s="9" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="H150" s="10"/>
     </row>
     <row r="151" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A151" s="11" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B151" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/search-suggestions-system/", "1268")</f>
@@ -5434,13 +5459,13 @@
         <v>11</v>
       </c>
       <c r="G151" s="16" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="H151" s="17"/>
     </row>
     <row r="152" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A152" s="3" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B152" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number/", "136")</f>
@@ -5460,13 +5485,13 @@
         <v>11</v>
       </c>
       <c r="G152" s="9" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="H152" s="10"/>
     </row>
     <row r="153" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A153" s="11" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B153" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/single-number-ii/", "137")</f>
@@ -5486,13 +5511,13 @@
         <v>11</v>
       </c>
       <c r="G153" s="16" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="H153" s="17"/>
     </row>
     <row r="154" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A154" s="3" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B154" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/number-of-1-bits/", "191")</f>
@@ -5512,13 +5537,13 @@
         <v>11</v>
       </c>
       <c r="G154" s="9" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="H154" s="10"/>
     </row>
     <row r="155" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A155" s="11" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B155" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/counting-bits/", "338")</f>
@@ -5538,13 +5563,13 @@
         <v>11</v>
       </c>
       <c r="G155" s="16" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="H155" s="17"/>
     </row>
     <row r="156" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A156" s="3" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B156" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/missing-number/", "268")</f>
@@ -5564,13 +5589,13 @@
         <v>11</v>
       </c>
       <c r="G156" s="9" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="H156" s="10"/>
     </row>
     <row r="157" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A157" s="11" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="B157" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/reverse-bits/", "190")</f>
@@ -5590,13 +5615,13 @@
         <v>11</v>
       </c>
       <c r="G157" s="16" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="H157" s="17"/>
     </row>
     <row r="158" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A158" s="3" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B158" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/climbing-stairs/", "70")</f>
@@ -5616,13 +5641,13 @@
         <v>11</v>
       </c>
       <c r="G158" s="9" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="H158" s="10"/>
     </row>
     <row r="159" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A159" s="11" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B159" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber/", "198")</f>
@@ -5642,13 +5667,13 @@
         <v>11</v>
       </c>
       <c r="G159" s="16" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="H159" s="17"/>
     </row>
     <row r="160" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A160" s="3" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B160" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/house-robber-ii/", "213")</f>
@@ -5668,13 +5693,13 @@
         <v>11</v>
       </c>
       <c r="G160" s="9" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="H160" s="10"/>
     </row>
     <row r="161" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A161" s="11" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B161" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change/", "322")</f>
@@ -5694,13 +5719,13 @@
         <v>11</v>
       </c>
       <c r="G161" s="16" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="H161" s="17"/>
     </row>
     <row r="162" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A162" s="3" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B162" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/perfect-squares/", "279")</f>
@@ -5720,13 +5745,13 @@
         <v>11</v>
       </c>
       <c r="G162" s="9" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="H162" s="10"/>
     </row>
     <row r="163" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A163" s="11" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B163" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-increasing-subsequence/", "300")</f>
@@ -5746,13 +5771,13 @@
         <v>11</v>
       </c>
       <c r="G163" s="16" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="H163" s="17"/>
     </row>
     <row r="164" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A164" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B164" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/partition-equal-subset-sum/", "416")</f>
@@ -5772,13 +5797,13 @@
         <v>11</v>
       </c>
       <c r="G164" s="9" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="H164" s="10"/>
     </row>
     <row r="165" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A165" s="11" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B165" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/target-sum/", "494")</f>
@@ -5798,13 +5823,13 @@
         <v>11</v>
       </c>
       <c r="G165" s="16" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="H165" s="17"/>
     </row>
     <row r="166" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A166" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B166" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/coin-change-ii/", "518")</f>
@@ -5824,13 +5849,13 @@
         <v>11</v>
       </c>
       <c r="G166" s="9" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="H166" s="10"/>
     </row>
     <row r="167" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A167" s="11" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B167" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/ones-and-zeroes/", "474")</f>
@@ -5850,13 +5875,13 @@
         <v>11</v>
       </c>
       <c r="G167" s="16" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="H167" s="17"/>
     </row>
     <row r="168" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A168" s="3" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B168" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/last-stone-weight-ii/", "1049")</f>
@@ -5876,13 +5901,13 @@
         <v>11</v>
       </c>
       <c r="G168" s="9" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="H168" s="10"/>
     </row>
     <row r="169" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A169" s="11" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B169" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/profitable-schemes/", "879")</f>
@@ -5902,13 +5927,13 @@
         <v>11</v>
       </c>
       <c r="G169" s="16" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="H169" s="17"/>
     </row>
     <row r="170" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A170" s="3" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B170" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths/", "62")</f>
@@ -5928,13 +5953,13 @@
         <v>11</v>
       </c>
       <c r="G170" s="9" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="H170" s="10"/>
     </row>
     <row r="171" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A171" s="11" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B171" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/unique-paths-ii/", "63")</f>
@@ -5954,13 +5979,13 @@
         <v>11</v>
       </c>
       <c r="G171" s="16" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="H171" s="17"/>
     </row>
     <row r="172" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="3" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B172" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-path-sum/", "64")</f>
@@ -5980,13 +6005,13 @@
         <v>11</v>
       </c>
       <c r="G172" s="9" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="H172" s="10"/>
     </row>
     <row r="173" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="11" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B173" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/maximal-square/", "221")</f>
@@ -6006,13 +6031,13 @@
         <v>11</v>
       </c>
       <c r="G173" s="16" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="H173" s="17"/>
     </row>
     <row r="174" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A174" s="3" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B174" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-falling-path-sum/", "931")</f>
@@ -6032,13 +6057,13 @@
         <v>11</v>
       </c>
       <c r="G174" s="9" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="H174" s="10"/>
     </row>
     <row r="175" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A175" s="11" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B175" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/triangle/", "120")</f>
@@ -6058,13 +6083,13 @@
         <v>11</v>
       </c>
       <c r="G175" s="16" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="H175" s="17"/>
     </row>
     <row r="176" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A176" s="3" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B176" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/longest-common-subsequence/", "1143")</f>
@@ -6084,13 +6109,13 @@
         <v>11</v>
       </c>
       <c r="G176" s="9" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="H176" s="10"/>
     </row>
     <row r="177" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A177" s="11" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B177" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/edit-distance/", "72")</f>
@@ -6110,13 +6135,13 @@
         <v>11</v>
       </c>
       <c r="G177" s="16" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="H177" s="17"/>
     </row>
     <row r="178" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A178" s="3" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B178" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/distinct-subsequences/", "115")</f>
@@ -6136,13 +6161,13 @@
         <v>11</v>
       </c>
       <c r="G178" s="9" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="H178" s="10"/>
     </row>
     <row r="179" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A179" s="11" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B179" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/delete-operation-for-two-strings/", "583")</f>
@@ -6162,13 +6187,13 @@
         <v>11</v>
       </c>
       <c r="G179" s="16" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="H179" s="17"/>
     </row>
     <row r="180" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A180" s="3" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B180" s="4" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/interleaving-string/", "97")</f>
@@ -6188,13 +6213,13 @@
         <v>11</v>
       </c>
       <c r="G180" s="9" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="H180" s="10"/>
     </row>
     <row r="181" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A181" s="11" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B181" s="12" t="str">
         <f aca="false">HYPERLINK("https://leetcode.com/problems/minimum-insertion-steps-to-make-a-string-palindrome/", "1312")</f>
@@ -6214,7 +6239,7 @@
         <v>11</v>
       </c>
       <c r="G181" s="16" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="H181" s="17"/>
     </row>

</xml_diff>